<commit_message>
v2.1 update: agent security, ISO 42001 checks, audit checklist, AI apps, print fix
- RCM v2.1: +9 controls (GL-9, LC-12, LC-13, SE-8, SE-9, SE-10, OM-4, PR-7, CO-4) from ISACA
  Securing AI Agents (2026), ISO 42001 checklist and AI Security Audit Checklist v1.0; refs extended
- New GT AI Security & Agent Audit Checklist v2.0 (125 items, auto-scored, findings register)
- Risk framework v1.1: 52-risk taxonomy, agent secure-by-default baseline, data classification for AI
- Readiness tool v1.1: printer-friendly page setup, larger radar, PDF guidance, updated guidance
- Strategy deck: AI apps portfolio + AI-powered BCP and Financial Statements apps (in preparation)
- Shared printfix helper applied to all workbooks

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X8ossW6xvKTGEs2GV44CxS
</commit_message>
<xml_diff>
--- a/01_AI_Governance_Risk_Compliance/1.2_AI_Risk_Assessment_Framework/GT_AI_Risk_Assessment_Toolkit_Template.xlsx
+++ b/01_AI_Governance_Risk_Compliance/1.2_AI_Risk_Assessment_Framework/GT_AI_Risk_Assessment_Toolkit_Template.xlsx
@@ -2,7 +2,6 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
@@ -18,8 +17,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="9" state="hidden" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4. Risk Register'!$A$4:$T$62</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Taxonomy'!$A$4:$G$52</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Guide'!$A$1:$C$11</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'1. Use Case Profile'!$A$1:$D$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'2. Prohibited Screen'!$A$1:$D$14</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'3. Risk Tiering'!$A$1:$G$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4. Risk Register'!$A$4:$T$66</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'4. Risk Register'!$A$1:$V$66</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'5. Heat Map &amp; Summary'!$A$1:$N$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Taxonomy'!$A$4:$G$56</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'Taxonomy'!$A$1:$G$56</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="7">'Scales'!$A$1:$I$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -973,7 +980,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Companion to the GT AI Risk Assessment Framework (v1.0, 2026). Grant Thornton Bahrain - AI Governance, Risk &amp; Compliance.</t>
+          <t>Companion to the GT AI Risk Assessment Framework (v1.1, 2026). Grant Thornton Bahrain - AI Governance, Risk &amp; Compliance.</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1028,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Work through the 48 taxonomy risks: mark applicability, tailor scenarios, rate likelihood &amp; impact, evaluate existing control effectiveness (mapped to RCM v2.0 controls) and plan treatment. Add bespoke risks in rows BSP-01..10.</t>
+          <t>Work through the 52 taxonomy risks: mark applicability, tailor scenarios, rate likelihood &amp; impact, evaluate existing control effectiveness (mapped to RCM v2.1 controls) and plan treatment. Add bespoke risks in rows BSP-01..10.</t>
         </is>
       </c>
     </row>
@@ -1078,8 +1085,9 @@
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <printOptions gridLines="0"/>
+  <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.25" footer="0.25"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1257,8 +1265,9 @@
       <formula1>=Lists!$H$1:$H$4</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <printOptions gridLines="0"/>
+  <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.25" footer="0.25"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1473,8 +1482,9 @@
       <formula1>=Lists!$A$1:$A$2</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <printOptions gridLines="0"/>
+  <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.25" footer="0.25"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1989,8 +1999,9 @@
       <formula1>=Lists!$U$1:$U$5</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <printOptions gridLines="0"/>
+  <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.25" footer="0.25"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2001,7 +2012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V62"/>
+  <dimension ref="A1:V66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2089,7 +2100,7 @@
       </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>Existing / required controls (RCM v2.0)</t>
+          <t>Existing / required controls (RCM v2.1)</t>
         </is>
       </c>
       <c r="K4" s="6" t="inlineStr">
@@ -3772,22 +3783,22 @@
       <c r="A30" s="15" t="n"/>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>TRA-01</t>
+          <t>PER-05</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>Transparency, Explainability &amp; Contestability</t>
+          <t>Model Performance, Reliability &amp; Robustness</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Undisclosed AI interaction or content</t>
+          <t>Uncontrolled prompt / configuration changes</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Users are unaware they interact with AI or that content is AI-generated.</t>
+          <t>Changes to prompts, guardrails, tool permissions or retrieval sources degrade safety or behaviour without regression testing.</t>
         </is>
       </c>
       <c r="F30" s="15" t="n"/>
@@ -3802,7 +3813,7 @@
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>CO-1, LC-7</t>
+          <t>LC-12</t>
         </is>
       </c>
       <c r="K30" s="15" t="n"/>
@@ -3825,7 +3836,7 @@
       <c r="S30" s="15" t="n"/>
       <c r="T30" s="5" t="inlineStr">
         <is>
-          <t>AI touchpoints lacking disclosure</t>
+          <t>Releases without passing LLM regression suite</t>
         </is>
       </c>
       <c r="V30">
@@ -3837,7 +3848,7 @@
       <c r="A31" s="15" t="n"/>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>TRA-02</t>
+          <t>TRA-01</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
@@ -3847,12 +3858,12 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Unexplainable decisions</t>
+          <t>Undisclosed AI interaction or content</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Organisation cannot explain AI-supported decisions to affected persons, regulators or auditors.</t>
+          <t>Users are unaware they interact with AI or that content is AI-generated.</t>
         </is>
       </c>
       <c r="F31" s="15" t="n"/>
@@ -3867,7 +3878,7 @@
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>RS-4, LC-4</t>
+          <t>CO-1, LC-7</t>
         </is>
       </c>
       <c r="K31" s="15" t="n"/>
@@ -3890,7 +3901,7 @@
       <c r="S31" s="15" t="n"/>
       <c r="T31" s="5" t="inlineStr">
         <is>
-          <t>Explanation requests not satisfied</t>
+          <t>AI touchpoints lacking disclosure</t>
         </is>
       </c>
       <c r="V31">
@@ -3902,7 +3913,7 @@
       <c r="A32" s="15" t="n"/>
       <c r="B32" s="12" t="inlineStr">
         <is>
-          <t>TRA-03</t>
+          <t>TRA-02</t>
         </is>
       </c>
       <c r="C32" s="12" t="inlineStr">
@@ -3912,12 +3923,12 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>No effective contest or redress route</t>
+          <t>Unexplainable decisions</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Affected persons cannot challenge or obtain human review of AI-supported decisions.</t>
+          <t>Organisation cannot explain AI-supported decisions to affected persons, regulators or auditors.</t>
         </is>
       </c>
       <c r="F32" s="15" t="n"/>
@@ -3932,7 +3943,7 @@
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>CO-3, PR-5</t>
+          <t>RS-4, LC-4</t>
         </is>
       </c>
       <c r="K32" s="15" t="n"/>
@@ -3955,7 +3966,7 @@
       <c r="S32" s="15" t="n"/>
       <c r="T32" s="5" t="inlineStr">
         <is>
-          <t>Appeals exceeding SLA</t>
+          <t>Explanation requests not satisfied</t>
         </is>
       </c>
       <c r="V32">
@@ -3967,7 +3978,7 @@
       <c r="A33" s="15" t="n"/>
       <c r="B33" s="12" t="inlineStr">
         <is>
-          <t>TRA-04</t>
+          <t>TRA-03</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
@@ -3977,12 +3988,12 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Inadequate documentation and records</t>
+          <t>No effective contest or redress route</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Technical documentation, logs or decisions are insufficient for audit or regulatory inspection.</t>
+          <t>Affected persons cannot challenge or obtain human review of AI-supported decisions.</t>
         </is>
       </c>
       <c r="F33" s="15" t="n"/>
@@ -3997,7 +4008,7 @@
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>LC-4, OM-2, RO-3</t>
+          <t>CO-3, PR-5</t>
         </is>
       </c>
       <c r="K33" s="15" t="n"/>
@@ -4020,7 +4031,7 @@
       <c r="S33" s="15" t="n"/>
       <c r="T33" s="5" t="inlineStr">
         <is>
-          <t>Systems with incomplete documentation pack</t>
+          <t>Appeals exceeding SLA</t>
         </is>
       </c>
       <c r="V33">
@@ -4032,22 +4043,22 @@
       <c r="A34" s="15" t="n"/>
       <c r="B34" s="12" t="inlineStr">
         <is>
-          <t>SEC-01</t>
+          <t>TRA-04</t>
         </is>
       </c>
       <c r="C34" s="12" t="inlineStr">
         <is>
-          <t>Security of AI Systems</t>
+          <t>Transparency, Explainability &amp; Contestability</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Prompt injection and jailbreak</t>
+          <t>Inadequate documentation and records</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Attacker manipulates model behaviour via direct or indirect (embedded content) instructions.</t>
+          <t>Technical documentation, logs or decisions are insufficient for audit or regulatory inspection.</t>
         </is>
       </c>
       <c r="F34" s="15" t="n"/>
@@ -4062,7 +4073,7 @@
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>SE-6</t>
+          <t>LC-4, OM-2, RO-3</t>
         </is>
       </c>
       <c r="K34" s="15" t="n"/>
@@ -4085,7 +4096,7 @@
       <c r="S34" s="15" t="n"/>
       <c r="T34" s="5" t="inlineStr">
         <is>
-          <t>Blocked injection attempts / bypasses in testing</t>
+          <t>Systems with incomplete documentation pack</t>
         </is>
       </c>
       <c r="V34">
@@ -4097,7 +4108,7 @@
       <c r="A35" s="15" t="n"/>
       <c r="B35" s="12" t="inlineStr">
         <is>
-          <t>SEC-02</t>
+          <t>SEC-01</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr">
@@ -4107,12 +4118,12 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Data or model poisoning</t>
+          <t>Prompt injection and jailbreak</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Training, fine-tuning or retrieval data is manipulated to corrupt outputs or insert backdoors.</t>
+          <t>Attacker manipulates model behaviour via direct or indirect (embedded content) instructions.</t>
         </is>
       </c>
       <c r="F35" s="15" t="n"/>
@@ -4127,7 +4138,7 @@
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>SE-6, LC-1, SE-7</t>
+          <t>SE-6</t>
         </is>
       </c>
       <c r="K35" s="15" t="n"/>
@@ -4150,7 +4161,7 @@
       <c r="S35" s="15" t="n"/>
       <c r="T35" s="5" t="inlineStr">
         <is>
-          <t>Integrity check failures</t>
+          <t>Blocked injection attempts / bypasses in testing</t>
         </is>
       </c>
       <c r="V35">
@@ -4162,7 +4173,7 @@
       <c r="A36" s="15" t="n"/>
       <c r="B36" s="12" t="inlineStr">
         <is>
-          <t>SEC-03</t>
+          <t>SEC-02</t>
         </is>
       </c>
       <c r="C36" s="12" t="inlineStr">
@@ -4172,12 +4183,12 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Model theft, extraction or inversion</t>
+          <t>Data or model poisoning</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Model weights, system prompts or training data are extracted.</t>
+          <t>Training, fine-tuning or retrieval data is manipulated to corrupt outputs or insert backdoors.</t>
         </is>
       </c>
       <c r="F36" s="15" t="n"/>
@@ -4192,7 +4203,7 @@
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>SE-4, SE-6</t>
+          <t>SE-6, LC-1, SE-7</t>
         </is>
       </c>
       <c r="K36" s="15" t="n"/>
@@ -4215,7 +4226,7 @@
       <c r="S36" s="15" t="n"/>
       <c r="T36" s="5" t="inlineStr">
         <is>
-          <t>Anomalous query volumes</t>
+          <t>Integrity check failures</t>
         </is>
       </c>
       <c r="V36">
@@ -4227,7 +4238,7 @@
       <c r="A37" s="15" t="n"/>
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>SEC-04</t>
+          <t>SEC-03</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
@@ -4237,12 +4248,12 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Insecure integration and excessive privilege</t>
+          <t>Model theft, extraction or inversion</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>AI components have excessive permissions or insecure APIs/plugins, enabling unauthorised actions.</t>
+          <t>Model weights, system prompts or training data are extracted.</t>
         </is>
       </c>
       <c r="F37" s="15" t="n"/>
@@ -4257,7 +4268,7 @@
       </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>SE-2, LC-8</t>
+          <t>SE-4, SE-6</t>
         </is>
       </c>
       <c r="K37" s="15" t="n"/>
@@ -4280,7 +4291,7 @@
       <c r="S37" s="15" t="n"/>
       <c r="T37" s="5" t="inlineStr">
         <is>
-          <t>Agents / integrations with privileged standing access</t>
+          <t>Anomalous query volumes</t>
         </is>
       </c>
       <c r="V37">
@@ -4292,7 +4303,7 @@
       <c r="A38" s="15" t="n"/>
       <c r="B38" s="12" t="inlineStr">
         <is>
-          <t>SEC-05</t>
+          <t>SEC-04</t>
         </is>
       </c>
       <c r="C38" s="12" t="inlineStr">
@@ -4302,12 +4313,12 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Compromised AI supply chain</t>
+          <t>Insecure integration and excessive privilege</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Malicious or vulnerable third-party models, libraries, plugins or MCP servers.</t>
+          <t>AI components have excessive permissions or insecure APIs/plugins, enabling unauthorised actions.</t>
         </is>
       </c>
       <c r="F38" s="15" t="n"/>
@@ -4322,7 +4333,7 @@
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>SE-7</t>
+          <t>SE-2, LC-8</t>
         </is>
       </c>
       <c r="K38" s="15" t="n"/>
@@ -4345,7 +4356,7 @@
       <c r="S38" s="15" t="n"/>
       <c r="T38" s="5" t="inlineStr">
         <is>
-          <t>Unscanned model artefacts</t>
+          <t>Agents / integrations with privileged standing access</t>
         </is>
       </c>
       <c r="V38">
@@ -4357,22 +4368,22 @@
       <c r="A39" s="15" t="n"/>
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>HUM-01</t>
+          <t>SEC-06</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr">
         <is>
-          <t>Human Oversight &amp; Autonomy</t>
+          <t>Security of AI Systems</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Automation bias and over-reliance</t>
+          <t>Agent memory poisoning &amp; cross-session leakage</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>Users accept AI outputs without adequate scrutiny, eroding professional judgement.</t>
+          <t>Poisoned or unauthorised content persists in agent memory / vector stores, or context leaks across users, sessions or tenants.</t>
         </is>
       </c>
       <c r="F39" s="15" t="n"/>
@@ -4387,7 +4398,7 @@
       </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
-          <t>RS-1, GL-4, LC-7</t>
+          <t>SE-8</t>
         </is>
       </c>
       <c r="K39" s="15" t="n"/>
@@ -4410,7 +4421,7 @@
       <c r="S39" s="15" t="n"/>
       <c r="T39" s="5" t="inlineStr">
         <is>
-          <t>Override / challenge rate</t>
+          <t>Cross-tenant retrieval test failures</t>
         </is>
       </c>
       <c r="V39">
@@ -4422,22 +4433,22 @@
       <c r="A40" s="15" t="n"/>
       <c r="B40" s="12" t="inlineStr">
         <is>
-          <t>HUM-02</t>
+          <t>SEC-07</t>
         </is>
       </c>
       <c r="C40" s="12" t="inlineStr">
         <is>
-          <t>Human Oversight &amp; Autonomy</t>
+          <t>Security of AI Systems</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Ineffective human oversight</t>
+          <t>Unsafe code execution, SSRF &amp; sandbox escape</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Oversight persons lack competence, authority, time or information to intervene.</t>
+          <t>Agent-generated code or tool calls reach internal networks, cloud metadata services or production secrets.</t>
         </is>
       </c>
       <c r="F40" s="15" t="n"/>
@@ -4452,7 +4463,7 @@
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>RS-1, GL-4</t>
+          <t>SE-9, SE-10</t>
         </is>
       </c>
       <c r="K40" s="15" t="n"/>
@@ -4475,7 +4486,7 @@
       <c r="S40" s="15" t="n"/>
       <c r="T40" s="5" t="inlineStr">
         <is>
-          <t>Oversight roles without training</t>
+          <t>Blocked egress / SSRF attempts</t>
         </is>
       </c>
       <c r="V40">
@@ -4487,22 +4498,22 @@
       <c r="A41" s="15" t="n"/>
       <c r="B41" s="12" t="inlineStr">
         <is>
-          <t>HUM-03</t>
+          <t>SEC-05</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr">
         <is>
-          <t>Human Oversight &amp; Autonomy</t>
+          <t>Security of AI Systems</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Unbounded autonomous agent actions</t>
+          <t>Compromised AI supply chain</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>AI agents take high-impact actions (payments, communications, code execution) without adequate limits or approval.</t>
+          <t>Malicious or vulnerable third-party models, libraries, plugins or MCP servers.</t>
         </is>
       </c>
       <c r="F41" s="15" t="n"/>
@@ -4517,7 +4528,7 @@
       </c>
       <c r="J41" s="5" t="inlineStr">
         <is>
-          <t>LC-8</t>
+          <t>SE-7</t>
         </is>
       </c>
       <c r="K41" s="15" t="n"/>
@@ -4540,7 +4551,7 @@
       <c r="S41" s="15" t="n"/>
       <c r="T41" s="5" t="inlineStr">
         <is>
-          <t>High-impact agent actions without approval</t>
+          <t>Unscanned model artefacts</t>
         </is>
       </c>
       <c r="V41">
@@ -4552,7 +4563,7 @@
       <c r="A42" s="15" t="n"/>
       <c r="B42" s="12" t="inlineStr">
         <is>
-          <t>HUM-04</t>
+          <t>HUM-01</t>
         </is>
       </c>
       <c r="C42" s="12" t="inlineStr">
@@ -4562,12 +4573,12 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Adverse workforce impact</t>
+          <t>Automation bias and over-reliance</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>AI adoption causes skills erosion, job anxiety or unconsulted changes to working conditions.</t>
+          <t>Users accept AI outputs without adequate scrutiny, eroding professional judgement.</t>
         </is>
       </c>
       <c r="F42" s="15" t="n"/>
@@ -4582,7 +4593,7 @@
       </c>
       <c r="J42" s="5" t="inlineStr">
         <is>
-          <t>RS-9, GL-4</t>
+          <t>RS-1, GL-4, LC-7</t>
         </is>
       </c>
       <c r="K42" s="15" t="n"/>
@@ -4605,7 +4616,7 @@
       <c r="S42" s="15" t="n"/>
       <c r="T42" s="5" t="inlineStr">
         <is>
-          <t>Staff sentiment / attrition in affected roles</t>
+          <t>Override / challenge rate</t>
         </is>
       </c>
       <c r="V42">
@@ -4617,22 +4628,22 @@
       <c r="A43" s="15" t="n"/>
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t>TPR-01</t>
+          <t>HUM-02</t>
         </is>
       </c>
       <c r="C43" s="12" t="inlineStr">
         <is>
-          <t>Third-Party &amp; Supply Chain</t>
+          <t>Human Oversight &amp; Autonomy</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Vendor lock-in and concentration</t>
+          <t>Ineffective human oversight</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>Critical dependence on a single AI provider or cloud creates resilience and bargaining risk.</t>
+          <t>Oversight persons lack competence, authority, time or information to intervene.</t>
         </is>
       </c>
       <c r="F43" s="15" t="n"/>
@@ -4647,7 +4658,7 @@
       </c>
       <c r="J43" s="5" t="inlineStr">
         <is>
-          <t>TP-2, TP-3</t>
+          <t>RS-1, GL-4</t>
         </is>
       </c>
       <c r="K43" s="15" t="n"/>
@@ -4670,7 +4681,7 @@
       <c r="S43" s="15" t="n"/>
       <c r="T43" s="5" t="inlineStr">
         <is>
-          <t>% critical AI workloads on single provider</t>
+          <t>Oversight roles without training</t>
         </is>
       </c>
       <c r="V43">
@@ -4682,22 +4693,22 @@
       <c r="A44" s="15" t="n"/>
       <c r="B44" s="12" t="inlineStr">
         <is>
-          <t>TPR-02</t>
+          <t>HUM-03</t>
         </is>
       </c>
       <c r="C44" s="12" t="inlineStr">
         <is>
-          <t>Third-Party &amp; Supply Chain</t>
+          <t>Human Oversight &amp; Autonomy</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Inadequate vendor transparency and assurance</t>
+          <t>Unbounded autonomous agent actions</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>Vendor cannot provide documentation, testing evidence or incident information needed for compliance.</t>
+          <t>AI agents take high-impact actions (payments, communications, code execution) without adequate limits or approval.</t>
         </is>
       </c>
       <c r="F44" s="15" t="n"/>
@@ -4712,7 +4723,7 @@
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>TP-1, TP-3, LC-6</t>
+          <t>LC-8</t>
         </is>
       </c>
       <c r="K44" s="15" t="n"/>
@@ -4735,7 +4746,7 @@
       <c r="S44" s="15" t="n"/>
       <c r="T44" s="5" t="inlineStr">
         <is>
-          <t>Vendors without current assurance evidence</t>
+          <t>High-impact agent actions without approval</t>
         </is>
       </c>
       <c r="V44">
@@ -4747,22 +4758,22 @@
       <c r="A45" s="15" t="n"/>
       <c r="B45" s="12" t="inlineStr">
         <is>
-          <t>TPR-03</t>
+          <t>HUM-04</t>
         </is>
       </c>
       <c r="C45" s="12" t="inlineStr">
         <is>
-          <t>Third-Party &amp; Supply Chain</t>
+          <t>Human Oversight &amp; Autonomy</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Vendor use of organisation data</t>
+          <t>Adverse workforce impact</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>Provider uses prompts, outputs or client data to train models or retains data beyond agreed terms.</t>
+          <t>AI adoption causes skills erosion, job anxiety or unconsulted changes to working conditions.</t>
         </is>
       </c>
       <c r="F45" s="15" t="n"/>
@@ -4777,7 +4788,7 @@
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>TP-3, PR-6</t>
+          <t>RS-9, GL-4</t>
         </is>
       </c>
       <c r="K45" s="15" t="n"/>
@@ -4800,7 +4811,7 @@
       <c r="S45" s="15" t="n"/>
       <c r="T45" s="5" t="inlineStr">
         <is>
-          <t>Contracts lacking no-training clause</t>
+          <t>Staff sentiment / attrition in affected roles</t>
         </is>
       </c>
       <c r="V45">
@@ -4812,22 +4823,22 @@
       <c r="A46" s="15" t="n"/>
       <c r="B46" s="12" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>TPR-01</t>
         </is>
       </c>
       <c r="C46" s="12" t="inlineStr">
         <is>
-          <t>Operational, Financial &amp; Sustainability</t>
+          <t>Third-Party &amp; Supply Chain</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>AI service outage or degradation</t>
+          <t>Vendor lock-in and concentration</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Business processes dependent on AI are disrupted by service unavailability or latency.</t>
+          <t>Critical dependence on a single AI provider or cloud creates resilience and bargaining risk.</t>
         </is>
       </c>
       <c r="F46" s="15" t="n"/>
@@ -4842,7 +4853,7 @@
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>OM-1, SE-1</t>
+          <t>TP-2, TP-3</t>
         </is>
       </c>
       <c r="K46" s="15" t="n"/>
@@ -4865,7 +4876,7 @@
       <c r="S46" s="15" t="n"/>
       <c r="T46" s="5" t="inlineStr">
         <is>
-          <t>AI service availability vs SLA</t>
+          <t>% critical AI workloads on single provider</t>
         </is>
       </c>
       <c r="V46">
@@ -4877,22 +4888,22 @@
       <c r="A47" s="15" t="n"/>
       <c r="B47" s="12" t="inlineStr">
         <is>
-          <t>OPS-02</t>
+          <t>TPR-02</t>
         </is>
       </c>
       <c r="C47" s="12" t="inlineStr">
         <is>
-          <t>Operational, Financial &amp; Sustainability</t>
+          <t>Third-Party &amp; Supply Chain</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Uncontrolled AI cost and consumption</t>
+          <t>Inadequate vendor transparency and assurance</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>Compute and API spend escalate without governance (incl. denial-of-wallet attacks).</t>
+          <t>Vendor cannot provide documentation, testing evidence or incident information needed for compliance.</t>
         </is>
       </c>
       <c r="F47" s="15" t="n"/>
@@ -4907,7 +4918,7 @@
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>GL-6, SE-6</t>
+          <t>TP-1, TP-3, LC-6</t>
         </is>
       </c>
       <c r="K47" s="15" t="n"/>
@@ -4930,7 +4941,7 @@
       <c r="S47" s="15" t="n"/>
       <c r="T47" s="5" t="inlineStr">
         <is>
-          <t>AI spend vs budget</t>
+          <t>Vendors without current assurance evidence</t>
         </is>
       </c>
       <c r="V47">
@@ -4942,22 +4953,22 @@
       <c r="A48" s="15" t="n"/>
       <c r="B48" s="12" t="inlineStr">
         <is>
-          <t>OPS-03</t>
+          <t>TPR-03</t>
         </is>
       </c>
       <c r="C48" s="12" t="inlineStr">
         <is>
-          <t>Operational, Financial &amp; Sustainability</t>
+          <t>Third-Party &amp; Supply Chain</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Environmental impact of AI</t>
+          <t>Vendor use of organisation data</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>Energy, water and carbon footprint of AI workloads conflicts with sustainability commitments.</t>
+          <t>Provider uses prompts, outputs or client data to train models or retains data beyond agreed terms.</t>
         </is>
       </c>
       <c r="F48" s="15" t="n"/>
@@ -4972,7 +4983,7 @@
       </c>
       <c r="J48" s="5" t="inlineStr">
         <is>
-          <t>RS-8</t>
+          <t>TP-3, PR-6</t>
         </is>
       </c>
       <c r="K48" s="15" t="n"/>
@@ -4995,7 +5006,7 @@
       <c r="S48" s="15" t="n"/>
       <c r="T48" s="5" t="inlineStr">
         <is>
-          <t>kgCO2e per 1,000 inferences</t>
+          <t>Contracts lacking no-training clause</t>
         </is>
       </c>
       <c r="V48">
@@ -5007,22 +5018,22 @@
       <c r="A49" s="15" t="n"/>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>SOC-01</t>
+          <t>OPS-01</t>
         </is>
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>Societal, Reputational &amp; AI-Enabled Threats</t>
+          <t>Operational, Financial &amp; Sustainability</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Harmful, toxic or unsafe content</t>
+          <t>AI service outage or degradation</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>AI generates offensive, dangerous or culturally inappropriate content.</t>
+          <t>Business processes dependent on AI are disrupted by service unavailability or latency.</t>
         </is>
       </c>
       <c r="F49" s="15" t="n"/>
@@ -5037,7 +5048,7 @@
       </c>
       <c r="J49" s="5" t="inlineStr">
         <is>
-          <t>RS-2, SE-6</t>
+          <t>OM-1, SE-1</t>
         </is>
       </c>
       <c r="K49" s="15" t="n"/>
@@ -5060,7 +5071,7 @@
       <c r="S49" s="15" t="n"/>
       <c r="T49" s="5" t="inlineStr">
         <is>
-          <t>Content-policy violations per 1,000 outputs</t>
+          <t>AI service availability vs SLA</t>
         </is>
       </c>
       <c r="V49">
@@ -5072,22 +5083,22 @@
       <c r="A50" s="15" t="n"/>
       <c r="B50" s="12" t="inlineStr">
         <is>
-          <t>SOC-02</t>
+          <t>OPS-02</t>
         </is>
       </c>
       <c r="C50" s="12" t="inlineStr">
         <is>
-          <t>Societal, Reputational &amp; AI-Enabled Threats</t>
+          <t>Operational, Financial &amp; Sustainability</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Misinformation and loss of stakeholder trust</t>
+          <t>Uncontrolled AI cost and consumption</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>AI-generated errors or undisclosed AI use damage client, regulator or public trust.</t>
+          <t>Compute and API spend escalate without governance (incl. denial-of-wallet attacks).</t>
         </is>
       </c>
       <c r="F50" s="15" t="n"/>
@@ -5102,7 +5113,7 @@
       </c>
       <c r="J50" s="5" t="inlineStr">
         <is>
-          <t>LC-7, CO-1, CO-2</t>
+          <t>GL-6, SE-6</t>
         </is>
       </c>
       <c r="K50" s="15" t="n"/>
@@ -5125,7 +5136,7 @@
       <c r="S50" s="15" t="n"/>
       <c r="T50" s="5" t="inlineStr">
         <is>
-          <t>Client complaints linked to AI</t>
+          <t>AI spend vs budget</t>
         </is>
       </c>
       <c r="V50">
@@ -5137,22 +5148,22 @@
       <c r="A51" s="15" t="n"/>
       <c r="B51" s="12" t="inlineStr">
         <is>
-          <t>SOC-03</t>
+          <t>OPS-04</t>
         </is>
       </c>
       <c r="C51" s="12" t="inlineStr">
         <is>
-          <t>Societal, Reputational &amp; AI-Enabled Threats</t>
+          <t>Operational, Financial &amp; Sustainability</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Deepfake and AI-enabled fraud against the organisation</t>
+          <t>No safe degradation or kill switch</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>Voice/video impersonation or AI-crafted phishing leads to fraudulent payments or data release.</t>
+          <t>A failing or compromised AI system cannot be stopped quickly or the business process cannot revert to manual operation.</t>
         </is>
       </c>
       <c r="F51" s="15" t="n"/>
@@ -5167,7 +5178,7 @@
       </c>
       <c r="J51" s="5" t="inlineStr">
         <is>
-          <t>AT-3, GL-4</t>
+          <t>OM-4</t>
         </is>
       </c>
       <c r="K51" s="15" t="n"/>
@@ -5190,7 +5201,7 @@
       <c r="S51" s="15" t="n"/>
       <c r="T51" s="5" t="inlineStr">
         <is>
-          <t>Deepfake / BEC attempts detected</t>
+          <t>Kill-switch test age (days)</t>
         </is>
       </c>
       <c r="V51">
@@ -5202,22 +5213,22 @@
       <c r="A52" s="15" t="n"/>
       <c r="B52" s="12" t="inlineStr">
         <is>
-          <t>SOC-04</t>
+          <t>OPS-03</t>
         </is>
       </c>
       <c r="C52" s="12" t="inlineStr">
         <is>
-          <t>Societal, Reputational &amp; AI-Enabled Threats</t>
+          <t>Operational, Financial &amp; Sustainability</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>AI-accelerated cyber attacks</t>
+          <t>Environmental impact of AI</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>Adversaries use AI for automated discovery, exploit chaining and scaled social engineering, outpacing defences.</t>
+          <t>Energy, water and carbon footprint of AI workloads conflicts with sustainability commitments.</t>
         </is>
       </c>
       <c r="F52" s="15" t="n"/>
@@ -5232,7 +5243,7 @@
       </c>
       <c r="J52" s="5" t="inlineStr">
         <is>
-          <t>AT-1, AT-2, AT-4</t>
+          <t>RS-8</t>
         </is>
       </c>
       <c r="K52" s="15" t="n"/>
@@ -5255,7 +5266,7 @@
       <c r="S52" s="15" t="n"/>
       <c r="T52" s="5" t="inlineStr">
         <is>
-          <t>Mean time to remediate critical vulnerabilities</t>
+          <t>kgCO2e per 1,000 inferences</t>
         </is>
       </c>
       <c r="V52">
@@ -5267,12 +5278,24 @@
       <c r="A53" s="15" t="n"/>
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t>BSP-01</t>
-        </is>
-      </c>
-      <c r="C53" s="12" t="n"/>
-      <c r="D53" s="4" t="n"/>
-      <c r="E53" s="5" t="n"/>
+          <t>SOC-01</t>
+        </is>
+      </c>
+      <c r="C53" s="12" t="inlineStr">
+        <is>
+          <t>Societal, Reputational &amp; AI-Enabled Threats</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>Harmful, toxic or unsafe content</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>AI generates offensive, dangerous or culturally inappropriate content.</t>
+        </is>
+      </c>
       <c r="F53" s="15" t="n"/>
       <c r="G53" s="15" t="n"/>
       <c r="H53" s="7">
@@ -5283,7 +5306,11 @@
         <f>IF(H53="","",IF(H53&gt;=17,"Critical",IF(H53&gt;=10,"High",IF(H53&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="J53" s="5" t="n"/>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>RS-2, SE-6</t>
+        </is>
+      </c>
       <c r="K53" s="15" t="n"/>
       <c r="L53" s="7">
         <f>IF(OR(H53="",K53=""),"",ROUND(H53*VLOOKUP(K53,Scales!$A$22:$B$25,2,FALSE),1))</f>
@@ -5302,7 +5329,11 @@
       <c r="Q53" s="15" t="n"/>
       <c r="R53" s="15" t="n"/>
       <c r="S53" s="15" t="n"/>
-      <c r="T53" s="5" t="n"/>
+      <c r="T53" s="5" t="inlineStr">
+        <is>
+          <t>Content-policy violations per 1,000 outputs</t>
+        </is>
+      </c>
       <c r="V53">
         <f>IF(L53="","",L53+ROW()/100000)</f>
         <v/>
@@ -5312,12 +5343,24 @@
       <c r="A54" s="15" t="n"/>
       <c r="B54" s="12" t="inlineStr">
         <is>
-          <t>BSP-02</t>
-        </is>
-      </c>
-      <c r="C54" s="12" t="n"/>
-      <c r="D54" s="4" t="n"/>
-      <c r="E54" s="5" t="n"/>
+          <t>SOC-02</t>
+        </is>
+      </c>
+      <c r="C54" s="12" t="inlineStr">
+        <is>
+          <t>Societal, Reputational &amp; AI-Enabled Threats</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Misinformation and loss of stakeholder trust</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>AI-generated errors or undisclosed AI use damage client, regulator or public trust.</t>
+        </is>
+      </c>
       <c r="F54" s="15" t="n"/>
       <c r="G54" s="15" t="n"/>
       <c r="H54" s="7">
@@ -5328,7 +5371,11 @@
         <f>IF(H54="","",IF(H54&gt;=17,"Critical",IF(H54&gt;=10,"High",IF(H54&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="J54" s="5" t="n"/>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>LC-7, CO-1, CO-2</t>
+        </is>
+      </c>
       <c r="K54" s="15" t="n"/>
       <c r="L54" s="7">
         <f>IF(OR(H54="",K54=""),"",ROUND(H54*VLOOKUP(K54,Scales!$A$22:$B$25,2,FALSE),1))</f>
@@ -5347,7 +5394,11 @@
       <c r="Q54" s="15" t="n"/>
       <c r="R54" s="15" t="n"/>
       <c r="S54" s="15" t="n"/>
-      <c r="T54" s="5" t="n"/>
+      <c r="T54" s="5" t="inlineStr">
+        <is>
+          <t>Client complaints linked to AI</t>
+        </is>
+      </c>
       <c r="V54">
         <f>IF(L54="","",L54+ROW()/100000)</f>
         <v/>
@@ -5357,12 +5408,24 @@
       <c r="A55" s="15" t="n"/>
       <c r="B55" s="12" t="inlineStr">
         <is>
-          <t>BSP-03</t>
-        </is>
-      </c>
-      <c r="C55" s="12" t="n"/>
-      <c r="D55" s="4" t="n"/>
-      <c r="E55" s="5" t="n"/>
+          <t>SOC-03</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="inlineStr">
+        <is>
+          <t>Societal, Reputational &amp; AI-Enabled Threats</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>Deepfake and AI-enabled fraud against the organisation</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Voice/video impersonation or AI-crafted phishing leads to fraudulent payments or data release.</t>
+        </is>
+      </c>
       <c r="F55" s="15" t="n"/>
       <c r="G55" s="15" t="n"/>
       <c r="H55" s="7">
@@ -5373,7 +5436,11 @@
         <f>IF(H55="","",IF(H55&gt;=17,"Critical",IF(H55&gt;=10,"High",IF(H55&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="J55" s="5" t="n"/>
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>AT-3, GL-4</t>
+        </is>
+      </c>
       <c r="K55" s="15" t="n"/>
       <c r="L55" s="7">
         <f>IF(OR(H55="",K55=""),"",ROUND(H55*VLOOKUP(K55,Scales!$A$22:$B$25,2,FALSE),1))</f>
@@ -5392,7 +5459,11 @@
       <c r="Q55" s="15" t="n"/>
       <c r="R55" s="15" t="n"/>
       <c r="S55" s="15" t="n"/>
-      <c r="T55" s="5" t="n"/>
+      <c r="T55" s="5" t="inlineStr">
+        <is>
+          <t>Deepfake / BEC attempts detected</t>
+        </is>
+      </c>
       <c r="V55">
         <f>IF(L55="","",L55+ROW()/100000)</f>
         <v/>
@@ -5402,12 +5473,24 @@
       <c r="A56" s="15" t="n"/>
       <c r="B56" s="12" t="inlineStr">
         <is>
-          <t>BSP-04</t>
-        </is>
-      </c>
-      <c r="C56" s="12" t="n"/>
-      <c r="D56" s="4" t="n"/>
-      <c r="E56" s="5" t="n"/>
+          <t>SOC-04</t>
+        </is>
+      </c>
+      <c r="C56" s="12" t="inlineStr">
+        <is>
+          <t>Societal, Reputational &amp; AI-Enabled Threats</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>AI-accelerated cyber attacks</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Adversaries use AI for automated discovery, exploit chaining and scaled social engineering, outpacing defences.</t>
+        </is>
+      </c>
       <c r="F56" s="15" t="n"/>
       <c r="G56" s="15" t="n"/>
       <c r="H56" s="7">
@@ -5418,7 +5501,11 @@
         <f>IF(H56="","",IF(H56&gt;=17,"Critical",IF(H56&gt;=10,"High",IF(H56&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="J56" s="5" t="n"/>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>AT-1, AT-2, AT-4</t>
+        </is>
+      </c>
       <c r="K56" s="15" t="n"/>
       <c r="L56" s="7">
         <f>IF(OR(H56="",K56=""),"",ROUND(H56*VLOOKUP(K56,Scales!$A$22:$B$25,2,FALSE),1))</f>
@@ -5437,7 +5524,11 @@
       <c r="Q56" s="15" t="n"/>
       <c r="R56" s="15" t="n"/>
       <c r="S56" s="15" t="n"/>
-      <c r="T56" s="5" t="n"/>
+      <c r="T56" s="5" t="inlineStr">
+        <is>
+          <t>Mean time to remediate critical vulnerabilities</t>
+        </is>
+      </c>
       <c r="V56">
         <f>IF(L56="","",L56+ROW()/100000)</f>
         <v/>
@@ -5447,7 +5538,7 @@
       <c r="A57" s="15" t="n"/>
       <c r="B57" s="12" t="inlineStr">
         <is>
-          <t>BSP-05</t>
+          <t>BSP-01</t>
         </is>
       </c>
       <c r="C57" s="12" t="n"/>
@@ -5492,7 +5583,7 @@
       <c r="A58" s="15" t="n"/>
       <c r="B58" s="12" t="inlineStr">
         <is>
-          <t>BSP-06</t>
+          <t>BSP-02</t>
         </is>
       </c>
       <c r="C58" s="12" t="n"/>
@@ -5537,7 +5628,7 @@
       <c r="A59" s="15" t="n"/>
       <c r="B59" s="12" t="inlineStr">
         <is>
-          <t>BSP-07</t>
+          <t>BSP-03</t>
         </is>
       </c>
       <c r="C59" s="12" t="n"/>
@@ -5582,7 +5673,7 @@
       <c r="A60" s="15" t="n"/>
       <c r="B60" s="12" t="inlineStr">
         <is>
-          <t>BSP-08</t>
+          <t>BSP-04</t>
         </is>
       </c>
       <c r="C60" s="12" t="n"/>
@@ -5627,7 +5718,7 @@
       <c r="A61" s="15" t="n"/>
       <c r="B61" s="12" t="inlineStr">
         <is>
-          <t>BSP-09</t>
+          <t>BSP-05</t>
         </is>
       </c>
       <c r="C61" s="12" t="n"/>
@@ -5672,7 +5763,7 @@
       <c r="A62" s="15" t="n"/>
       <c r="B62" s="12" t="inlineStr">
         <is>
-          <t>BSP-10</t>
+          <t>BSP-06</t>
         </is>
       </c>
       <c r="C62" s="12" t="n"/>
@@ -5713,13 +5804,193 @@
         <v/>
       </c>
     </row>
+    <row r="63" ht="44" customHeight="1">
+      <c r="A63" s="15" t="n"/>
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>BSP-07</t>
+        </is>
+      </c>
+      <c r="C63" s="12" t="n"/>
+      <c r="D63" s="4" t="n"/>
+      <c r="E63" s="5" t="n"/>
+      <c r="F63" s="15" t="n"/>
+      <c r="G63" s="15" t="n"/>
+      <c r="H63" s="7">
+        <f>IF(OR($A63&lt;&gt;"Yes",F63="",G63=""),"",MATCH(F63,Lists!$B$1:$B$5,0)*MATCH(G63,Lists!$C$1:$C$5,0))</f>
+        <v/>
+      </c>
+      <c r="I63" s="7">
+        <f>IF(H63="","",IF(H63&gt;=17,"Critical",IF(H63&gt;=10,"High",IF(H63&gt;=5,"Medium","Low"))))</f>
+        <v/>
+      </c>
+      <c r="J63" s="5" t="n"/>
+      <c r="K63" s="15" t="n"/>
+      <c r="L63" s="7">
+        <f>IF(OR(H63="",K63=""),"",ROUND(H63*VLOOKUP(K63,Scales!$A$22:$B$25,2,FALSE),1))</f>
+        <v/>
+      </c>
+      <c r="M63" s="7">
+        <f>IF(L63="","",IF(L63&gt;=17,"Critical",IF(L63&gt;=10,"High",IF(L63&gt;=5,"Medium","Low"))))</f>
+        <v/>
+      </c>
+      <c r="N63" s="7">
+        <f>IF(M63="","",IF(OR(M63="Low",M63="Medium"),"Yes","No"))</f>
+        <v/>
+      </c>
+      <c r="O63" s="15" t="n"/>
+      <c r="P63" s="5" t="n"/>
+      <c r="Q63" s="15" t="n"/>
+      <c r="R63" s="15" t="n"/>
+      <c r="S63" s="15" t="n"/>
+      <c r="T63" s="5" t="n"/>
+      <c r="V63">
+        <f>IF(L63="","",L63+ROW()/100000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" ht="44" customHeight="1">
+      <c r="A64" s="15" t="n"/>
+      <c r="B64" s="12" t="inlineStr">
+        <is>
+          <t>BSP-08</t>
+        </is>
+      </c>
+      <c r="C64" s="12" t="n"/>
+      <c r="D64" s="4" t="n"/>
+      <c r="E64" s="5" t="n"/>
+      <c r="F64" s="15" t="n"/>
+      <c r="G64" s="15" t="n"/>
+      <c r="H64" s="7">
+        <f>IF(OR($A64&lt;&gt;"Yes",F64="",G64=""),"",MATCH(F64,Lists!$B$1:$B$5,0)*MATCH(G64,Lists!$C$1:$C$5,0))</f>
+        <v/>
+      </c>
+      <c r="I64" s="7">
+        <f>IF(H64="","",IF(H64&gt;=17,"Critical",IF(H64&gt;=10,"High",IF(H64&gt;=5,"Medium","Low"))))</f>
+        <v/>
+      </c>
+      <c r="J64" s="5" t="n"/>
+      <c r="K64" s="15" t="n"/>
+      <c r="L64" s="7">
+        <f>IF(OR(H64="",K64=""),"",ROUND(H64*VLOOKUP(K64,Scales!$A$22:$B$25,2,FALSE),1))</f>
+        <v/>
+      </c>
+      <c r="M64" s="7">
+        <f>IF(L64="","",IF(L64&gt;=17,"Critical",IF(L64&gt;=10,"High",IF(L64&gt;=5,"Medium","Low"))))</f>
+        <v/>
+      </c>
+      <c r="N64" s="7">
+        <f>IF(M64="","",IF(OR(M64="Low",M64="Medium"),"Yes","No"))</f>
+        <v/>
+      </c>
+      <c r="O64" s="15" t="n"/>
+      <c r="P64" s="5" t="n"/>
+      <c r="Q64" s="15" t="n"/>
+      <c r="R64" s="15" t="n"/>
+      <c r="S64" s="15" t="n"/>
+      <c r="T64" s="5" t="n"/>
+      <c r="V64">
+        <f>IF(L64="","",L64+ROW()/100000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="44" customHeight="1">
+      <c r="A65" s="15" t="n"/>
+      <c r="B65" s="12" t="inlineStr">
+        <is>
+          <t>BSP-09</t>
+        </is>
+      </c>
+      <c r="C65" s="12" t="n"/>
+      <c r="D65" s="4" t="n"/>
+      <c r="E65" s="5" t="n"/>
+      <c r="F65" s="15" t="n"/>
+      <c r="G65" s="15" t="n"/>
+      <c r="H65" s="7">
+        <f>IF(OR($A65&lt;&gt;"Yes",F65="",G65=""),"",MATCH(F65,Lists!$B$1:$B$5,0)*MATCH(G65,Lists!$C$1:$C$5,0))</f>
+        <v/>
+      </c>
+      <c r="I65" s="7">
+        <f>IF(H65="","",IF(H65&gt;=17,"Critical",IF(H65&gt;=10,"High",IF(H65&gt;=5,"Medium","Low"))))</f>
+        <v/>
+      </c>
+      <c r="J65" s="5" t="n"/>
+      <c r="K65" s="15" t="n"/>
+      <c r="L65" s="7">
+        <f>IF(OR(H65="",K65=""),"",ROUND(H65*VLOOKUP(K65,Scales!$A$22:$B$25,2,FALSE),1))</f>
+        <v/>
+      </c>
+      <c r="M65" s="7">
+        <f>IF(L65="","",IF(L65&gt;=17,"Critical",IF(L65&gt;=10,"High",IF(L65&gt;=5,"Medium","Low"))))</f>
+        <v/>
+      </c>
+      <c r="N65" s="7">
+        <f>IF(M65="","",IF(OR(M65="Low",M65="Medium"),"Yes","No"))</f>
+        <v/>
+      </c>
+      <c r="O65" s="15" t="n"/>
+      <c r="P65" s="5" t="n"/>
+      <c r="Q65" s="15" t="n"/>
+      <c r="R65" s="15" t="n"/>
+      <c r="S65" s="15" t="n"/>
+      <c r="T65" s="5" t="n"/>
+      <c r="V65">
+        <f>IF(L65="","",L65+ROW()/100000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" ht="44" customHeight="1">
+      <c r="A66" s="15" t="n"/>
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>BSP-10</t>
+        </is>
+      </c>
+      <c r="C66" s="12" t="n"/>
+      <c r="D66" s="4" t="n"/>
+      <c r="E66" s="5" t="n"/>
+      <c r="F66" s="15" t="n"/>
+      <c r="G66" s="15" t="n"/>
+      <c r="H66" s="7">
+        <f>IF(OR($A66&lt;&gt;"Yes",F66="",G66=""),"",MATCH(F66,Lists!$B$1:$B$5,0)*MATCH(G66,Lists!$C$1:$C$5,0))</f>
+        <v/>
+      </c>
+      <c r="I66" s="7">
+        <f>IF(H66="","",IF(H66&gt;=17,"Critical",IF(H66&gt;=10,"High",IF(H66&gt;=5,"Medium","Low"))))</f>
+        <v/>
+      </c>
+      <c r="J66" s="5" t="n"/>
+      <c r="K66" s="15" t="n"/>
+      <c r="L66" s="7">
+        <f>IF(OR(H66="",K66=""),"",ROUND(H66*VLOOKUP(K66,Scales!$A$22:$B$25,2,FALSE),1))</f>
+        <v/>
+      </c>
+      <c r="M66" s="7">
+        <f>IF(L66="","",IF(L66&gt;=17,"Critical",IF(L66&gt;=10,"High",IF(L66&gt;=5,"Medium","Low"))))</f>
+        <v/>
+      </c>
+      <c r="N66" s="7">
+        <f>IF(M66="","",IF(OR(M66="Low",M66="Medium"),"Yes","No"))</f>
+        <v/>
+      </c>
+      <c r="O66" s="15" t="n"/>
+      <c r="P66" s="5" t="n"/>
+      <c r="Q66" s="15" t="n"/>
+      <c r="R66" s="15" t="n"/>
+      <c r="S66" s="15" t="n"/>
+      <c r="T66" s="5" t="n"/>
+      <c r="V66">
+        <f>IF(L66="","",L66+ROW()/100000)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:T62"/>
+  <autoFilter ref="A4:T66"/>
   <mergeCells count="2">
     <mergeCell ref="A1:T1"/>
     <mergeCell ref="A2:T2"/>
   </mergeCells>
-  <conditionalFormatting sqref="I5:I62">
+  <conditionalFormatting sqref="I5:I66">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
       <formula>"Low"</formula>
     </cfRule>
@@ -5736,7 +6007,7 @@
       <formula>"Prohibited"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M5:M62">
+  <conditionalFormatting sqref="M5:M66">
     <cfRule type="cellIs" priority="6" operator="equal" dxfId="2">
       <formula>"Low"</formula>
     </cfRule>
@@ -5753,38 +6024,39 @@
       <formula>"Prohibited"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N5:N62">
+  <conditionalFormatting sqref="N5:N66">
     <cfRule type="cellIs" priority="11" operator="equal" dxfId="6">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:T62">
+  <conditionalFormatting sqref="A5:T66">
     <cfRule type="expression" priority="12" dxfId="7">
       <formula>$A5="No"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="6">
-    <dataValidation sqref="A5:A62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A5:A66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$A$1:$A$2</formula1>
     </dataValidation>
-    <dataValidation sqref="F5:F62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$B$1:$B$5</formula1>
     </dataValidation>
-    <dataValidation sqref="G5:G62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$C$1:$C$5</formula1>
     </dataValidation>
-    <dataValidation sqref="K5:K62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K5:K66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$D$1:$D$4</formula1>
     </dataValidation>
-    <dataValidation sqref="O5:O62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O5:O66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$E$1:$E$4</formula1>
     </dataValidation>
-    <dataValidation sqref="S5:S62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="S5:S66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$F$1:$F$5</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <printOptions gridLines="0"/>
+  <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.25" footer="0.25"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -5888,23 +6160,23 @@
         </is>
       </c>
       <c r="B6" s="18">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Almost certain",'4. Risk Register'!$G$5:$G$62,"Insignificant")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Almost certain",'4. Risk Register'!$G$5:$G$66,"Insignificant")</f>
         <v/>
       </c>
       <c r="C6" s="19">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Almost certain",'4. Risk Register'!$G$5:$G$62,"Minor")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Almost certain",'4. Risk Register'!$G$5:$G$66,"Minor")</f>
         <v/>
       </c>
       <c r="D6" s="19">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Almost certain",'4. Risk Register'!$G$5:$G$62,"Moderate")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Almost certain",'4. Risk Register'!$G$5:$G$66,"Moderate")</f>
         <v/>
       </c>
       <c r="E6" s="20">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Almost certain",'4. Risk Register'!$G$5:$G$62,"Major")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Almost certain",'4. Risk Register'!$G$5:$G$66,"Major")</f>
         <v/>
       </c>
       <c r="F6" s="20">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Almost certain",'4. Risk Register'!$G$5:$G$62,"Severe")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Almost certain",'4. Risk Register'!$G$5:$G$66,"Severe")</f>
         <v/>
       </c>
       <c r="H6" s="21" t="inlineStr">
@@ -5913,11 +6185,11 @@
         </is>
       </c>
       <c r="I6" s="7">
-        <f>COUNTIF('4. Risk Register'!$I$5:$I$62,"Critical")</f>
+        <f>COUNTIF('4. Risk Register'!$I$5:$I$66,"Critical")</f>
         <v/>
       </c>
       <c r="J6" s="7">
-        <f>COUNTIF('4. Risk Register'!$M$5:$M$62,"Critical")</f>
+        <f>COUNTIF('4. Risk Register'!$M$5:$M$66,"Critical")</f>
         <v/>
       </c>
     </row>
@@ -5928,23 +6200,23 @@
         </is>
       </c>
       <c r="B7" s="22">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Likely",'4. Risk Register'!$G$5:$G$62,"Insignificant")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Likely",'4. Risk Register'!$G$5:$G$66,"Insignificant")</f>
         <v/>
       </c>
       <c r="C7" s="18">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Likely",'4. Risk Register'!$G$5:$G$62,"Minor")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Likely",'4. Risk Register'!$G$5:$G$66,"Minor")</f>
         <v/>
       </c>
       <c r="D7" s="19">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Likely",'4. Risk Register'!$G$5:$G$62,"Moderate")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Likely",'4. Risk Register'!$G$5:$G$66,"Moderate")</f>
         <v/>
       </c>
       <c r="E7" s="19">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Likely",'4. Risk Register'!$G$5:$G$62,"Major")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Likely",'4. Risk Register'!$G$5:$G$66,"Major")</f>
         <v/>
       </c>
       <c r="F7" s="20">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Likely",'4. Risk Register'!$G$5:$G$62,"Severe")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Likely",'4. Risk Register'!$G$5:$G$66,"Severe")</f>
         <v/>
       </c>
       <c r="H7" s="23" t="inlineStr">
@@ -5953,11 +6225,11 @@
         </is>
       </c>
       <c r="I7" s="7">
-        <f>COUNTIF('4. Risk Register'!$I$5:$I$62,"High")</f>
+        <f>COUNTIF('4. Risk Register'!$I$5:$I$66,"High")</f>
         <v/>
       </c>
       <c r="J7" s="7">
-        <f>COUNTIF('4. Risk Register'!$M$5:$M$62,"High")</f>
+        <f>COUNTIF('4. Risk Register'!$M$5:$M$66,"High")</f>
         <v/>
       </c>
     </row>
@@ -5968,23 +6240,23 @@
         </is>
       </c>
       <c r="B8" s="22">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Possible",'4. Risk Register'!$G$5:$G$62,"Insignificant")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Possible",'4. Risk Register'!$G$5:$G$66,"Insignificant")</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Possible",'4. Risk Register'!$G$5:$G$62,"Minor")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Possible",'4. Risk Register'!$G$5:$G$66,"Minor")</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Possible",'4. Risk Register'!$G$5:$G$62,"Moderate")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Possible",'4. Risk Register'!$G$5:$G$66,"Moderate")</f>
         <v/>
       </c>
       <c r="E8" s="19">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Possible",'4. Risk Register'!$G$5:$G$62,"Major")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Possible",'4. Risk Register'!$G$5:$G$66,"Major")</f>
         <v/>
       </c>
       <c r="F8" s="19">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Possible",'4. Risk Register'!$G$5:$G$62,"Severe")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Possible",'4. Risk Register'!$G$5:$G$66,"Severe")</f>
         <v/>
       </c>
       <c r="H8" s="24" t="inlineStr">
@@ -5993,11 +6265,11 @@
         </is>
       </c>
       <c r="I8" s="7">
-        <f>COUNTIF('4. Risk Register'!$I$5:$I$62,"Medium")</f>
+        <f>COUNTIF('4. Risk Register'!$I$5:$I$66,"Medium")</f>
         <v/>
       </c>
       <c r="J8" s="7">
-        <f>COUNTIF('4. Risk Register'!$M$5:$M$62,"Medium")</f>
+        <f>COUNTIF('4. Risk Register'!$M$5:$M$66,"Medium")</f>
         <v/>
       </c>
     </row>
@@ -6008,23 +6280,23 @@
         </is>
       </c>
       <c r="B9" s="22">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Unlikely",'4. Risk Register'!$G$5:$G$62,"Insignificant")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Unlikely",'4. Risk Register'!$G$5:$G$66,"Insignificant")</f>
         <v/>
       </c>
       <c r="C9" s="22">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Unlikely",'4. Risk Register'!$G$5:$G$62,"Minor")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Unlikely",'4. Risk Register'!$G$5:$G$66,"Minor")</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Unlikely",'4. Risk Register'!$G$5:$G$62,"Moderate")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Unlikely",'4. Risk Register'!$G$5:$G$66,"Moderate")</f>
         <v/>
       </c>
       <c r="E9" s="18">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Unlikely",'4. Risk Register'!$G$5:$G$62,"Major")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Unlikely",'4. Risk Register'!$G$5:$G$66,"Major")</f>
         <v/>
       </c>
       <c r="F9" s="19">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Unlikely",'4. Risk Register'!$G$5:$G$62,"Severe")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Unlikely",'4. Risk Register'!$G$5:$G$66,"Severe")</f>
         <v/>
       </c>
       <c r="H9" s="25" t="inlineStr">
@@ -6033,11 +6305,11 @@
         </is>
       </c>
       <c r="I9" s="7">
-        <f>COUNTIF('4. Risk Register'!$I$5:$I$62,"Low")</f>
+        <f>COUNTIF('4. Risk Register'!$I$5:$I$66,"Low")</f>
         <v/>
       </c>
       <c r="J9" s="7">
-        <f>COUNTIF('4. Risk Register'!$M$5:$M$62,"Low")</f>
+        <f>COUNTIF('4. Risk Register'!$M$5:$M$66,"Low")</f>
         <v/>
       </c>
     </row>
@@ -6048,23 +6320,23 @@
         </is>
       </c>
       <c r="B10" s="22">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Rare",'4. Risk Register'!$G$5:$G$62,"Insignificant")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Rare",'4. Risk Register'!$G$5:$G$66,"Insignificant")</f>
         <v/>
       </c>
       <c r="C10" s="22">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Rare",'4. Risk Register'!$G$5:$G$62,"Minor")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Rare",'4. Risk Register'!$G$5:$G$66,"Minor")</f>
         <v/>
       </c>
       <c r="D10" s="22">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Rare",'4. Risk Register'!$G$5:$G$62,"Moderate")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Rare",'4. Risk Register'!$G$5:$G$66,"Moderate")</f>
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Rare",'4. Risk Register'!$G$5:$G$62,"Major")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Rare",'4. Risk Register'!$G$5:$G$66,"Major")</f>
         <v/>
       </c>
       <c r="F10" s="18">
-        <f>COUNTIFS('4. Risk Register'!$A$5:$A$62,"Yes",'4. Risk Register'!$F$5:$F$62,"Rare",'4. Risk Register'!$G$5:$G$62,"Severe")</f>
+        <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Rare",'4. Risk Register'!$G$5:$G$66,"Severe")</f>
         <v/>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -6151,27 +6423,27 @@
         </is>
       </c>
       <c r="D16" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Governance &amp; Accountability",'4. Risk Register'!$A$5:$A$62,"Yes")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Governance &amp; Accountability",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
         <v/>
       </c>
       <c r="E16" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Governance &amp; Accountability",'4. Risk Register'!$M$5:$M$62,"Critical")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Governance &amp; Accountability",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
         <v/>
       </c>
       <c r="F16" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Governance &amp; Accountability",'4. Risk Register'!$M$5:$M$62,"High")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Governance &amp; Accountability",'4. Risk Register'!$M$5:$M$66,"High")</f>
         <v/>
       </c>
       <c r="G16" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Governance &amp; Accountability",'4. Risk Register'!$M$5:$M$62,"Medium")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Governance &amp; Accountability",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
         <v/>
       </c>
       <c r="H16" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Governance &amp; Accountability",'4. Risk Register'!$M$5:$M$62,"Low")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Governance &amp; Accountability",'4. Risk Register'!$M$5:$M$66,"Low")</f>
         <v/>
       </c>
       <c r="I16" s="7">
-        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$62,'4. Risk Register'!$C$5:$C$62,"Governance &amp; Accountability",'4. Risk Register'!$A$5:$A$62,"Yes"),1),"-")</f>
+        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Governance &amp; Accountability",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
         <v/>
       </c>
     </row>
@@ -6182,27 +6454,27 @@
         </is>
       </c>
       <c r="D17" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Legal, Regulatory &amp; Compliance",'4. Risk Register'!$A$5:$A$62,"Yes")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Legal, Regulatory &amp; Compliance",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
         <v/>
       </c>
       <c r="E17" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Legal, Regulatory &amp; Compliance",'4. Risk Register'!$M$5:$M$62,"Critical")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Legal, Regulatory &amp; Compliance",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
         <v/>
       </c>
       <c r="F17" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Legal, Regulatory &amp; Compliance",'4. Risk Register'!$M$5:$M$62,"High")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Legal, Regulatory &amp; Compliance",'4. Risk Register'!$M$5:$M$66,"High")</f>
         <v/>
       </c>
       <c r="G17" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Legal, Regulatory &amp; Compliance",'4. Risk Register'!$M$5:$M$62,"Medium")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Legal, Regulatory &amp; Compliance",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
         <v/>
       </c>
       <c r="H17" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Legal, Regulatory &amp; Compliance",'4. Risk Register'!$M$5:$M$62,"Low")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Legal, Regulatory &amp; Compliance",'4. Risk Register'!$M$5:$M$66,"Low")</f>
         <v/>
       </c>
       <c r="I17" s="7">
-        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$62,'4. Risk Register'!$C$5:$C$62,"Legal, Regulatory &amp; Compliance",'4. Risk Register'!$A$5:$A$62,"Yes"),1),"-")</f>
+        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Legal, Regulatory &amp; Compliance",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
         <v/>
       </c>
     </row>
@@ -6213,27 +6485,27 @@
         </is>
       </c>
       <c r="D18" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Fairness, Bias &amp; Human Rights",'4. Risk Register'!$A$5:$A$62,"Yes")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Fairness, Bias &amp; Human Rights",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
         <v/>
       </c>
       <c r="E18" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Fairness, Bias &amp; Human Rights",'4. Risk Register'!$M$5:$M$62,"Critical")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Fairness, Bias &amp; Human Rights",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
         <v/>
       </c>
       <c r="F18" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Fairness, Bias &amp; Human Rights",'4. Risk Register'!$M$5:$M$62,"High")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Fairness, Bias &amp; Human Rights",'4. Risk Register'!$M$5:$M$66,"High")</f>
         <v/>
       </c>
       <c r="G18" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Fairness, Bias &amp; Human Rights",'4. Risk Register'!$M$5:$M$62,"Medium")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Fairness, Bias &amp; Human Rights",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
         <v/>
       </c>
       <c r="H18" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Fairness, Bias &amp; Human Rights",'4. Risk Register'!$M$5:$M$62,"Low")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Fairness, Bias &amp; Human Rights",'4. Risk Register'!$M$5:$M$66,"Low")</f>
         <v/>
       </c>
       <c r="I18" s="7">
-        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$62,'4. Risk Register'!$C$5:$C$62,"Fairness, Bias &amp; Human Rights",'4. Risk Register'!$A$5:$A$62,"Yes"),1),"-")</f>
+        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Fairness, Bias &amp; Human Rights",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
         <v/>
       </c>
     </row>
@@ -6244,27 +6516,27 @@
         </is>
       </c>
       <c r="D19" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Privacy &amp; Data Protection",'4. Risk Register'!$A$5:$A$62,"Yes")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Privacy &amp; Data Protection",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
         <v/>
       </c>
       <c r="E19" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Privacy &amp; Data Protection",'4. Risk Register'!$M$5:$M$62,"Critical")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Privacy &amp; Data Protection",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
         <v/>
       </c>
       <c r="F19" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Privacy &amp; Data Protection",'4. Risk Register'!$M$5:$M$62,"High")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Privacy &amp; Data Protection",'4. Risk Register'!$M$5:$M$66,"High")</f>
         <v/>
       </c>
       <c r="G19" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Privacy &amp; Data Protection",'4. Risk Register'!$M$5:$M$62,"Medium")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Privacy &amp; Data Protection",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
         <v/>
       </c>
       <c r="H19" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Privacy &amp; Data Protection",'4. Risk Register'!$M$5:$M$62,"Low")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Privacy &amp; Data Protection",'4. Risk Register'!$M$5:$M$66,"Low")</f>
         <v/>
       </c>
       <c r="I19" s="7">
-        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$62,'4. Risk Register'!$C$5:$C$62,"Privacy &amp; Data Protection",'4. Risk Register'!$A$5:$A$62,"Yes"),1),"-")</f>
+        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Privacy &amp; Data Protection",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
         <v/>
       </c>
     </row>
@@ -6275,27 +6547,27 @@
         </is>
       </c>
       <c r="D20" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Data Quality &amp; Integrity",'4. Risk Register'!$A$5:$A$62,"Yes")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Data Quality &amp; Integrity",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
         <v/>
       </c>
       <c r="E20" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Data Quality &amp; Integrity",'4. Risk Register'!$M$5:$M$62,"Critical")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Data Quality &amp; Integrity",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
         <v/>
       </c>
       <c r="F20" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Data Quality &amp; Integrity",'4. Risk Register'!$M$5:$M$62,"High")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Data Quality &amp; Integrity",'4. Risk Register'!$M$5:$M$66,"High")</f>
         <v/>
       </c>
       <c r="G20" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Data Quality &amp; Integrity",'4. Risk Register'!$M$5:$M$62,"Medium")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Data Quality &amp; Integrity",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
         <v/>
       </c>
       <c r="H20" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Data Quality &amp; Integrity",'4. Risk Register'!$M$5:$M$62,"Low")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Data Quality &amp; Integrity",'4. Risk Register'!$M$5:$M$66,"Low")</f>
         <v/>
       </c>
       <c r="I20" s="7">
-        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$62,'4. Risk Register'!$C$5:$C$62,"Data Quality &amp; Integrity",'4. Risk Register'!$A$5:$A$62,"Yes"),1),"-")</f>
+        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Data Quality &amp; Integrity",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
         <v/>
       </c>
     </row>
@@ -6306,27 +6578,27 @@
         </is>
       </c>
       <c r="D21" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Model Performance, Reliability &amp; Robustness",'4. Risk Register'!$A$5:$A$62,"Yes")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Model Performance, Reliability &amp; Robustness",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
         <v/>
       </c>
       <c r="E21" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Model Performance, Reliability &amp; Robustness",'4. Risk Register'!$M$5:$M$62,"Critical")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Model Performance, Reliability &amp; Robustness",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
         <v/>
       </c>
       <c r="F21" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Model Performance, Reliability &amp; Robustness",'4. Risk Register'!$M$5:$M$62,"High")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Model Performance, Reliability &amp; Robustness",'4. Risk Register'!$M$5:$M$66,"High")</f>
         <v/>
       </c>
       <c r="G21" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Model Performance, Reliability &amp; Robustness",'4. Risk Register'!$M$5:$M$62,"Medium")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Model Performance, Reliability &amp; Robustness",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
         <v/>
       </c>
       <c r="H21" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Model Performance, Reliability &amp; Robustness",'4. Risk Register'!$M$5:$M$62,"Low")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Model Performance, Reliability &amp; Robustness",'4. Risk Register'!$M$5:$M$66,"Low")</f>
         <v/>
       </c>
       <c r="I21" s="7">
-        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$62,'4. Risk Register'!$C$5:$C$62,"Model Performance, Reliability &amp; Robustness",'4. Risk Register'!$A$5:$A$62,"Yes"),1),"-")</f>
+        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Model Performance, Reliability &amp; Robustness",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
         <v/>
       </c>
     </row>
@@ -6337,27 +6609,27 @@
         </is>
       </c>
       <c r="D22" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Transparency, Explainability &amp; Contestability",'4. Risk Register'!$A$5:$A$62,"Yes")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Transparency, Explainability &amp; Contestability",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
         <v/>
       </c>
       <c r="E22" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Transparency, Explainability &amp; Contestability",'4. Risk Register'!$M$5:$M$62,"Critical")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Transparency, Explainability &amp; Contestability",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
         <v/>
       </c>
       <c r="F22" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Transparency, Explainability &amp; Contestability",'4. Risk Register'!$M$5:$M$62,"High")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Transparency, Explainability &amp; Contestability",'4. Risk Register'!$M$5:$M$66,"High")</f>
         <v/>
       </c>
       <c r="G22" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Transparency, Explainability &amp; Contestability",'4. Risk Register'!$M$5:$M$62,"Medium")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Transparency, Explainability &amp; Contestability",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
         <v/>
       </c>
       <c r="H22" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Transparency, Explainability &amp; Contestability",'4. Risk Register'!$M$5:$M$62,"Low")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Transparency, Explainability &amp; Contestability",'4. Risk Register'!$M$5:$M$66,"Low")</f>
         <v/>
       </c>
       <c r="I22" s="7">
-        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$62,'4. Risk Register'!$C$5:$C$62,"Transparency, Explainability &amp; Contestability",'4. Risk Register'!$A$5:$A$62,"Yes"),1),"-")</f>
+        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Transparency, Explainability &amp; Contestability",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
         <v/>
       </c>
     </row>
@@ -6368,27 +6640,27 @@
         </is>
       </c>
       <c r="D23" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Security of AI Systems",'4. Risk Register'!$A$5:$A$62,"Yes")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Security of AI Systems",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
         <v/>
       </c>
       <c r="E23" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Security of AI Systems",'4. Risk Register'!$M$5:$M$62,"Critical")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Security of AI Systems",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
         <v/>
       </c>
       <c r="F23" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Security of AI Systems",'4. Risk Register'!$M$5:$M$62,"High")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Security of AI Systems",'4. Risk Register'!$M$5:$M$66,"High")</f>
         <v/>
       </c>
       <c r="G23" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Security of AI Systems",'4. Risk Register'!$M$5:$M$62,"Medium")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Security of AI Systems",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
         <v/>
       </c>
       <c r="H23" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Security of AI Systems",'4. Risk Register'!$M$5:$M$62,"Low")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Security of AI Systems",'4. Risk Register'!$M$5:$M$66,"Low")</f>
         <v/>
       </c>
       <c r="I23" s="7">
-        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$62,'4. Risk Register'!$C$5:$C$62,"Security of AI Systems",'4. Risk Register'!$A$5:$A$62,"Yes"),1),"-")</f>
+        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Security of AI Systems",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
         <v/>
       </c>
     </row>
@@ -6399,27 +6671,27 @@
         </is>
       </c>
       <c r="D24" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Human Oversight &amp; Autonomy",'4. Risk Register'!$A$5:$A$62,"Yes")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Human Oversight &amp; Autonomy",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
         <v/>
       </c>
       <c r="E24" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Human Oversight &amp; Autonomy",'4. Risk Register'!$M$5:$M$62,"Critical")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Human Oversight &amp; Autonomy",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
         <v/>
       </c>
       <c r="F24" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Human Oversight &amp; Autonomy",'4. Risk Register'!$M$5:$M$62,"High")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Human Oversight &amp; Autonomy",'4. Risk Register'!$M$5:$M$66,"High")</f>
         <v/>
       </c>
       <c r="G24" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Human Oversight &amp; Autonomy",'4. Risk Register'!$M$5:$M$62,"Medium")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Human Oversight &amp; Autonomy",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
         <v/>
       </c>
       <c r="H24" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Human Oversight &amp; Autonomy",'4. Risk Register'!$M$5:$M$62,"Low")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Human Oversight &amp; Autonomy",'4. Risk Register'!$M$5:$M$66,"Low")</f>
         <v/>
       </c>
       <c r="I24" s="7">
-        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$62,'4. Risk Register'!$C$5:$C$62,"Human Oversight &amp; Autonomy",'4. Risk Register'!$A$5:$A$62,"Yes"),1),"-")</f>
+        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Human Oversight &amp; Autonomy",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
         <v/>
       </c>
     </row>
@@ -6430,27 +6702,27 @@
         </is>
       </c>
       <c r="D25" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Third-Party &amp; Supply Chain",'4. Risk Register'!$A$5:$A$62,"Yes")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Third-Party &amp; Supply Chain",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
         <v/>
       </c>
       <c r="E25" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Third-Party &amp; Supply Chain",'4. Risk Register'!$M$5:$M$62,"Critical")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Third-Party &amp; Supply Chain",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
         <v/>
       </c>
       <c r="F25" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Third-Party &amp; Supply Chain",'4. Risk Register'!$M$5:$M$62,"High")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Third-Party &amp; Supply Chain",'4. Risk Register'!$M$5:$M$66,"High")</f>
         <v/>
       </c>
       <c r="G25" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Third-Party &amp; Supply Chain",'4. Risk Register'!$M$5:$M$62,"Medium")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Third-Party &amp; Supply Chain",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
         <v/>
       </c>
       <c r="H25" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Third-Party &amp; Supply Chain",'4. Risk Register'!$M$5:$M$62,"Low")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Third-Party &amp; Supply Chain",'4. Risk Register'!$M$5:$M$66,"Low")</f>
         <v/>
       </c>
       <c r="I25" s="7">
-        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$62,'4. Risk Register'!$C$5:$C$62,"Third-Party &amp; Supply Chain",'4. Risk Register'!$A$5:$A$62,"Yes"),1),"-")</f>
+        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Third-Party &amp; Supply Chain",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
         <v/>
       </c>
     </row>
@@ -6461,27 +6733,27 @@
         </is>
       </c>
       <c r="D26" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Operational, Financial &amp; Sustainability",'4. Risk Register'!$A$5:$A$62,"Yes")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Operational, Financial &amp; Sustainability",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
         <v/>
       </c>
       <c r="E26" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Operational, Financial &amp; Sustainability",'4. Risk Register'!$M$5:$M$62,"Critical")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Operational, Financial &amp; Sustainability",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
         <v/>
       </c>
       <c r="F26" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Operational, Financial &amp; Sustainability",'4. Risk Register'!$M$5:$M$62,"High")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Operational, Financial &amp; Sustainability",'4. Risk Register'!$M$5:$M$66,"High")</f>
         <v/>
       </c>
       <c r="G26" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Operational, Financial &amp; Sustainability",'4. Risk Register'!$M$5:$M$62,"Medium")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Operational, Financial &amp; Sustainability",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
         <v/>
       </c>
       <c r="H26" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Operational, Financial &amp; Sustainability",'4. Risk Register'!$M$5:$M$62,"Low")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Operational, Financial &amp; Sustainability",'4. Risk Register'!$M$5:$M$66,"Low")</f>
         <v/>
       </c>
       <c r="I26" s="7">
-        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$62,'4. Risk Register'!$C$5:$C$62,"Operational, Financial &amp; Sustainability",'4. Risk Register'!$A$5:$A$62,"Yes"),1),"-")</f>
+        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Operational, Financial &amp; Sustainability",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
         <v/>
       </c>
     </row>
@@ -6492,27 +6764,27 @@
         </is>
       </c>
       <c r="D27" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Societal, Reputational &amp; AI-Enabled Threats",'4. Risk Register'!$A$5:$A$62,"Yes")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Societal, Reputational &amp; AI-Enabled Threats",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
         <v/>
       </c>
       <c r="E27" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Societal, Reputational &amp; AI-Enabled Threats",'4. Risk Register'!$M$5:$M$62,"Critical")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Societal, Reputational &amp; AI-Enabled Threats",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
         <v/>
       </c>
       <c r="F27" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Societal, Reputational &amp; AI-Enabled Threats",'4. Risk Register'!$M$5:$M$62,"High")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Societal, Reputational &amp; AI-Enabled Threats",'4. Risk Register'!$M$5:$M$66,"High")</f>
         <v/>
       </c>
       <c r="G27" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Societal, Reputational &amp; AI-Enabled Threats",'4. Risk Register'!$M$5:$M$62,"Medium")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Societal, Reputational &amp; AI-Enabled Threats",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
         <v/>
       </c>
       <c r="H27" s="7">
-        <f>COUNTIFS('4. Risk Register'!$C$5:$C$62,"Societal, Reputational &amp; AI-Enabled Threats",'4. Risk Register'!$M$5:$M$62,"Low")</f>
+        <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Societal, Reputational &amp; AI-Enabled Threats",'4. Risk Register'!$M$5:$M$66,"Low")</f>
         <v/>
       </c>
       <c r="I27" s="7">
-        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$62,'4. Risk Register'!$C$5:$C$62,"Societal, Reputational &amp; AI-Enabled Threats",'4. Risk Register'!$A$5:$A$62,"Yes"),1),"-")</f>
+        <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Societal, Reputational &amp; AI-Enabled Threats",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
         <v/>
       </c>
     </row>
@@ -6573,34 +6845,34 @@
         <v>1</v>
       </c>
       <c r="B32" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,1),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,1),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="C32" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,1),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,1),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D32" s="12" t="n"/>
       <c r="E32" s="12" t="n"/>
       <c r="F32" s="12" t="n"/>
       <c r="G32" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,1),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,1),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="H32" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,1),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,1),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="I32" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,1),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,1),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="J32" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,1),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,1),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="K32" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,1),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,1),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -6609,34 +6881,34 @@
         <v>2</v>
       </c>
       <c r="B33" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,2),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,2),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="C33" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,2),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,2),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D33" s="12" t="n"/>
       <c r="E33" s="12" t="n"/>
       <c r="F33" s="12" t="n"/>
       <c r="G33" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,2),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,2),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="H33" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,2),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,2),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="I33" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,2),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,2),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="J33" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,2),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,2),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="K33" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,2),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,2),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -6645,34 +6917,34 @@
         <v>3</v>
       </c>
       <c r="B34" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,3),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,3),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="C34" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,3),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,3),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D34" s="12" t="n"/>
       <c r="E34" s="12" t="n"/>
       <c r="F34" s="12" t="n"/>
       <c r="G34" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,3),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,3),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="H34" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,3),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,3),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="I34" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,3),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,3),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="J34" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,3),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,3),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="K34" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,3),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,3),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -6681,34 +6953,34 @@
         <v>4</v>
       </c>
       <c r="B35" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,4),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,4),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="C35" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,4),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,4),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D35" s="12" t="n"/>
       <c r="E35" s="12" t="n"/>
       <c r="F35" s="12" t="n"/>
       <c r="G35" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,4),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,4),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="H35" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,4),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,4),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="I35" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,4),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,4),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="J35" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,4),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,4),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="K35" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,4),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,4),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -6717,34 +6989,34 @@
         <v>5</v>
       </c>
       <c r="B36" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,5),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,5),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="C36" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,5),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,5),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D36" s="12" t="n"/>
       <c r="E36" s="12" t="n"/>
       <c r="F36" s="12" t="n"/>
       <c r="G36" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,5),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,5),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="H36" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,5),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,5),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="I36" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,5),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,5),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="J36" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,5),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,5),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="K36" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,5),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,5),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -6753,34 +7025,34 @@
         <v>6</v>
       </c>
       <c r="B37" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,6),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,6),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="C37" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,6),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,6),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D37" s="12" t="n"/>
       <c r="E37" s="12" t="n"/>
       <c r="F37" s="12" t="n"/>
       <c r="G37" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,6),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,6),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="H37" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,6),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,6),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="I37" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,6),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,6),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="J37" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,6),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,6),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="K37" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,6),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,6),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -6789,34 +7061,34 @@
         <v>7</v>
       </c>
       <c r="B38" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,7),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,7),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="C38" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,7),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,7),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D38" s="12" t="n"/>
       <c r="E38" s="12" t="n"/>
       <c r="F38" s="12" t="n"/>
       <c r="G38" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,7),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,7),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="H38" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,7),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,7),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="I38" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,7),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,7),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="J38" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,7),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,7),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="K38" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,7),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,7),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -6825,34 +7097,34 @@
         <v>8</v>
       </c>
       <c r="B39" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,8),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,8),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="C39" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,8),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,8),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D39" s="12" t="n"/>
       <c r="E39" s="12" t="n"/>
       <c r="F39" s="12" t="n"/>
       <c r="G39" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,8),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,8),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="H39" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,8),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,8),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="I39" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,8),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,8),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="J39" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,8),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,8),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="K39" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,8),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,8),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -6861,34 +7133,34 @@
         <v>9</v>
       </c>
       <c r="B40" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,9),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,9),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="C40" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,9),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,9),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D40" s="12" t="n"/>
       <c r="E40" s="12" t="n"/>
       <c r="F40" s="12" t="n"/>
       <c r="G40" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,9),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,9),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="H40" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,9),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,9),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="I40" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,9),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,9),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="J40" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,9),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,9),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="K40" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,9),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,9),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -6897,34 +7169,34 @@
         <v>10</v>
       </c>
       <c r="B41" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,10),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,10),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="C41" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,10),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,10),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D41" s="12" t="n"/>
       <c r="E41" s="12" t="n"/>
       <c r="F41" s="12" t="n"/>
       <c r="G41" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,10),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,10),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="H41" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,10),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,10),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="I41" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,10),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,10),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="J41" s="12">
-        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,10),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,10),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="K41" s="7">
-        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$62,MATCH(LARGE('4. Risk Register'!$V$5:$V$62,10),'4. Risk Register'!$V$5:$V$62,0)),"")</f>
+        <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,10),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -7116,8 +7388,9 @@
       <formula>"Prohibited"</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <printOptions gridLines="0"/>
+  <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.25" footer="0.25"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -7129,7 +7402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -7151,7 +7424,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>48 risks in 12 categories. Sources: NIST AI RMF &amp; AI 600-1, ISO/IEC 23894, EU AI Act, OWASP LLM / Agentic Top 10, MITRE ATLAS, MIT AI Risk Repository, GT AI Ready7. RCM IDs refer to GT AI RCM v2.0.</t>
+          <t>52 risks in 12 categories. Sources: NIST AI RMF &amp; AI 600-1, ISO/IEC 23894, EU AI Act, OWASP LLM / Agentic Top 10, MITRE ATLAS, MIT AI Risk Repository, GT AI Ready7. RCM IDs refer to GT AI RCM v2.1; agent risks draw on ISACA Securing AI Agents (2026).</t>
         </is>
       </c>
     </row>
@@ -7183,7 +7456,7 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>RCM v2.0 controls</t>
+          <t>RCM v2.1 controls</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -8120,44 +8393,44 @@
     <row r="30" ht="36" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>TRA-01</t>
+          <t>PER-05</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Transparency, Explainability &amp; Contestability</t>
+          <t>Model Performance, Reliability &amp; Robustness</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Undisclosed AI interaction or content</t>
+          <t>Uncontrolled prompt / configuration changes</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Users are unaware they interact with AI or that content is AI-generated.</t>
+          <t>Changes to prompts, guardrails, tool permissions or retrieval sources degrade safety or behaviour without regression testing.</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>EU AI Act Art. 50</t>
+          <t>ISACA Securing AI Agents (2026)</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>CO-1, LC-7</t>
+          <t>LC-12</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>AI touchpoints lacking disclosure</t>
+          <t>Releases without passing LLM regression suite</t>
         </is>
       </c>
     </row>
     <row r="31" ht="36" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>TRA-02</t>
+          <t>TRA-01</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -8167,34 +8440,34 @@
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>Unexplainable decisions</t>
+          <t>Undisclosed AI interaction or content</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Organisation cannot explain AI-supported decisions to affected persons, regulators or auditors.</t>
+          <t>Users are unaware they interact with AI or that content is AI-generated.</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>EU AI Act Art. 13, 86; NIST IR 8312</t>
+          <t>EU AI Act Art. 50</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>RS-4, LC-4</t>
+          <t>CO-1, LC-7</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>Explanation requests not satisfied</t>
+          <t>AI touchpoints lacking disclosure</t>
         </is>
       </c>
     </row>
     <row r="32" ht="36" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>TRA-03</t>
+          <t>TRA-02</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -8204,34 +8477,34 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>No effective contest or redress route</t>
+          <t>Unexplainable decisions</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Affected persons cannot challenge or obtain human review of AI-supported decisions.</t>
+          <t>Organisation cannot explain AI-supported decisions to affected persons, regulators or auditors.</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>EU AI Act Art. 86; NSW AIAF</t>
+          <t>EU AI Act Art. 13, 86; NIST IR 8312</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>CO-3, PR-5</t>
+          <t>RS-4, LC-4</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Appeals exceeding SLA</t>
+          <t>Explanation requests not satisfied</t>
         </is>
       </c>
     </row>
     <row r="33" ht="36" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>TRA-04</t>
+          <t>TRA-03</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -8241,71 +8514,71 @@
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>Inadequate documentation and records</t>
+          <t>No effective contest or redress route</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Technical documentation, logs or decisions are insufficient for audit or regulatory inspection.</t>
+          <t>Affected persons cannot challenge or obtain human review of AI-supported decisions.</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>EU AI Act Art. 11-12, 18-19</t>
+          <t>EU AI Act Art. 86; NSW AIAF</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>LC-4, OM-2, RO-3</t>
+          <t>CO-3, PR-5</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Systems with incomplete documentation pack</t>
+          <t>Appeals exceeding SLA</t>
         </is>
       </c>
     </row>
     <row r="34" ht="36" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>SEC-01</t>
+          <t>TRA-04</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Security of AI Systems</t>
+          <t>Transparency, Explainability &amp; Contestability</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Prompt injection and jailbreak</t>
+          <t>Inadequate documentation and records</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Attacker manipulates model behaviour via direct or indirect (embedded content) instructions.</t>
+          <t>Technical documentation, logs or decisions are insufficient for audit or regulatory inspection.</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>OWASP LLM01:2025; MITRE ATLAS</t>
+          <t>EU AI Act Art. 11-12, 18-19</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>SE-6</t>
+          <t>LC-4, OM-2, RO-3</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Blocked injection attempts / bypasses in testing</t>
+          <t>Systems with incomplete documentation pack</t>
         </is>
       </c>
     </row>
     <row r="35" ht="36" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>SEC-02</t>
+          <t>SEC-01</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -8315,34 +8588,34 @@
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>Data or model poisoning</t>
+          <t>Prompt injection and jailbreak</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Training, fine-tuning or retrieval data is manipulated to corrupt outputs or insert backdoors.</t>
+          <t>Attacker manipulates model behaviour via direct or indirect (embedded content) instructions.</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>OWASP LLM04:2025; NIST AI 100-2</t>
+          <t>OWASP LLM01:2025; MITRE ATLAS</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>SE-6, LC-1, SE-7</t>
+          <t>SE-6</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Integrity check failures</t>
+          <t>Blocked injection attempts / bypasses in testing</t>
         </is>
       </c>
     </row>
     <row r="36" ht="36" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>SEC-03</t>
+          <t>SEC-02</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -8352,34 +8625,34 @@
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Model theft, extraction or inversion</t>
+          <t>Data or model poisoning</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Model weights, system prompts or training data are extracted.</t>
+          <t>Training, fine-tuning or retrieval data is manipulated to corrupt outputs or insert backdoors.</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>OWASP LLM07/LLM10:2025; MITRE ATLAS</t>
+          <t>OWASP LLM04:2025; NIST AI 100-2</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>SE-4, SE-6</t>
+          <t>SE-6, LC-1, SE-7</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Anomalous query volumes</t>
+          <t>Integrity check failures</t>
         </is>
       </c>
     </row>
     <row r="37" ht="36" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>SEC-04</t>
+          <t>SEC-03</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -8389,34 +8662,34 @@
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>Insecure integration and excessive privilege</t>
+          <t>Model theft, extraction or inversion</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>AI components have excessive permissions or insecure APIs/plugins, enabling unauthorised actions.</t>
+          <t>Model weights, system prompts or training data are extracted.</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>OWASP LLM05/LLM06:2025; AI Ready7 4.2-4.3</t>
+          <t>OWASP LLM07/LLM10:2025; MITRE ATLAS</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>SE-2, LC-8</t>
+          <t>SE-4, SE-6</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>Agents / integrations with privileged standing access</t>
+          <t>Anomalous query volumes</t>
         </is>
       </c>
     </row>
     <row r="38" ht="36" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>SEC-05</t>
+          <t>SEC-04</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -8426,145 +8699,145 @@
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Compromised AI supply chain</t>
+          <t>Insecure integration and excessive privilege</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Malicious or vulnerable third-party models, libraries, plugins or MCP servers.</t>
+          <t>AI components have excessive permissions or insecure APIs/plugins, enabling unauthorised actions.</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>OWASP LLM03:2025; CISA AI Data Security</t>
+          <t>OWASP LLM05/LLM06:2025; AI Ready7 4.2-4.3</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>SE-7</t>
+          <t>SE-2, LC-8</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>Unscanned model artefacts</t>
+          <t>Agents / integrations with privileged standing access</t>
         </is>
       </c>
     </row>
     <row r="39" ht="36" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>HUM-01</t>
+          <t>SEC-06</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Human Oversight &amp; Autonomy</t>
+          <t>Security of AI Systems</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>Automation bias and over-reliance</t>
+          <t>Agent memory poisoning &amp; cross-session leakage</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Users accept AI outputs without adequate scrutiny, eroding professional judgement.</t>
+          <t>Poisoned or unauthorised content persists in agent memory / vector stores, or context leaks across users, sessions or tenants.</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>EU AI Act Art. 14(4)(b); NIST AI 600-1 (Human-AI configuration)</t>
+          <t>ISACA Securing AI Agents (2026); OWASP LLM08:2025</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>RS-1, GL-4, LC-7</t>
+          <t>SE-8</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>Override / challenge rate</t>
+          <t>Cross-tenant retrieval test failures</t>
         </is>
       </c>
     </row>
     <row r="40" ht="36" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>HUM-02</t>
+          <t>SEC-07</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Human Oversight &amp; Autonomy</t>
+          <t>Security of AI Systems</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Ineffective human oversight</t>
+          <t>Unsafe code execution, SSRF &amp; sandbox escape</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Oversight persons lack competence, authority, time or information to intervene.</t>
+          <t>Agent-generated code or tool calls reach internal networks, cloud metadata services or production secrets.</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>EU AI Act Art. 14, 26(2)</t>
+          <t>ISACA Securing AI Agents (2026); CWS ISO 42001 checklist 33</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>RS-1, GL-4</t>
+          <t>SE-9, SE-10</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>Oversight roles without training</t>
+          <t>Blocked egress / SSRF attempts</t>
         </is>
       </c>
     </row>
     <row r="41" ht="36" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>HUM-03</t>
+          <t>SEC-05</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Human Oversight &amp; Autonomy</t>
+          <t>Security of AI Systems</t>
         </is>
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>Unbounded autonomous agent actions</t>
+          <t>Compromised AI supply chain</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>AI agents take high-impact actions (payments, communications, code execution) without adequate limits or approval.</t>
+          <t>Malicious or vulnerable third-party models, libraries, plugins or MCP servers.</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>OWASP Agentic Top 10; Singapore Agentic AI framework</t>
+          <t>OWASP LLM03:2025; CISA AI Data Security</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>LC-8</t>
+          <t>SE-7</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>High-impact agent actions without approval</t>
+          <t>Unscanned model artefacts</t>
         </is>
       </c>
     </row>
     <row r="42" ht="36" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>HUM-04</t>
+          <t>HUM-01</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -8574,408 +8847,557 @@
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Adverse workforce impact</t>
+          <t>Automation bias and over-reliance</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>AI adoption causes skills erosion, job anxiety or unconsulted changes to working conditions.</t>
+          <t>Users accept AI outputs without adequate scrutiny, eroding professional judgement.</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>EU AI Act Art. 26(7); AI Ready7 3.4</t>
+          <t>EU AI Act Art. 14(4)(b); NIST AI 600-1 (Human-AI configuration)</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>RS-9, GL-4</t>
+          <t>RS-1, GL-4, LC-7</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>Staff sentiment / attrition in affected roles</t>
+          <t>Override / challenge rate</t>
         </is>
       </c>
     </row>
     <row r="43" ht="36" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>TPR-01</t>
+          <t>HUM-02</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Third-Party &amp; Supply Chain</t>
+          <t>Human Oversight &amp; Autonomy</t>
         </is>
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>Vendor lock-in and concentration</t>
+          <t>Ineffective human oversight</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Critical dependence on a single AI provider or cloud creates resilience and bargaining risk.</t>
+          <t>Oversight persons lack competence, authority, time or information to intervene.</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>ISO/IEC 42001 A.10; CBB outsourcing</t>
+          <t>EU AI Act Art. 14, 26(2)</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>TP-2, TP-3</t>
+          <t>RS-1, GL-4</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>% critical AI workloads on single provider</t>
+          <t>Oversight roles without training</t>
         </is>
       </c>
     </row>
     <row r="44" ht="36" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>TPR-02</t>
+          <t>HUM-03</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Third-Party &amp; Supply Chain</t>
+          <t>Human Oversight &amp; Autonomy</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Inadequate vendor transparency and assurance</t>
+          <t>Unbounded autonomous agent actions</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Vendor cannot provide documentation, testing evidence or incident information needed for compliance.</t>
+          <t>AI agents take high-impact actions (payments, communications, code execution) without adequate limits or approval.</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>EU AI Act Art. 25(4); ISO/IEC 42001 A.10.3</t>
+          <t>OWASP Agentic Top 10; Singapore Agentic AI framework</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>TP-1, TP-3, LC-6</t>
+          <t>LC-8</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>Vendors without current assurance evidence</t>
+          <t>High-impact agent actions without approval</t>
         </is>
       </c>
     </row>
     <row r="45" ht="36" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>TPR-03</t>
+          <t>HUM-04</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Third-Party &amp; Supply Chain</t>
+          <t>Human Oversight &amp; Autonomy</t>
         </is>
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>Vendor use of organisation data</t>
+          <t>Adverse workforce impact</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Provider uses prompts, outputs or client data to train models or retains data beyond agreed terms.</t>
+          <t>AI adoption causes skills erosion, job anxiety or unconsulted changes to working conditions.</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Contract / DPA; Bahrain PDPL</t>
+          <t>EU AI Act Art. 26(7); AI Ready7 3.4</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>TP-3, PR-6</t>
+          <t>RS-9, GL-4</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>Contracts lacking no-training clause</t>
+          <t>Staff sentiment / attrition in affected roles</t>
         </is>
       </c>
     </row>
     <row r="46" ht="36" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>OPS-01</t>
+          <t>TPR-01</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Operational, Financial &amp; Sustainability</t>
+          <t>Third-Party &amp; Supply Chain</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>AI service outage or degradation</t>
+          <t>Vendor lock-in and concentration</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Business processes dependent on AI are disrupted by service unavailability or latency.</t>
+          <t>Critical dependence on a single AI provider or cloud creates resilience and bargaining risk.</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>ISO/IEC 27001 A.5.30; CBB OM</t>
+          <t>ISO/IEC 42001 A.10; CBB outsourcing</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>OM-1, SE-1</t>
+          <t>TP-2, TP-3</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>AI service availability vs SLA</t>
+          <t>% critical AI workloads on single provider</t>
         </is>
       </c>
     </row>
     <row r="47" ht="36" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>OPS-02</t>
+          <t>TPR-02</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Operational, Financial &amp; Sustainability</t>
+          <t>Third-Party &amp; Supply Chain</t>
         </is>
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>Uncontrolled AI cost and consumption</t>
+          <t>Inadequate vendor transparency and assurance</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Compute and API spend escalate without governance (incl. denial-of-wallet attacks).</t>
+          <t>Vendor cannot provide documentation, testing evidence or incident information needed for compliance.</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>AI Ready7 4.5; OWASP LLM10:2025</t>
+          <t>EU AI Act Art. 25(4); ISO/IEC 42001 A.10.3</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>GL-6, SE-6</t>
+          <t>TP-1, TP-3, LC-6</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>AI spend vs budget</t>
+          <t>Vendors without current assurance evidence</t>
         </is>
       </c>
     </row>
     <row r="48" ht="36" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>OPS-03</t>
+          <t>TPR-03</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Operational, Financial &amp; Sustainability</t>
+          <t>Third-Party &amp; Supply Chain</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Environmental impact of AI</t>
+          <t>Vendor use of organisation data</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Energy, water and carbon footprint of AI workloads conflicts with sustainability commitments.</t>
+          <t>Provider uses prompts, outputs or client data to train models or retains data beyond agreed terms.</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>ISO/IEC TR 20226; ISO/IEC 42001</t>
+          <t>Contract / DPA; Bahrain PDPL</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>RS-8</t>
+          <t>TP-3, PR-6</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>kgCO2e per 1,000 inferences</t>
+          <t>Contracts lacking no-training clause</t>
         </is>
       </c>
     </row>
     <row r="49" ht="36" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>SOC-01</t>
+          <t>OPS-01</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Societal, Reputational &amp; AI-Enabled Threats</t>
+          <t>Operational, Financial &amp; Sustainability</t>
         </is>
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>Harmful, toxic or unsafe content</t>
+          <t>AI service outage or degradation</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>AI generates offensive, dangerous or culturally inappropriate content.</t>
+          <t>Business processes dependent on AI are disrupted by service unavailability or latency.</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>NIST AI 600-1; GCC AI Ethics Manual</t>
+          <t>ISO/IEC 27001 A.5.30; CBB OM</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>RS-2, SE-6</t>
+          <t>OM-1, SE-1</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>Content-policy violations per 1,000 outputs</t>
+          <t>AI service availability vs SLA</t>
         </is>
       </c>
     </row>
     <row r="50" ht="36" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>SOC-02</t>
+          <t>OPS-02</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Societal, Reputational &amp; AI-Enabled Threats</t>
+          <t>Operational, Financial &amp; Sustainability</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Misinformation and loss of stakeholder trust</t>
+          <t>Uncontrolled AI cost and consumption</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>AI-generated errors or undisclosed AI use damage client, regulator or public trust.</t>
+          <t>Compute and API spend escalate without governance (incl. denial-of-wallet attacks).</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>NIST AI 600-1 (Information integrity); AI Ready7 1.4</t>
+          <t>AI Ready7 4.5; OWASP LLM10:2025</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>LC-7, CO-1, CO-2</t>
+          <t>GL-6, SE-6</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>Client complaints linked to AI</t>
+          <t>AI spend vs budget</t>
         </is>
       </c>
     </row>
     <row r="51" ht="36" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>SOC-03</t>
+          <t>OPS-04</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Societal, Reputational &amp; AI-Enabled Threats</t>
+          <t>Operational, Financial &amp; Sustainability</t>
         </is>
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>Deepfake and AI-enabled fraud against the organisation</t>
+          <t>No safe degradation or kill switch</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Voice/video impersonation or AI-crafted phishing leads to fraudulent payments or data release.</t>
+          <t>A failing or compromised AI system cannot be stopped quickly or the business process cannot revert to manual operation.</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>FinCEN FIN-2024-Alert004; AI Ready7 7.3</t>
+          <t>ISACA Securing AI Agents (2026); ISO 22301</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>AT-3, GL-4</t>
+          <t>OM-4</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>Deepfake / BEC attempts detected</t>
+          <t>Kill-switch test age (days)</t>
         </is>
       </c>
     </row>
     <row r="52" ht="36" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
         <is>
+          <t>OPS-03</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Operational, Financial &amp; Sustainability</t>
+        </is>
+      </c>
+      <c r="C52" s="11" t="inlineStr">
+        <is>
+          <t>Environmental impact of AI</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>Energy, water and carbon footprint of AI workloads conflicts with sustainability commitments.</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>ISO/IEC TR 20226; ISO/IEC 42001</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>RS-8</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>kgCO2e per 1,000 inferences</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="36" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>SOC-01</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Societal, Reputational &amp; AI-Enabled Threats</t>
+        </is>
+      </c>
+      <c r="C53" s="11" t="inlineStr">
+        <is>
+          <t>Harmful, toxic or unsafe content</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>AI generates offensive, dangerous or culturally inappropriate content.</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>NIST AI 600-1; GCC AI Ethics Manual</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>RS-2, SE-6</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>Content-policy violations per 1,000 outputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="36" customHeight="1">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>SOC-02</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Societal, Reputational &amp; AI-Enabled Threats</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="inlineStr">
+        <is>
+          <t>Misinformation and loss of stakeholder trust</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>AI-generated errors or undisclosed AI use damage client, regulator or public trust.</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>NIST AI 600-1 (Information integrity); AI Ready7 1.4</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>LC-7, CO-1, CO-2</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>Client complaints linked to AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="36" customHeight="1">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>SOC-03</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Societal, Reputational &amp; AI-Enabled Threats</t>
+        </is>
+      </c>
+      <c r="C55" s="11" t="inlineStr">
+        <is>
+          <t>Deepfake and AI-enabled fraud against the organisation</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>Voice/video impersonation or AI-crafted phishing leads to fraudulent payments or data release.</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>FinCEN FIN-2024-Alert004; AI Ready7 7.3</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>AT-3, GL-4</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>Deepfake / BEC attempts detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="36" customHeight="1">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
           <t>SOC-04</t>
         </is>
       </c>
-      <c r="B52" s="4" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>Societal, Reputational &amp; AI-Enabled Threats</t>
         </is>
       </c>
-      <c r="C52" s="11" t="inlineStr">
+      <c r="C56" s="11" t="inlineStr">
         <is>
           <t>AI-accelerated cyber attacks</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr">
+      <c r="D56" s="4" t="inlineStr">
         <is>
           <t>Adversaries use AI for automated discovery, exploit chaining and scaled social engineering, outpacing defences.</t>
         </is>
       </c>
-      <c r="E52" s="4" t="inlineStr">
+      <c r="E56" s="4" t="inlineStr">
         <is>
           <t>AI Ready7 7.1-7.5; MITRE ATLAS</t>
         </is>
       </c>
-      <c r="F52" s="4" t="inlineStr">
+      <c r="F56" s="4" t="inlineStr">
         <is>
           <t>AT-1, AT-2, AT-4</t>
         </is>
       </c>
-      <c r="G52" s="4" t="inlineStr">
+      <c r="G56" s="4" t="inlineStr">
         <is>
           <t>Mean time to remediate critical vulnerabilities</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G52"/>
+  <autoFilter ref="A4:G56"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <printOptions gridLines="0"/>
+  <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.25" footer="0.25"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -9828,8 +10250,9 @@
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="C35:E35"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <printOptions gridLines="0"/>
+  <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.25" footer="0.25"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Restore radar chart; store calculated values in all workbooks (cache_values.py)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X8ossW6xvKTGEs2GV44CxS
</commit_message>
<xml_diff>
--- a/01_AI_Governance_Risk_Compliance/1.2_AI_Risk_Assessment_Framework/GT_AI_Risk_Assessment_Toolkit_Template.xlsx
+++ b/01_AI_Governance_Risk_Compliance/1.2_AI_Risk_Assessment_Framework/GT_AI_Risk_Assessment_Toolkit_Template.xlsx
@@ -1457,9 +1457,9 @@
           <t>Screening result</t>
         </is>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="9" t="str">
         <f>IF(COUNTA(C5:C12)&lt;8,"Incomplete",IF(COUNTIF(C5:C12,"Yes")&gt;0,"PROHIBITED","Pass"))</f>
-        <v/>
+        <v>Incomplete</v>
       </c>
       <c r="D14" s="10" t="n"/>
     </row>
@@ -1565,14 +1565,14 @@
         </is>
       </c>
       <c r="C5" s="5" t="n"/>
-      <c r="D5" s="7">
+      <c r="D5" s="7" t="str">
         <f>IF(C5="","",MATCH(C5,Lists!$L$1:$L$5,0)-1)</f>
         <v/>
       </c>
       <c r="E5" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="7" t="str">
         <f>IF(D5="","",D5*E5)</f>
         <v/>
       </c>
@@ -1589,14 +1589,14 @@
         </is>
       </c>
       <c r="C6" s="5" t="n"/>
-      <c r="D6" s="7">
+      <c r="D6" s="7" t="str">
         <f>IF(C6="","",MATCH(C6,Lists!$M$1:$M$5,0)-1)</f>
         <v/>
       </c>
       <c r="E6" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="7" t="str">
         <f>IF(D6="","",D6*E6)</f>
         <v/>
       </c>
@@ -1613,14 +1613,14 @@
         </is>
       </c>
       <c r="C7" s="5" t="n"/>
-      <c r="D7" s="7">
+      <c r="D7" s="7" t="str">
         <f>IF(C7="","",MATCH(C7,Lists!$N$1:$N$5,0)-1)</f>
         <v/>
       </c>
       <c r="E7" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="7" t="str">
         <f>IF(D7="","",D7*E7)</f>
         <v/>
       </c>
@@ -1637,14 +1637,14 @@
         </is>
       </c>
       <c r="C8" s="5" t="n"/>
-      <c r="D8" s="7">
+      <c r="D8" s="7" t="str">
         <f>IF(C8="","",MATCH(C8,Lists!$O$1:$O$5,0)-1)</f>
         <v/>
       </c>
       <c r="E8" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="7" t="str">
         <f>IF(D8="","",D8*E8)</f>
         <v/>
       </c>
@@ -1661,14 +1661,14 @@
         </is>
       </c>
       <c r="C9" s="5" t="n"/>
-      <c r="D9" s="7">
+      <c r="D9" s="7" t="str">
         <f>IF(C9="","",MATCH(C9,Lists!$P$1:$P$5,0)-1)</f>
         <v/>
       </c>
       <c r="E9" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="7" t="str">
         <f>IF(D9="","",D9*E9)</f>
         <v/>
       </c>
@@ -1685,14 +1685,14 @@
         </is>
       </c>
       <c r="C10" s="5" t="n"/>
-      <c r="D10" s="7">
+      <c r="D10" s="7" t="str">
         <f>IF(C10="","",MATCH(C10,Lists!$Q$1:$Q$5,0)-1)</f>
         <v/>
       </c>
       <c r="E10" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="7" t="str">
         <f>IF(D10="","",D10*E10)</f>
         <v/>
       </c>
@@ -1709,14 +1709,14 @@
         </is>
       </c>
       <c r="C11" s="5" t="n"/>
-      <c r="D11" s="7">
+      <c r="D11" s="7" t="str">
         <f>IF(C11="","",MATCH(C11,Lists!$R$1:$R$5,0)-1)</f>
         <v/>
       </c>
       <c r="E11" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F11" s="7">
+      <c r="F11" s="7" t="str">
         <f>IF(D11="","",D11*E11)</f>
         <v/>
       </c>
@@ -1733,14 +1733,14 @@
         </is>
       </c>
       <c r="C12" s="5" t="n"/>
-      <c r="D12" s="7">
+      <c r="D12" s="7" t="str">
         <f>IF(C12="","",MATCH(C12,Lists!$S$1:$S$5,0)-1)</f>
         <v/>
       </c>
       <c r="E12" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="7">
+      <c r="F12" s="7" t="str">
         <f>IF(D12="","",D12*E12)</f>
         <v/>
       </c>
@@ -1757,14 +1757,14 @@
         </is>
       </c>
       <c r="C13" s="5" t="n"/>
-      <c r="D13" s="7">
+      <c r="D13" s="7" t="str">
         <f>IF(C13="","",MATCH(C13,Lists!$T$1:$T$5,0)-1)</f>
         <v/>
       </c>
       <c r="E13" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="7">
+      <c r="F13" s="7" t="str">
         <f>IF(D13="","",D13*E13)</f>
         <v/>
       </c>
@@ -1781,14 +1781,14 @@
         </is>
       </c>
       <c r="C14" s="5" t="n"/>
-      <c r="D14" s="7">
+      <c r="D14" s="7" t="str">
         <f>IF(C14="","",MATCH(C14,Lists!$U$1:$U$5,0)-1)</f>
         <v/>
       </c>
       <c r="E14" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="7">
+      <c r="F14" s="7" t="str">
         <f>IF(D14="","",D14*E14)</f>
         <v/>
       </c>
@@ -1799,9 +1799,9 @@
           <t>Factors answered</t>
         </is>
       </c>
-      <c r="C16" s="12">
+      <c r="C16" s="12" t="str">
         <f>COUNT(D5:D14)&amp;" of 10"</f>
-        <v/>
+        <v>0 of 10</v>
       </c>
       <c r="D16" s="13" t="n"/>
       <c r="E16" s="13" t="n"/>
@@ -1813,7 +1813,7 @@
           <t>Weighted score (0-100)</t>
         </is>
       </c>
-      <c r="C17" s="12">
+      <c r="C17" s="12" t="str">
         <f>IF(COUNT(D5:D14)&lt;10,"",ROUND(SUM(F5:F14)/(4*SUM(E5:E14))*100,0))</f>
         <v/>
       </c>
@@ -1827,7 +1827,7 @@
           <t>Score-based tier</t>
         </is>
       </c>
-      <c r="C18" s="12">
+      <c r="C18" s="12" t="str">
         <f>IF(C17="","",IF(C17&gt;=75,"Critical",IF(C17&gt;=50,"High",IF(C17&gt;=25,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -1841,7 +1841,7 @@
           <t>Override triggered</t>
         </is>
       </c>
-      <c r="C19" s="12">
+      <c r="C19" s="12" t="str">
         <f>IF(C17="","",IF(AND(D5=4,D6=4),"Critical - significant decisions made autonomously",IF(OR(D5=4,D11=4),"Min. High - significant-effect decisions or high-risk classification",IF(AND(D5&gt;=3,D6&gt;=3),"Min. High - material decisions with limited oversight",IF(D7=4,"Min. Medium - sensitive data","None")))))</f>
         <v/>
       </c>
@@ -1855,9 +1855,9 @@
           <t>Prohibited-practice screen</t>
         </is>
       </c>
-      <c r="C20" s="12">
+      <c r="C20" s="12" t="str">
         <f>'2. Prohibited Screen'!C14</f>
-        <v/>
+        <v>Incomplete</v>
       </c>
       <c r="D20" s="13" t="n"/>
       <c r="E20" s="13" t="n"/>
@@ -1869,9 +1869,9 @@
           <t>FINAL INHERENT RISK TIER</t>
         </is>
       </c>
-      <c r="C21" s="14">
+      <c r="C21" s="14" t="str">
         <f>IF(C20="PROHIBITED","Prohibited",IF(C17="","Incomplete",IF(LEFT(C19,8)="Critical","Critical",IF(AND(LEFT(C19,9)="Min. High",C18&lt;&gt;"Critical"),"High",IF(AND(LEFT(C19,11)="Min. Medium",C18="Low"),"Medium",C18)))))</f>
-        <v/>
+        <v>Incomplete</v>
       </c>
       <c r="D21" s="13" t="n"/>
       <c r="E21" s="13" t="n"/>
@@ -1883,7 +1883,7 @@
           <t>Assessment requirements</t>
         </is>
       </c>
-      <c r="C22" s="12">
+      <c r="C22" s="12" t="str">
         <f>IFERROR(VLOOKUP(C21,Scales!$A$36:$H$39,3,FALSE),IF(C21="Prohibited","Do not proceed. Refer to Legal and AI Committee.",""))</f>
         <v/>
       </c>
@@ -1897,7 +1897,7 @@
           <t>Approval authority</t>
         </is>
       </c>
-      <c r="C23" s="12">
+      <c r="C23" s="12" t="str">
         <f>IFERROR(VLOOKUP(C21,Scales!$A$36:$H$39,6,FALSE),IF(C21="Prohibited","Legal + Executive Committee",""))</f>
         <v/>
       </c>
@@ -1911,7 +1911,7 @@
           <t>Review frequency</t>
         </is>
       </c>
-      <c r="C24" s="12">
+      <c r="C24" s="12" t="str">
         <f>IFERROR(VLOOKUP(C21,Scales!$A$36:$H$39,8,FALSE),"")</f>
         <v/>
       </c>
@@ -2178,11 +2178,11 @@
       </c>
       <c r="F5" s="15" t="n"/>
       <c r="G5" s="15" t="n"/>
-      <c r="H5" s="7">
+      <c r="H5" s="7" t="str">
         <f>IF(OR($A5&lt;&gt;"Yes",F5="",G5=""),"",MATCH(F5,Lists!$B$1:$B$5,0)*MATCH(G5,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="7" t="str">
         <f>IF(H5="","",IF(H5&gt;=17,"Critical",IF(H5&gt;=10,"High",IF(H5&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -2192,15 +2192,15 @@
         </is>
       </c>
       <c r="K5" s="15" t="n"/>
-      <c r="L5" s="7">
+      <c r="L5" s="7" t="str">
         <f>IF(OR(H5="",K5=""),"",ROUND(H5*VLOOKUP(K5,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M5" s="7">
+      <c r="M5" s="7" t="str">
         <f>IF(L5="","",IF(L5&gt;=17,"Critical",IF(L5&gt;=10,"High",IF(L5&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N5" s="7">
+      <c r="N5" s="7" t="str">
         <f>IF(M5="","",IF(OR(M5="Low",M5="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -2214,7 +2214,7 @@
           <t>% AI systems in register without named owner</t>
         </is>
       </c>
-      <c r="V5">
+      <c r="V5" t="str">
         <f>IF(L5="","",L5+ROW()/100000)</f>
         <v/>
       </c>
@@ -2243,11 +2243,11 @@
       </c>
       <c r="F6" s="15" t="n"/>
       <c r="G6" s="15" t="n"/>
-      <c r="H6" s="7">
+      <c r="H6" s="7" t="str">
         <f>IF(OR($A6&lt;&gt;"Yes",F6="",G6=""),"",MATCH(F6,Lists!$B$1:$B$5,0)*MATCH(G6,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="7" t="str">
         <f>IF(H6="","",IF(H6&gt;=17,"Critical",IF(H6&gt;=10,"High",IF(H6&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -2257,15 +2257,15 @@
         </is>
       </c>
       <c r="K6" s="15" t="n"/>
-      <c r="L6" s="7">
+      <c r="L6" s="7" t="str">
         <f>IF(OR(H6="",K6=""),"",ROUND(H6*VLOOKUP(K6,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M6" s="7">
+      <c r="M6" s="7" t="str">
         <f>IF(L6="","",IF(L6&gt;=17,"Critical",IF(L6&gt;=10,"High",IF(L6&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N6" s="7">
+      <c r="N6" s="7" t="str">
         <f>IF(M6="","",IF(OR(M6="Low",M6="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -2279,7 +2279,7 @@
           <t>Unsanctioned AI services detected per month</t>
         </is>
       </c>
-      <c r="V6">
+      <c r="V6" t="str">
         <f>IF(L6="","",L6+ROW()/100000)</f>
         <v/>
       </c>
@@ -2308,11 +2308,11 @@
       </c>
       <c r="F7" s="15" t="n"/>
       <c r="G7" s="15" t="n"/>
-      <c r="H7" s="7">
+      <c r="H7" s="7" t="str">
         <f>IF(OR($A7&lt;&gt;"Yes",F7="",G7=""),"",MATCH(F7,Lists!$B$1:$B$5,0)*MATCH(G7,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I7" s="7">
+      <c r="I7" s="7" t="str">
         <f>IF(H7="","",IF(H7&gt;=17,"Critical",IF(H7&gt;=10,"High",IF(H7&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -2322,15 +2322,15 @@
         </is>
       </c>
       <c r="K7" s="15" t="n"/>
-      <c r="L7" s="7">
+      <c r="L7" s="7" t="str">
         <f>IF(OR(H7="",K7=""),"",ROUND(H7*VLOOKUP(K7,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M7" s="7">
+      <c r="M7" s="7" t="str">
         <f>IF(L7="","",IF(L7&gt;=17,"Critical",IF(L7&gt;=10,"High",IF(L7&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N7" s="7">
+      <c r="N7" s="7" t="str">
         <f>IF(M7="","",IF(OR(M7="Low",M7="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -2344,7 +2344,7 @@
           <t>% production AI systems with current assessment</t>
         </is>
       </c>
-      <c r="V7">
+      <c r="V7" t="str">
         <f>IF(L7="","",L7+ROW()/100000)</f>
         <v/>
       </c>
@@ -2373,11 +2373,11 @@
       </c>
       <c r="F8" s="15" t="n"/>
       <c r="G8" s="15" t="n"/>
-      <c r="H8" s="7">
+      <c r="H8" s="7" t="str">
         <f>IF(OR($A8&lt;&gt;"Yes",F8="",G8=""),"",MATCH(F8,Lists!$B$1:$B$5,0)*MATCH(G8,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="7" t="str">
         <f>IF(H8="","",IF(H8&gt;=17,"Critical",IF(H8&gt;=10,"High",IF(H8&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -2387,15 +2387,15 @@
         </is>
       </c>
       <c r="K8" s="15" t="n"/>
-      <c r="L8" s="7">
+      <c r="L8" s="7" t="str">
         <f>IF(OR(H8="",K8=""),"",ROUND(H8*VLOOKUP(K8,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M8" s="7">
+      <c r="M8" s="7" t="str">
         <f>IF(L8="","",IF(L8&gt;=17,"Critical",IF(L8&gt;=10,"High",IF(L8&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N8" s="7">
+      <c r="N8" s="7" t="str">
         <f>IF(M8="","",IF(OR(M8="Low",M8="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -2409,7 +2409,7 @@
           <t>% AI initiatives meeting benefit KPIs</t>
         </is>
       </c>
-      <c r="V8">
+      <c r="V8" t="str">
         <f>IF(L8="","",L8+ROW()/100000)</f>
         <v/>
       </c>
@@ -2438,11 +2438,11 @@
       </c>
       <c r="F9" s="15" t="n"/>
       <c r="G9" s="15" t="n"/>
-      <c r="H9" s="7">
+      <c r="H9" s="7" t="str">
         <f>IF(OR($A9&lt;&gt;"Yes",F9="",G9=""),"",MATCH(F9,Lists!$B$1:$B$5,0)*MATCH(G9,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="7" t="str">
         <f>IF(H9="","",IF(H9&gt;=17,"Critical",IF(H9&gt;=10,"High",IF(H9&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -2452,15 +2452,15 @@
         </is>
       </c>
       <c r="K9" s="15" t="n"/>
-      <c r="L9" s="7">
+      <c r="L9" s="7" t="str">
         <f>IF(OR(H9="",K9=""),"",ROUND(H9*VLOOKUP(K9,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M9" s="7">
+      <c r="M9" s="7" t="str">
         <f>IF(L9="","",IF(L9&gt;=17,"Critical",IF(L9&gt;=10,"High",IF(L9&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N9" s="7">
+      <c r="N9" s="7" t="str">
         <f>IF(M9="","",IF(OR(M9="Low",M9="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -2474,7 +2474,7 @@
           <t>Number of use cases failing prohibited-practice screen</t>
         </is>
       </c>
-      <c r="V9">
+      <c r="V9" t="str">
         <f>IF(L9="","",L9+ROW()/100000)</f>
         <v/>
       </c>
@@ -2503,11 +2503,11 @@
       </c>
       <c r="F10" s="15" t="n"/>
       <c r="G10" s="15" t="n"/>
-      <c r="H10" s="7">
+      <c r="H10" s="7" t="str">
         <f>IF(OR($A10&lt;&gt;"Yes",F10="",G10=""),"",MATCH(F10,Lists!$B$1:$B$5,0)*MATCH(G10,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="7" t="str">
         <f>IF(H10="","",IF(H10&gt;=17,"Critical",IF(H10&gt;=10,"High",IF(H10&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -2517,15 +2517,15 @@
         </is>
       </c>
       <c r="K10" s="15" t="n"/>
-      <c r="L10" s="7">
+      <c r="L10" s="7" t="str">
         <f>IF(OR(H10="",K10=""),"",ROUND(H10*VLOOKUP(K10,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M10" s="7">
+      <c r="M10" s="7" t="str">
         <f>IF(L10="","",IF(L10&gt;=17,"Critical",IF(L10&gt;=10,"High",IF(L10&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N10" s="7">
+      <c r="N10" s="7" t="str">
         <f>IF(M10="","",IF(OR(M10="Low",M10="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -2539,7 +2539,7 @@
           <t>Open compliance gaps on high-risk systems</t>
         </is>
       </c>
-      <c r="V10">
+      <c r="V10" t="str">
         <f>IF(L10="","",L10+ROW()/100000)</f>
         <v/>
       </c>
@@ -2568,11 +2568,11 @@
       </c>
       <c r="F11" s="15" t="n"/>
       <c r="G11" s="15" t="n"/>
-      <c r="H11" s="7">
+      <c r="H11" s="7" t="str">
         <f>IF(OR($A11&lt;&gt;"Yes",F11="",G11=""),"",MATCH(F11,Lists!$B$1:$B$5,0)*MATCH(G11,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="7" t="str">
         <f>IF(H11="","",IF(H11&gt;=17,"Critical",IF(H11&gt;=10,"High",IF(H11&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -2582,15 +2582,15 @@
         </is>
       </c>
       <c r="K11" s="15" t="n"/>
-      <c r="L11" s="7">
+      <c r="L11" s="7" t="str">
         <f>IF(OR(H11="",K11=""),"",ROUND(H11*VLOOKUP(K11,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M11" s="7">
+      <c r="M11" s="7" t="str">
         <f>IF(L11="","",IF(L11&gt;=17,"Critical",IF(L11&gt;=10,"High",IF(L11&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N11" s="7">
+      <c r="N11" s="7" t="str">
         <f>IF(M11="","",IF(OR(M11="Low",M11="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -2604,7 +2604,7 @@
           <t>Regulatory findings related to AI</t>
         </is>
       </c>
-      <c r="V11">
+      <c r="V11" t="str">
         <f>IF(L11="","",L11+ROW()/100000)</f>
         <v/>
       </c>
@@ -2633,11 +2633,11 @@
       </c>
       <c r="F12" s="15" t="n"/>
       <c r="G12" s="15" t="n"/>
-      <c r="H12" s="7">
+      <c r="H12" s="7" t="str">
         <f>IF(OR($A12&lt;&gt;"Yes",F12="",G12=""),"",MATCH(F12,Lists!$B$1:$B$5,0)*MATCH(G12,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I12" s="7">
+      <c r="I12" s="7" t="str">
         <f>IF(H12="","",IF(H12&gt;=17,"Critical",IF(H12&gt;=10,"High",IF(H12&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -2647,15 +2647,15 @@
         </is>
       </c>
       <c r="K12" s="15" t="n"/>
-      <c r="L12" s="7">
+      <c r="L12" s="7" t="str">
         <f>IF(OR(H12="",K12=""),"",ROUND(H12*VLOOKUP(K12,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M12" s="7">
+      <c r="M12" s="7" t="str">
         <f>IF(L12="","",IF(L12&gt;=17,"Critical",IF(L12&gt;=10,"High",IF(L12&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N12" s="7">
+      <c r="N12" s="7" t="str">
         <f>IF(M12="","",IF(OR(M12="Low",M12="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -2669,7 +2669,7 @@
           <t>IP complaints / takedown requests</t>
         </is>
       </c>
-      <c r="V12">
+      <c r="V12" t="str">
         <f>IF(L12="","",L12+ROW()/100000)</f>
         <v/>
       </c>
@@ -2698,11 +2698,11 @@
       </c>
       <c r="F13" s="15" t="n"/>
       <c r="G13" s="15" t="n"/>
-      <c r="H13" s="7">
+      <c r="H13" s="7" t="str">
         <f>IF(OR($A13&lt;&gt;"Yes",F13="",G13=""),"",MATCH(F13,Lists!$B$1:$B$5,0)*MATCH(G13,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I13" s="7">
+      <c r="I13" s="7" t="str">
         <f>IF(H13="","",IF(H13&gt;=17,"Critical",IF(H13&gt;=10,"High",IF(H13&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -2712,15 +2712,15 @@
         </is>
       </c>
       <c r="K13" s="15" t="n"/>
-      <c r="L13" s="7">
+      <c r="L13" s="7" t="str">
         <f>IF(OR(H13="",K13=""),"",ROUND(H13*VLOOKUP(K13,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M13" s="7">
+      <c r="M13" s="7" t="str">
         <f>IF(L13="","",IF(L13&gt;=17,"Critical",IF(L13&gt;=10,"High",IF(L13&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N13" s="7">
+      <c r="N13" s="7" t="str">
         <f>IF(M13="","",IF(OR(M13="Low",M13="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -2734,7 +2734,7 @@
           <t>Claims / complaints attributed to AI</t>
         </is>
       </c>
-      <c r="V13">
+      <c r="V13" t="str">
         <f>IF(L13="","",L13+ROW()/100000)</f>
         <v/>
       </c>
@@ -2763,11 +2763,11 @@
       </c>
       <c r="F14" s="15" t="n"/>
       <c r="G14" s="15" t="n"/>
-      <c r="H14" s="7">
+      <c r="H14" s="7" t="str">
         <f>IF(OR($A14&lt;&gt;"Yes",F14="",G14=""),"",MATCH(F14,Lists!$B$1:$B$5,0)*MATCH(G14,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I14" s="7">
+      <c r="I14" s="7" t="str">
         <f>IF(H14="","",IF(H14&gt;=17,"Critical",IF(H14&gt;=10,"High",IF(H14&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -2777,15 +2777,15 @@
         </is>
       </c>
       <c r="K14" s="15" t="n"/>
-      <c r="L14" s="7">
+      <c r="L14" s="7" t="str">
         <f>IF(OR(H14="",K14=""),"",ROUND(H14*VLOOKUP(K14,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M14" s="7">
+      <c r="M14" s="7" t="str">
         <f>IF(L14="","",IF(L14&gt;=17,"Critical",IF(L14&gt;=10,"High",IF(L14&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N14" s="7">
+      <c r="N14" s="7" t="str">
         <f>IF(M14="","",IF(OR(M14="Low",M14="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -2799,7 +2799,7 @@
           <t>Disparate impact ratio across cohorts</t>
         </is>
       </c>
-      <c r="V14">
+      <c r="V14" t="str">
         <f>IF(L14="","",L14+ROW()/100000)</f>
         <v/>
       </c>
@@ -2828,11 +2828,11 @@
       </c>
       <c r="F15" s="15" t="n"/>
       <c r="G15" s="15" t="n"/>
-      <c r="H15" s="7">
+      <c r="H15" s="7" t="str">
         <f>IF(OR($A15&lt;&gt;"Yes",F15="",G15=""),"",MATCH(F15,Lists!$B$1:$B$5,0)*MATCH(G15,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I15" s="7">
+      <c r="I15" s="7" t="str">
         <f>IF(H15="","",IF(H15&gt;=17,"Critical",IF(H15&gt;=10,"High",IF(H15&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -2842,15 +2842,15 @@
         </is>
       </c>
       <c r="K15" s="15" t="n"/>
-      <c r="L15" s="7">
+      <c r="L15" s="7" t="str">
         <f>IF(OR(H15="",K15=""),"",ROUND(H15*VLOOKUP(K15,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M15" s="7">
+      <c r="M15" s="7" t="str">
         <f>IF(L15="","",IF(L15&gt;=17,"Critical",IF(L15&gt;=10,"High",IF(L15&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N15" s="7">
+      <c r="N15" s="7" t="str">
         <f>IF(M15="","",IF(OR(M15="Low",M15="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -2864,7 +2864,7 @@
           <t>Coverage gaps by segment in evaluation set</t>
         </is>
       </c>
-      <c r="V15">
+      <c r="V15" t="str">
         <f>IF(L15="","",L15+ROW()/100000)</f>
         <v/>
       </c>
@@ -2893,11 +2893,11 @@
       </c>
       <c r="F16" s="15" t="n"/>
       <c r="G16" s="15" t="n"/>
-      <c r="H16" s="7">
+      <c r="H16" s="7" t="str">
         <f>IF(OR($A16&lt;&gt;"Yes",F16="",G16=""),"",MATCH(F16,Lists!$B$1:$B$5,0)*MATCH(G16,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I16" s="7">
+      <c r="I16" s="7" t="str">
         <f>IF(H16="","",IF(H16&gt;=17,"Critical",IF(H16&gt;=10,"High",IF(H16&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -2907,15 +2907,15 @@
         </is>
       </c>
       <c r="K16" s="15" t="n"/>
-      <c r="L16" s="7">
+      <c r="L16" s="7" t="str">
         <f>IF(OR(H16="",K16=""),"",ROUND(H16*VLOOKUP(K16,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M16" s="7">
+      <c r="M16" s="7" t="str">
         <f>IF(L16="","",IF(L16&gt;=17,"Critical",IF(L16&gt;=10,"High",IF(L16&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N16" s="7">
+      <c r="N16" s="7" t="str">
         <f>IF(M16="","",IF(OR(M16="Low",M16="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -2929,7 +2929,7 @@
           <t>FRIAs outstanding for in-scope systems</t>
         </is>
       </c>
-      <c r="V16">
+      <c r="V16" t="str">
         <f>IF(L16="","",L16+ROW()/100000)</f>
         <v/>
       </c>
@@ -2958,11 +2958,11 @@
       </c>
       <c r="F17" s="15" t="n"/>
       <c r="G17" s="15" t="n"/>
-      <c r="H17" s="7">
+      <c r="H17" s="7" t="str">
         <f>IF(OR($A17&lt;&gt;"Yes",F17="",G17=""),"",MATCH(F17,Lists!$B$1:$B$5,0)*MATCH(G17,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I17" s="7">
+      <c r="I17" s="7" t="str">
         <f>IF(H17="","",IF(H17&gt;=17,"Critical",IF(H17&gt;=10,"High",IF(H17&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -2972,15 +2972,15 @@
         </is>
       </c>
       <c r="K17" s="15" t="n"/>
-      <c r="L17" s="7">
+      <c r="L17" s="7" t="str">
         <f>IF(OR(H17="",K17=""),"",ROUND(H17*VLOOKUP(K17,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M17" s="7">
+      <c r="M17" s="7" t="str">
         <f>IF(L17="","",IF(L17&gt;=17,"Critical",IF(L17&gt;=10,"High",IF(L17&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N17" s="7">
+      <c r="N17" s="7" t="str">
         <f>IF(M17="","",IF(OR(M17="Low",M17="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -2994,7 +2994,7 @@
           <t>Accessibility defects open</t>
         </is>
       </c>
-      <c r="V17">
+      <c r="V17" t="str">
         <f>IF(L17="","",L17+ROW()/100000)</f>
         <v/>
       </c>
@@ -3023,11 +3023,11 @@
       </c>
       <c r="F18" s="15" t="n"/>
       <c r="G18" s="15" t="n"/>
-      <c r="H18" s="7">
+      <c r="H18" s="7" t="str">
         <f>IF(OR($A18&lt;&gt;"Yes",F18="",G18=""),"",MATCH(F18,Lists!$B$1:$B$5,0)*MATCH(G18,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I18" s="7">
+      <c r="I18" s="7" t="str">
         <f>IF(H18="","",IF(H18&gt;=17,"Critical",IF(H18&gt;=10,"High",IF(H18&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -3037,15 +3037,15 @@
         </is>
       </c>
       <c r="K18" s="15" t="n"/>
-      <c r="L18" s="7">
+      <c r="L18" s="7" t="str">
         <f>IF(OR(H18="",K18=""),"",ROUND(H18*VLOOKUP(K18,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M18" s="7">
+      <c r="M18" s="7" t="str">
         <f>IF(L18="","",IF(L18&gt;=17,"Critical",IF(L18&gt;=10,"High",IF(L18&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N18" s="7">
+      <c r="N18" s="7" t="str">
         <f>IF(M18="","",IF(OR(M18="Low",M18="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -3059,7 +3059,7 @@
           <t>AI systems processing personal data without DPIA</t>
         </is>
       </c>
-      <c r="V18">
+      <c r="V18" t="str">
         <f>IF(L18="","",L18+ROW()/100000)</f>
         <v/>
       </c>
@@ -3088,11 +3088,11 @@
       </c>
       <c r="F19" s="15" t="n"/>
       <c r="G19" s="15" t="n"/>
-      <c r="H19" s="7">
+      <c r="H19" s="7" t="str">
         <f>IF(OR($A19&lt;&gt;"Yes",F19="",G19=""),"",MATCH(F19,Lists!$B$1:$B$5,0)*MATCH(G19,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I19" s="7">
+      <c r="I19" s="7" t="str">
         <f>IF(H19="","",IF(H19&gt;=17,"Critical",IF(H19&gt;=10,"High",IF(H19&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -3102,15 +3102,15 @@
         </is>
       </c>
       <c r="K19" s="15" t="n"/>
-      <c r="L19" s="7">
+      <c r="L19" s="7" t="str">
         <f>IF(OR(H19="",K19=""),"",ROUND(H19*VLOOKUP(K19,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M19" s="7">
+      <c r="M19" s="7" t="str">
         <f>IF(L19="","",IF(L19&gt;=17,"Critical",IF(L19&gt;=10,"High",IF(L19&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N19" s="7">
+      <c r="N19" s="7" t="str">
         <f>IF(M19="","",IF(OR(M19="Low",M19="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -3124,7 +3124,7 @@
           <t>DLP events involving AI services</t>
         </is>
       </c>
-      <c r="V19">
+      <c r="V19" t="str">
         <f>IF(L19="","",L19+ROW()/100000)</f>
         <v/>
       </c>
@@ -3153,11 +3153,11 @@
       </c>
       <c r="F20" s="15" t="n"/>
       <c r="G20" s="15" t="n"/>
-      <c r="H20" s="7">
+      <c r="H20" s="7" t="str">
         <f>IF(OR($A20&lt;&gt;"Yes",F20="",G20=""),"",MATCH(F20,Lists!$B$1:$B$5,0)*MATCH(G20,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I20" s="7">
+      <c r="I20" s="7" t="str">
         <f>IF(H20="","",IF(H20&gt;=17,"Critical",IF(H20&gt;=10,"High",IF(H20&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -3167,15 +3167,15 @@
         </is>
       </c>
       <c r="K20" s="15" t="n"/>
-      <c r="L20" s="7">
+      <c r="L20" s="7" t="str">
         <f>IF(OR(H20="",K20=""),"",ROUND(H20*VLOOKUP(K20,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M20" s="7">
+      <c r="M20" s="7" t="str">
         <f>IF(L20="","",IF(L20&gt;=17,"Critical",IF(L20&gt;=10,"High",IF(L20&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N20" s="7">
+      <c r="N20" s="7" t="str">
         <f>IF(M20="","",IF(OR(M20="Low",M20="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -3189,7 +3189,7 @@
           <t>AI services hosted outside approved regions</t>
         </is>
       </c>
-      <c r="V20">
+      <c r="V20" t="str">
         <f>IF(L20="","",L20+ROW()/100000)</f>
         <v/>
       </c>
@@ -3218,11 +3218,11 @@
       </c>
       <c r="F21" s="15" t="n"/>
       <c r="G21" s="15" t="n"/>
-      <c r="H21" s="7">
+      <c r="H21" s="7" t="str">
         <f>IF(OR($A21&lt;&gt;"Yes",F21="",G21=""),"",MATCH(F21,Lists!$B$1:$B$5,0)*MATCH(G21,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I21" s="7">
+      <c r="I21" s="7" t="str">
         <f>IF(H21="","",IF(H21&gt;=17,"Critical",IF(H21&gt;=10,"High",IF(H21&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -3232,15 +3232,15 @@
         </is>
       </c>
       <c r="K21" s="15" t="n"/>
-      <c r="L21" s="7">
+      <c r="L21" s="7" t="str">
         <f>IF(OR(H21="",K21=""),"",ROUND(H21*VLOOKUP(K21,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M21" s="7">
+      <c r="M21" s="7" t="str">
         <f>IF(L21="","",IF(L21&gt;=17,"Critical",IF(L21&gt;=10,"High",IF(L21&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N21" s="7">
+      <c r="N21" s="7" t="str">
         <f>IF(M21="","",IF(OR(M21="Low",M21="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -3254,7 +3254,7 @@
           <t>DSRs involving AI exceeding SLA</t>
         </is>
       </c>
-      <c r="V21">
+      <c r="V21" t="str">
         <f>IF(L21="","",L21+ROW()/100000)</f>
         <v/>
       </c>
@@ -3283,11 +3283,11 @@
       </c>
       <c r="F22" s="15" t="n"/>
       <c r="G22" s="15" t="n"/>
-      <c r="H22" s="7">
+      <c r="H22" s="7" t="str">
         <f>IF(OR($A22&lt;&gt;"Yes",F22="",G22=""),"",MATCH(F22,Lists!$B$1:$B$5,0)*MATCH(G22,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I22" s="7">
+      <c r="I22" s="7" t="str">
         <f>IF(H22="","",IF(H22&gt;=17,"Critical",IF(H22&gt;=10,"High",IF(H22&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -3297,15 +3297,15 @@
         </is>
       </c>
       <c r="K22" s="15" t="n"/>
-      <c r="L22" s="7">
+      <c r="L22" s="7" t="str">
         <f>IF(OR(H22="",K22=""),"",ROUND(H22*VLOOKUP(K22,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M22" s="7">
+      <c r="M22" s="7" t="str">
         <f>IF(L22="","",IF(L22&gt;=17,"Critical",IF(L22&gt;=10,"High",IF(L22&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N22" s="7">
+      <c r="N22" s="7" t="str">
         <f>IF(M22="","",IF(OR(M22="Low",M22="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -3319,7 +3319,7 @@
           <t>Re-identification test failures</t>
         </is>
       </c>
-      <c r="V22">
+      <c r="V22" t="str">
         <f>IF(L22="","",L22+ROW()/100000)</f>
         <v/>
       </c>
@@ -3348,11 +3348,11 @@
       </c>
       <c r="F23" s="15" t="n"/>
       <c r="G23" s="15" t="n"/>
-      <c r="H23" s="7">
+      <c r="H23" s="7" t="str">
         <f>IF(OR($A23&lt;&gt;"Yes",F23="",G23=""),"",MATCH(F23,Lists!$B$1:$B$5,0)*MATCH(G23,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I23" s="7">
+      <c r="I23" s="7" t="str">
         <f>IF(H23="","",IF(H23&gt;=17,"Critical",IF(H23&gt;=10,"High",IF(H23&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -3362,15 +3362,15 @@
         </is>
       </c>
       <c r="K23" s="15" t="n"/>
-      <c r="L23" s="7">
+      <c r="L23" s="7" t="str">
         <f>IF(OR(H23="",K23=""),"",ROUND(H23*VLOOKUP(K23,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M23" s="7">
+      <c r="M23" s="7" t="str">
         <f>IF(L23="","",IF(L23&gt;=17,"Critical",IF(L23&gt;=10,"High",IF(L23&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N23" s="7">
+      <c r="N23" s="7" t="str">
         <f>IF(M23="","",IF(OR(M23="Low",M23="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -3384,7 +3384,7 @@
           <t>Data-quality rule failures</t>
         </is>
       </c>
-      <c r="V23">
+      <c r="V23" t="str">
         <f>IF(L23="","",L23+ROW()/100000)</f>
         <v/>
       </c>
@@ -3413,11 +3413,11 @@
       </c>
       <c r="F24" s="15" t="n"/>
       <c r="G24" s="15" t="n"/>
-      <c r="H24" s="7">
+      <c r="H24" s="7" t="str">
         <f>IF(OR($A24&lt;&gt;"Yes",F24="",G24=""),"",MATCH(F24,Lists!$B$1:$B$5,0)*MATCH(G24,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I24" s="7">
+      <c r="I24" s="7" t="str">
         <f>IF(H24="","",IF(H24&gt;=17,"Critical",IF(H24&gt;=10,"High",IF(H24&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -3427,15 +3427,15 @@
         </is>
       </c>
       <c r="K24" s="15" t="n"/>
-      <c r="L24" s="7">
+      <c r="L24" s="7" t="str">
         <f>IF(OR(H24="",K24=""),"",ROUND(H24*VLOOKUP(K24,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M24" s="7">
+      <c r="M24" s="7" t="str">
         <f>IF(L24="","",IF(L24&gt;=17,"Critical",IF(L24&gt;=10,"High",IF(L24&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N24" s="7">
+      <c r="N24" s="7" t="str">
         <f>IF(M24="","",IF(OR(M24="Low",M24="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -3449,7 +3449,7 @@
           <t>% datasets with documented lineage</t>
         </is>
       </c>
-      <c r="V24">
+      <c r="V24" t="str">
         <f>IF(L24="","",L24+ROW()/100000)</f>
         <v/>
       </c>
@@ -3478,11 +3478,11 @@
       </c>
       <c r="F25" s="15" t="n"/>
       <c r="G25" s="15" t="n"/>
-      <c r="H25" s="7">
+      <c r="H25" s="7" t="str">
         <f>IF(OR($A25&lt;&gt;"Yes",F25="",G25=""),"",MATCH(F25,Lists!$B$1:$B$5,0)*MATCH(G25,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I25" s="7">
+      <c r="I25" s="7" t="str">
         <f>IF(H25="","",IF(H25&gt;=17,"Critical",IF(H25&gt;=10,"High",IF(H25&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -3492,15 +3492,15 @@
         </is>
       </c>
       <c r="K25" s="15" t="n"/>
-      <c r="L25" s="7">
+      <c r="L25" s="7" t="str">
         <f>IF(OR(H25="",K25=""),"",ROUND(H25*VLOOKUP(K25,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M25" s="7">
+      <c r="M25" s="7" t="str">
         <f>IF(L25="","",IF(L25&gt;=17,"Critical",IF(L25&gt;=10,"High",IF(L25&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N25" s="7">
+      <c r="N25" s="7" t="str">
         <f>IF(M25="","",IF(OR(M25="Low",M25="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -3514,7 +3514,7 @@
           <t>Population stability index / drift score</t>
         </is>
       </c>
-      <c r="V25">
+      <c r="V25" t="str">
         <f>IF(L25="","",L25+ROW()/100000)</f>
         <v/>
       </c>
@@ -3543,11 +3543,11 @@
       </c>
       <c r="F26" s="15" t="n"/>
       <c r="G26" s="15" t="n"/>
-      <c r="H26" s="7">
+      <c r="H26" s="7" t="str">
         <f>IF(OR($A26&lt;&gt;"Yes",F26="",G26=""),"",MATCH(F26,Lists!$B$1:$B$5,0)*MATCH(G26,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I26" s="7">
+      <c r="I26" s="7" t="str">
         <f>IF(H26="","",IF(H26&gt;=17,"Critical",IF(H26&gt;=10,"High",IF(H26&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -3557,15 +3557,15 @@
         </is>
       </c>
       <c r="K26" s="15" t="n"/>
-      <c r="L26" s="7">
+      <c r="L26" s="7" t="str">
         <f>IF(OR(H26="",K26=""),"",ROUND(H26*VLOOKUP(K26,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M26" s="7">
+      <c r="M26" s="7" t="str">
         <f>IF(L26="","",IF(L26&gt;=17,"Critical",IF(L26&gt;=10,"High",IF(L26&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N26" s="7">
+      <c r="N26" s="7" t="str">
         <f>IF(M26="","",IF(OR(M26="Low",M26="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -3579,7 +3579,7 @@
           <t>Error rate vs threshold</t>
         </is>
       </c>
-      <c r="V26">
+      <c r="V26" t="str">
         <f>IF(L26="","",L26+ROW()/100000)</f>
         <v/>
       </c>
@@ -3608,11 +3608,11 @@
       </c>
       <c r="F27" s="15" t="n"/>
       <c r="G27" s="15" t="n"/>
-      <c r="H27" s="7">
+      <c r="H27" s="7" t="str">
         <f>IF(OR($A27&lt;&gt;"Yes",F27="",G27=""),"",MATCH(F27,Lists!$B$1:$B$5,0)*MATCH(G27,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I27" s="7">
+      <c r="I27" s="7" t="str">
         <f>IF(H27="","",IF(H27&gt;=17,"Critical",IF(H27&gt;=10,"High",IF(H27&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -3622,15 +3622,15 @@
         </is>
       </c>
       <c r="K27" s="15" t="n"/>
-      <c r="L27" s="7">
+      <c r="L27" s="7" t="str">
         <f>IF(OR(H27="",K27=""),"",ROUND(H27*VLOOKUP(K27,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M27" s="7">
+      <c r="M27" s="7" t="str">
         <f>IF(L27="","",IF(L27&gt;=17,"Critical",IF(L27&gt;=10,"High",IF(L27&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N27" s="7">
+      <c r="N27" s="7" t="str">
         <f>IF(M27="","",IF(OR(M27="Low",M27="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -3644,7 +3644,7 @@
           <t>Hallucination rate in evaluation / QA sampling</t>
         </is>
       </c>
-      <c r="V27">
+      <c r="V27" t="str">
         <f>IF(L27="","",L27+ROW()/100000)</f>
         <v/>
       </c>
@@ -3673,11 +3673,11 @@
       </c>
       <c r="F28" s="15" t="n"/>
       <c r="G28" s="15" t="n"/>
-      <c r="H28" s="7">
+      <c r="H28" s="7" t="str">
         <f>IF(OR($A28&lt;&gt;"Yes",F28="",G28=""),"",MATCH(F28,Lists!$B$1:$B$5,0)*MATCH(G28,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I28" s="7">
+      <c r="I28" s="7" t="str">
         <f>IF(H28="","",IF(H28&gt;=17,"Critical",IF(H28&gt;=10,"High",IF(H28&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -3687,15 +3687,15 @@
         </is>
       </c>
       <c r="K28" s="15" t="n"/>
-      <c r="L28" s="7">
+      <c r="L28" s="7" t="str">
         <f>IF(OR(H28="",K28=""),"",ROUND(H28*VLOOKUP(K28,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M28" s="7">
+      <c r="M28" s="7" t="str">
         <f>IF(L28="","",IF(L28&gt;=17,"Critical",IF(L28&gt;=10,"High",IF(L28&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N28" s="7">
+      <c r="N28" s="7" t="str">
         <f>IF(M28="","",IF(OR(M28="Low",M28="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -3709,7 +3709,7 @@
           <t>Robustness test pass rate</t>
         </is>
       </c>
-      <c r="V28">
+      <c r="V28" t="str">
         <f>IF(L28="","",L28+ROW()/100000)</f>
         <v/>
       </c>
@@ -3738,11 +3738,11 @@
       </c>
       <c r="F29" s="15" t="n"/>
       <c r="G29" s="15" t="n"/>
-      <c r="H29" s="7">
+      <c r="H29" s="7" t="str">
         <f>IF(OR($A29&lt;&gt;"Yes",F29="",G29=""),"",MATCH(F29,Lists!$B$1:$B$5,0)*MATCH(G29,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I29" s="7">
+      <c r="I29" s="7" t="str">
         <f>IF(H29="","",IF(H29&gt;=17,"Critical",IF(H29&gt;=10,"High",IF(H29&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -3752,15 +3752,15 @@
         </is>
       </c>
       <c r="K29" s="15" t="n"/>
-      <c r="L29" s="7">
+      <c r="L29" s="7" t="str">
         <f>IF(OR(H29="",K29=""),"",ROUND(H29*VLOOKUP(K29,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M29" s="7">
+      <c r="M29" s="7" t="str">
         <f>IF(L29="","",IF(L29&gt;=17,"Critical",IF(L29&gt;=10,"High",IF(L29&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N29" s="7">
+      <c r="N29" s="7" t="str">
         <f>IF(M29="","",IF(OR(M29="Low",M29="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -3774,7 +3774,7 @@
           <t>Unvalidated model version changes</t>
         </is>
       </c>
-      <c r="V29">
+      <c r="V29" t="str">
         <f>IF(L29="","",L29+ROW()/100000)</f>
         <v/>
       </c>
@@ -3803,11 +3803,11 @@
       </c>
       <c r="F30" s="15" t="n"/>
       <c r="G30" s="15" t="n"/>
-      <c r="H30" s="7">
+      <c r="H30" s="7" t="str">
         <f>IF(OR($A30&lt;&gt;"Yes",F30="",G30=""),"",MATCH(F30,Lists!$B$1:$B$5,0)*MATCH(G30,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I30" s="7">
+      <c r="I30" s="7" t="str">
         <f>IF(H30="","",IF(H30&gt;=17,"Critical",IF(H30&gt;=10,"High",IF(H30&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -3817,15 +3817,15 @@
         </is>
       </c>
       <c r="K30" s="15" t="n"/>
-      <c r="L30" s="7">
+      <c r="L30" s="7" t="str">
         <f>IF(OR(H30="",K30=""),"",ROUND(H30*VLOOKUP(K30,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M30" s="7">
+      <c r="M30" s="7" t="str">
         <f>IF(L30="","",IF(L30&gt;=17,"Critical",IF(L30&gt;=10,"High",IF(L30&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N30" s="7">
+      <c r="N30" s="7" t="str">
         <f>IF(M30="","",IF(OR(M30="Low",M30="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -3839,7 +3839,7 @@
           <t>Releases without passing LLM regression suite</t>
         </is>
       </c>
-      <c r="V30">
+      <c r="V30" t="str">
         <f>IF(L30="","",L30+ROW()/100000)</f>
         <v/>
       </c>
@@ -3868,11 +3868,11 @@
       </c>
       <c r="F31" s="15" t="n"/>
       <c r="G31" s="15" t="n"/>
-      <c r="H31" s="7">
+      <c r="H31" s="7" t="str">
         <f>IF(OR($A31&lt;&gt;"Yes",F31="",G31=""),"",MATCH(F31,Lists!$B$1:$B$5,0)*MATCH(G31,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I31" s="7">
+      <c r="I31" s="7" t="str">
         <f>IF(H31="","",IF(H31&gt;=17,"Critical",IF(H31&gt;=10,"High",IF(H31&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -3882,15 +3882,15 @@
         </is>
       </c>
       <c r="K31" s="15" t="n"/>
-      <c r="L31" s="7">
+      <c r="L31" s="7" t="str">
         <f>IF(OR(H31="",K31=""),"",ROUND(H31*VLOOKUP(K31,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M31" s="7">
+      <c r="M31" s="7" t="str">
         <f>IF(L31="","",IF(L31&gt;=17,"Critical",IF(L31&gt;=10,"High",IF(L31&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N31" s="7">
+      <c r="N31" s="7" t="str">
         <f>IF(M31="","",IF(OR(M31="Low",M31="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -3904,7 +3904,7 @@
           <t>AI touchpoints lacking disclosure</t>
         </is>
       </c>
-      <c r="V31">
+      <c r="V31" t="str">
         <f>IF(L31="","",L31+ROW()/100000)</f>
         <v/>
       </c>
@@ -3933,11 +3933,11 @@
       </c>
       <c r="F32" s="15" t="n"/>
       <c r="G32" s="15" t="n"/>
-      <c r="H32" s="7">
+      <c r="H32" s="7" t="str">
         <f>IF(OR($A32&lt;&gt;"Yes",F32="",G32=""),"",MATCH(F32,Lists!$B$1:$B$5,0)*MATCH(G32,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I32" s="7">
+      <c r="I32" s="7" t="str">
         <f>IF(H32="","",IF(H32&gt;=17,"Critical",IF(H32&gt;=10,"High",IF(H32&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -3947,15 +3947,15 @@
         </is>
       </c>
       <c r="K32" s="15" t="n"/>
-      <c r="L32" s="7">
+      <c r="L32" s="7" t="str">
         <f>IF(OR(H32="",K32=""),"",ROUND(H32*VLOOKUP(K32,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M32" s="7">
+      <c r="M32" s="7" t="str">
         <f>IF(L32="","",IF(L32&gt;=17,"Critical",IF(L32&gt;=10,"High",IF(L32&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N32" s="7">
+      <c r="N32" s="7" t="str">
         <f>IF(M32="","",IF(OR(M32="Low",M32="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -3969,7 +3969,7 @@
           <t>Explanation requests not satisfied</t>
         </is>
       </c>
-      <c r="V32">
+      <c r="V32" t="str">
         <f>IF(L32="","",L32+ROW()/100000)</f>
         <v/>
       </c>
@@ -3998,11 +3998,11 @@
       </c>
       <c r="F33" s="15" t="n"/>
       <c r="G33" s="15" t="n"/>
-      <c r="H33" s="7">
+      <c r="H33" s="7" t="str">
         <f>IF(OR($A33&lt;&gt;"Yes",F33="",G33=""),"",MATCH(F33,Lists!$B$1:$B$5,0)*MATCH(G33,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I33" s="7">
+      <c r="I33" s="7" t="str">
         <f>IF(H33="","",IF(H33&gt;=17,"Critical",IF(H33&gt;=10,"High",IF(H33&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -4012,15 +4012,15 @@
         </is>
       </c>
       <c r="K33" s="15" t="n"/>
-      <c r="L33" s="7">
+      <c r="L33" s="7" t="str">
         <f>IF(OR(H33="",K33=""),"",ROUND(H33*VLOOKUP(K33,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M33" s="7">
+      <c r="M33" s="7" t="str">
         <f>IF(L33="","",IF(L33&gt;=17,"Critical",IF(L33&gt;=10,"High",IF(L33&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N33" s="7">
+      <c r="N33" s="7" t="str">
         <f>IF(M33="","",IF(OR(M33="Low",M33="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -4034,7 +4034,7 @@
           <t>Appeals exceeding SLA</t>
         </is>
       </c>
-      <c r="V33">
+      <c r="V33" t="str">
         <f>IF(L33="","",L33+ROW()/100000)</f>
         <v/>
       </c>
@@ -4063,11 +4063,11 @@
       </c>
       <c r="F34" s="15" t="n"/>
       <c r="G34" s="15" t="n"/>
-      <c r="H34" s="7">
+      <c r="H34" s="7" t="str">
         <f>IF(OR($A34&lt;&gt;"Yes",F34="",G34=""),"",MATCH(F34,Lists!$B$1:$B$5,0)*MATCH(G34,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I34" s="7">
+      <c r="I34" s="7" t="str">
         <f>IF(H34="","",IF(H34&gt;=17,"Critical",IF(H34&gt;=10,"High",IF(H34&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -4077,15 +4077,15 @@
         </is>
       </c>
       <c r="K34" s="15" t="n"/>
-      <c r="L34" s="7">
+      <c r="L34" s="7" t="str">
         <f>IF(OR(H34="",K34=""),"",ROUND(H34*VLOOKUP(K34,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M34" s="7">
+      <c r="M34" s="7" t="str">
         <f>IF(L34="","",IF(L34&gt;=17,"Critical",IF(L34&gt;=10,"High",IF(L34&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N34" s="7">
+      <c r="N34" s="7" t="str">
         <f>IF(M34="","",IF(OR(M34="Low",M34="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -4099,7 +4099,7 @@
           <t>Systems with incomplete documentation pack</t>
         </is>
       </c>
-      <c r="V34">
+      <c r="V34" t="str">
         <f>IF(L34="","",L34+ROW()/100000)</f>
         <v/>
       </c>
@@ -4128,11 +4128,11 @@
       </c>
       <c r="F35" s="15" t="n"/>
       <c r="G35" s="15" t="n"/>
-      <c r="H35" s="7">
+      <c r="H35" s="7" t="str">
         <f>IF(OR($A35&lt;&gt;"Yes",F35="",G35=""),"",MATCH(F35,Lists!$B$1:$B$5,0)*MATCH(G35,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I35" s="7">
+      <c r="I35" s="7" t="str">
         <f>IF(H35="","",IF(H35&gt;=17,"Critical",IF(H35&gt;=10,"High",IF(H35&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -4142,15 +4142,15 @@
         </is>
       </c>
       <c r="K35" s="15" t="n"/>
-      <c r="L35" s="7">
+      <c r="L35" s="7" t="str">
         <f>IF(OR(H35="",K35=""),"",ROUND(H35*VLOOKUP(K35,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M35" s="7">
+      <c r="M35" s="7" t="str">
         <f>IF(L35="","",IF(L35&gt;=17,"Critical",IF(L35&gt;=10,"High",IF(L35&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N35" s="7">
+      <c r="N35" s="7" t="str">
         <f>IF(M35="","",IF(OR(M35="Low",M35="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -4164,7 +4164,7 @@
           <t>Blocked injection attempts / bypasses in testing</t>
         </is>
       </c>
-      <c r="V35">
+      <c r="V35" t="str">
         <f>IF(L35="","",L35+ROW()/100000)</f>
         <v/>
       </c>
@@ -4193,11 +4193,11 @@
       </c>
       <c r="F36" s="15" t="n"/>
       <c r="G36" s="15" t="n"/>
-      <c r="H36" s="7">
+      <c r="H36" s="7" t="str">
         <f>IF(OR($A36&lt;&gt;"Yes",F36="",G36=""),"",MATCH(F36,Lists!$B$1:$B$5,0)*MATCH(G36,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I36" s="7">
+      <c r="I36" s="7" t="str">
         <f>IF(H36="","",IF(H36&gt;=17,"Critical",IF(H36&gt;=10,"High",IF(H36&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -4207,15 +4207,15 @@
         </is>
       </c>
       <c r="K36" s="15" t="n"/>
-      <c r="L36" s="7">
+      <c r="L36" s="7" t="str">
         <f>IF(OR(H36="",K36=""),"",ROUND(H36*VLOOKUP(K36,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M36" s="7">
+      <c r="M36" s="7" t="str">
         <f>IF(L36="","",IF(L36&gt;=17,"Critical",IF(L36&gt;=10,"High",IF(L36&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N36" s="7">
+      <c r="N36" s="7" t="str">
         <f>IF(M36="","",IF(OR(M36="Low",M36="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -4229,7 +4229,7 @@
           <t>Integrity check failures</t>
         </is>
       </c>
-      <c r="V36">
+      <c r="V36" t="str">
         <f>IF(L36="","",L36+ROW()/100000)</f>
         <v/>
       </c>
@@ -4258,11 +4258,11 @@
       </c>
       <c r="F37" s="15" t="n"/>
       <c r="G37" s="15" t="n"/>
-      <c r="H37" s="7">
+      <c r="H37" s="7" t="str">
         <f>IF(OR($A37&lt;&gt;"Yes",F37="",G37=""),"",MATCH(F37,Lists!$B$1:$B$5,0)*MATCH(G37,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I37" s="7">
+      <c r="I37" s="7" t="str">
         <f>IF(H37="","",IF(H37&gt;=17,"Critical",IF(H37&gt;=10,"High",IF(H37&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -4272,15 +4272,15 @@
         </is>
       </c>
       <c r="K37" s="15" t="n"/>
-      <c r="L37" s="7">
+      <c r="L37" s="7" t="str">
         <f>IF(OR(H37="",K37=""),"",ROUND(H37*VLOOKUP(K37,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M37" s="7">
+      <c r="M37" s="7" t="str">
         <f>IF(L37="","",IF(L37&gt;=17,"Critical",IF(L37&gt;=10,"High",IF(L37&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N37" s="7">
+      <c r="N37" s="7" t="str">
         <f>IF(M37="","",IF(OR(M37="Low",M37="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -4294,7 +4294,7 @@
           <t>Anomalous query volumes</t>
         </is>
       </c>
-      <c r="V37">
+      <c r="V37" t="str">
         <f>IF(L37="","",L37+ROW()/100000)</f>
         <v/>
       </c>
@@ -4323,11 +4323,11 @@
       </c>
       <c r="F38" s="15" t="n"/>
       <c r="G38" s="15" t="n"/>
-      <c r="H38" s="7">
+      <c r="H38" s="7" t="str">
         <f>IF(OR($A38&lt;&gt;"Yes",F38="",G38=""),"",MATCH(F38,Lists!$B$1:$B$5,0)*MATCH(G38,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I38" s="7">
+      <c r="I38" s="7" t="str">
         <f>IF(H38="","",IF(H38&gt;=17,"Critical",IF(H38&gt;=10,"High",IF(H38&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -4337,15 +4337,15 @@
         </is>
       </c>
       <c r="K38" s="15" t="n"/>
-      <c r="L38" s="7">
+      <c r="L38" s="7" t="str">
         <f>IF(OR(H38="",K38=""),"",ROUND(H38*VLOOKUP(K38,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M38" s="7">
+      <c r="M38" s="7" t="str">
         <f>IF(L38="","",IF(L38&gt;=17,"Critical",IF(L38&gt;=10,"High",IF(L38&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N38" s="7">
+      <c r="N38" s="7" t="str">
         <f>IF(M38="","",IF(OR(M38="Low",M38="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -4359,7 +4359,7 @@
           <t>Agents / integrations with privileged standing access</t>
         </is>
       </c>
-      <c r="V38">
+      <c r="V38" t="str">
         <f>IF(L38="","",L38+ROW()/100000)</f>
         <v/>
       </c>
@@ -4388,11 +4388,11 @@
       </c>
       <c r="F39" s="15" t="n"/>
       <c r="G39" s="15" t="n"/>
-      <c r="H39" s="7">
+      <c r="H39" s="7" t="str">
         <f>IF(OR($A39&lt;&gt;"Yes",F39="",G39=""),"",MATCH(F39,Lists!$B$1:$B$5,0)*MATCH(G39,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I39" s="7">
+      <c r="I39" s="7" t="str">
         <f>IF(H39="","",IF(H39&gt;=17,"Critical",IF(H39&gt;=10,"High",IF(H39&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -4402,15 +4402,15 @@
         </is>
       </c>
       <c r="K39" s="15" t="n"/>
-      <c r="L39" s="7">
+      <c r="L39" s="7" t="str">
         <f>IF(OR(H39="",K39=""),"",ROUND(H39*VLOOKUP(K39,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M39" s="7">
+      <c r="M39" s="7" t="str">
         <f>IF(L39="","",IF(L39&gt;=17,"Critical",IF(L39&gt;=10,"High",IF(L39&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N39" s="7">
+      <c r="N39" s="7" t="str">
         <f>IF(M39="","",IF(OR(M39="Low",M39="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -4424,7 +4424,7 @@
           <t>Cross-tenant retrieval test failures</t>
         </is>
       </c>
-      <c r="V39">
+      <c r="V39" t="str">
         <f>IF(L39="","",L39+ROW()/100000)</f>
         <v/>
       </c>
@@ -4453,11 +4453,11 @@
       </c>
       <c r="F40" s="15" t="n"/>
       <c r="G40" s="15" t="n"/>
-      <c r="H40" s="7">
+      <c r="H40" s="7" t="str">
         <f>IF(OR($A40&lt;&gt;"Yes",F40="",G40=""),"",MATCH(F40,Lists!$B$1:$B$5,0)*MATCH(G40,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I40" s="7">
+      <c r="I40" s="7" t="str">
         <f>IF(H40="","",IF(H40&gt;=17,"Critical",IF(H40&gt;=10,"High",IF(H40&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -4467,15 +4467,15 @@
         </is>
       </c>
       <c r="K40" s="15" t="n"/>
-      <c r="L40" s="7">
+      <c r="L40" s="7" t="str">
         <f>IF(OR(H40="",K40=""),"",ROUND(H40*VLOOKUP(K40,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M40" s="7">
+      <c r="M40" s="7" t="str">
         <f>IF(L40="","",IF(L40&gt;=17,"Critical",IF(L40&gt;=10,"High",IF(L40&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N40" s="7">
+      <c r="N40" s="7" t="str">
         <f>IF(M40="","",IF(OR(M40="Low",M40="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -4489,7 +4489,7 @@
           <t>Blocked egress / SSRF attempts</t>
         </is>
       </c>
-      <c r="V40">
+      <c r="V40" t="str">
         <f>IF(L40="","",L40+ROW()/100000)</f>
         <v/>
       </c>
@@ -4518,11 +4518,11 @@
       </c>
       <c r="F41" s="15" t="n"/>
       <c r="G41" s="15" t="n"/>
-      <c r="H41" s="7">
+      <c r="H41" s="7" t="str">
         <f>IF(OR($A41&lt;&gt;"Yes",F41="",G41=""),"",MATCH(F41,Lists!$B$1:$B$5,0)*MATCH(G41,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I41" s="7">
+      <c r="I41" s="7" t="str">
         <f>IF(H41="","",IF(H41&gt;=17,"Critical",IF(H41&gt;=10,"High",IF(H41&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -4532,15 +4532,15 @@
         </is>
       </c>
       <c r="K41" s="15" t="n"/>
-      <c r="L41" s="7">
+      <c r="L41" s="7" t="str">
         <f>IF(OR(H41="",K41=""),"",ROUND(H41*VLOOKUP(K41,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M41" s="7">
+      <c r="M41" s="7" t="str">
         <f>IF(L41="","",IF(L41&gt;=17,"Critical",IF(L41&gt;=10,"High",IF(L41&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N41" s="7">
+      <c r="N41" s="7" t="str">
         <f>IF(M41="","",IF(OR(M41="Low",M41="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -4554,7 +4554,7 @@
           <t>Unscanned model artefacts</t>
         </is>
       </c>
-      <c r="V41">
+      <c r="V41" t="str">
         <f>IF(L41="","",L41+ROW()/100000)</f>
         <v/>
       </c>
@@ -4583,11 +4583,11 @@
       </c>
       <c r="F42" s="15" t="n"/>
       <c r="G42" s="15" t="n"/>
-      <c r="H42" s="7">
+      <c r="H42" s="7" t="str">
         <f>IF(OR($A42&lt;&gt;"Yes",F42="",G42=""),"",MATCH(F42,Lists!$B$1:$B$5,0)*MATCH(G42,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I42" s="7">
+      <c r="I42" s="7" t="str">
         <f>IF(H42="","",IF(H42&gt;=17,"Critical",IF(H42&gt;=10,"High",IF(H42&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -4597,15 +4597,15 @@
         </is>
       </c>
       <c r="K42" s="15" t="n"/>
-      <c r="L42" s="7">
+      <c r="L42" s="7" t="str">
         <f>IF(OR(H42="",K42=""),"",ROUND(H42*VLOOKUP(K42,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M42" s="7">
+      <c r="M42" s="7" t="str">
         <f>IF(L42="","",IF(L42&gt;=17,"Critical",IF(L42&gt;=10,"High",IF(L42&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N42" s="7">
+      <c r="N42" s="7" t="str">
         <f>IF(M42="","",IF(OR(M42="Low",M42="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -4619,7 +4619,7 @@
           <t>Override / challenge rate</t>
         </is>
       </c>
-      <c r="V42">
+      <c r="V42" t="str">
         <f>IF(L42="","",L42+ROW()/100000)</f>
         <v/>
       </c>
@@ -4648,11 +4648,11 @@
       </c>
       <c r="F43" s="15" t="n"/>
       <c r="G43" s="15" t="n"/>
-      <c r="H43" s="7">
+      <c r="H43" s="7" t="str">
         <f>IF(OR($A43&lt;&gt;"Yes",F43="",G43=""),"",MATCH(F43,Lists!$B$1:$B$5,0)*MATCH(G43,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I43" s="7">
+      <c r="I43" s="7" t="str">
         <f>IF(H43="","",IF(H43&gt;=17,"Critical",IF(H43&gt;=10,"High",IF(H43&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -4662,15 +4662,15 @@
         </is>
       </c>
       <c r="K43" s="15" t="n"/>
-      <c r="L43" s="7">
+      <c r="L43" s="7" t="str">
         <f>IF(OR(H43="",K43=""),"",ROUND(H43*VLOOKUP(K43,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M43" s="7">
+      <c r="M43" s="7" t="str">
         <f>IF(L43="","",IF(L43&gt;=17,"Critical",IF(L43&gt;=10,"High",IF(L43&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N43" s="7">
+      <c r="N43" s="7" t="str">
         <f>IF(M43="","",IF(OR(M43="Low",M43="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -4684,7 +4684,7 @@
           <t>Oversight roles without training</t>
         </is>
       </c>
-      <c r="V43">
+      <c r="V43" t="str">
         <f>IF(L43="","",L43+ROW()/100000)</f>
         <v/>
       </c>
@@ -4713,11 +4713,11 @@
       </c>
       <c r="F44" s="15" t="n"/>
       <c r="G44" s="15" t="n"/>
-      <c r="H44" s="7">
+      <c r="H44" s="7" t="str">
         <f>IF(OR($A44&lt;&gt;"Yes",F44="",G44=""),"",MATCH(F44,Lists!$B$1:$B$5,0)*MATCH(G44,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I44" s="7">
+      <c r="I44" s="7" t="str">
         <f>IF(H44="","",IF(H44&gt;=17,"Critical",IF(H44&gt;=10,"High",IF(H44&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -4727,15 +4727,15 @@
         </is>
       </c>
       <c r="K44" s="15" t="n"/>
-      <c r="L44" s="7">
+      <c r="L44" s="7" t="str">
         <f>IF(OR(H44="",K44=""),"",ROUND(H44*VLOOKUP(K44,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M44" s="7">
+      <c r="M44" s="7" t="str">
         <f>IF(L44="","",IF(L44&gt;=17,"Critical",IF(L44&gt;=10,"High",IF(L44&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N44" s="7">
+      <c r="N44" s="7" t="str">
         <f>IF(M44="","",IF(OR(M44="Low",M44="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -4749,7 +4749,7 @@
           <t>High-impact agent actions without approval</t>
         </is>
       </c>
-      <c r="V44">
+      <c r="V44" t="str">
         <f>IF(L44="","",L44+ROW()/100000)</f>
         <v/>
       </c>
@@ -4778,11 +4778,11 @@
       </c>
       <c r="F45" s="15" t="n"/>
       <c r="G45" s="15" t="n"/>
-      <c r="H45" s="7">
+      <c r="H45" s="7" t="str">
         <f>IF(OR($A45&lt;&gt;"Yes",F45="",G45=""),"",MATCH(F45,Lists!$B$1:$B$5,0)*MATCH(G45,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I45" s="7">
+      <c r="I45" s="7" t="str">
         <f>IF(H45="","",IF(H45&gt;=17,"Critical",IF(H45&gt;=10,"High",IF(H45&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -4792,15 +4792,15 @@
         </is>
       </c>
       <c r="K45" s="15" t="n"/>
-      <c r="L45" s="7">
+      <c r="L45" s="7" t="str">
         <f>IF(OR(H45="",K45=""),"",ROUND(H45*VLOOKUP(K45,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M45" s="7">
+      <c r="M45" s="7" t="str">
         <f>IF(L45="","",IF(L45&gt;=17,"Critical",IF(L45&gt;=10,"High",IF(L45&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N45" s="7">
+      <c r="N45" s="7" t="str">
         <f>IF(M45="","",IF(OR(M45="Low",M45="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -4814,7 +4814,7 @@
           <t>Staff sentiment / attrition in affected roles</t>
         </is>
       </c>
-      <c r="V45">
+      <c r="V45" t="str">
         <f>IF(L45="","",L45+ROW()/100000)</f>
         <v/>
       </c>
@@ -4843,11 +4843,11 @@
       </c>
       <c r="F46" s="15" t="n"/>
       <c r="G46" s="15" t="n"/>
-      <c r="H46" s="7">
+      <c r="H46" s="7" t="str">
         <f>IF(OR($A46&lt;&gt;"Yes",F46="",G46=""),"",MATCH(F46,Lists!$B$1:$B$5,0)*MATCH(G46,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I46" s="7">
+      <c r="I46" s="7" t="str">
         <f>IF(H46="","",IF(H46&gt;=17,"Critical",IF(H46&gt;=10,"High",IF(H46&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -4857,15 +4857,15 @@
         </is>
       </c>
       <c r="K46" s="15" t="n"/>
-      <c r="L46" s="7">
+      <c r="L46" s="7" t="str">
         <f>IF(OR(H46="",K46=""),"",ROUND(H46*VLOOKUP(K46,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M46" s="7">
+      <c r="M46" s="7" t="str">
         <f>IF(L46="","",IF(L46&gt;=17,"Critical",IF(L46&gt;=10,"High",IF(L46&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N46" s="7">
+      <c r="N46" s="7" t="str">
         <f>IF(M46="","",IF(OR(M46="Low",M46="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -4879,7 +4879,7 @@
           <t>% critical AI workloads on single provider</t>
         </is>
       </c>
-      <c r="V46">
+      <c r="V46" t="str">
         <f>IF(L46="","",L46+ROW()/100000)</f>
         <v/>
       </c>
@@ -4908,11 +4908,11 @@
       </c>
       <c r="F47" s="15" t="n"/>
       <c r="G47" s="15" t="n"/>
-      <c r="H47" s="7">
+      <c r="H47" s="7" t="str">
         <f>IF(OR($A47&lt;&gt;"Yes",F47="",G47=""),"",MATCH(F47,Lists!$B$1:$B$5,0)*MATCH(G47,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I47" s="7">
+      <c r="I47" s="7" t="str">
         <f>IF(H47="","",IF(H47&gt;=17,"Critical",IF(H47&gt;=10,"High",IF(H47&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -4922,15 +4922,15 @@
         </is>
       </c>
       <c r="K47" s="15" t="n"/>
-      <c r="L47" s="7">
+      <c r="L47" s="7" t="str">
         <f>IF(OR(H47="",K47=""),"",ROUND(H47*VLOOKUP(K47,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M47" s="7">
+      <c r="M47" s="7" t="str">
         <f>IF(L47="","",IF(L47&gt;=17,"Critical",IF(L47&gt;=10,"High",IF(L47&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N47" s="7">
+      <c r="N47" s="7" t="str">
         <f>IF(M47="","",IF(OR(M47="Low",M47="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -4944,7 +4944,7 @@
           <t>Vendors without current assurance evidence</t>
         </is>
       </c>
-      <c r="V47">
+      <c r="V47" t="str">
         <f>IF(L47="","",L47+ROW()/100000)</f>
         <v/>
       </c>
@@ -4973,11 +4973,11 @@
       </c>
       <c r="F48" s="15" t="n"/>
       <c r="G48" s="15" t="n"/>
-      <c r="H48" s="7">
+      <c r="H48" s="7" t="str">
         <f>IF(OR($A48&lt;&gt;"Yes",F48="",G48=""),"",MATCH(F48,Lists!$B$1:$B$5,0)*MATCH(G48,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I48" s="7">
+      <c r="I48" s="7" t="str">
         <f>IF(H48="","",IF(H48&gt;=17,"Critical",IF(H48&gt;=10,"High",IF(H48&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -4987,15 +4987,15 @@
         </is>
       </c>
       <c r="K48" s="15" t="n"/>
-      <c r="L48" s="7">
+      <c r="L48" s="7" t="str">
         <f>IF(OR(H48="",K48=""),"",ROUND(H48*VLOOKUP(K48,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M48" s="7">
+      <c r="M48" s="7" t="str">
         <f>IF(L48="","",IF(L48&gt;=17,"Critical",IF(L48&gt;=10,"High",IF(L48&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N48" s="7">
+      <c r="N48" s="7" t="str">
         <f>IF(M48="","",IF(OR(M48="Low",M48="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5009,7 +5009,7 @@
           <t>Contracts lacking no-training clause</t>
         </is>
       </c>
-      <c r="V48">
+      <c r="V48" t="str">
         <f>IF(L48="","",L48+ROW()/100000)</f>
         <v/>
       </c>
@@ -5038,11 +5038,11 @@
       </c>
       <c r="F49" s="15" t="n"/>
       <c r="G49" s="15" t="n"/>
-      <c r="H49" s="7">
+      <c r="H49" s="7" t="str">
         <f>IF(OR($A49&lt;&gt;"Yes",F49="",G49=""),"",MATCH(F49,Lists!$B$1:$B$5,0)*MATCH(G49,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I49" s="7">
+      <c r="I49" s="7" t="str">
         <f>IF(H49="","",IF(H49&gt;=17,"Critical",IF(H49&gt;=10,"High",IF(H49&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -5052,15 +5052,15 @@
         </is>
       </c>
       <c r="K49" s="15" t="n"/>
-      <c r="L49" s="7">
+      <c r="L49" s="7" t="str">
         <f>IF(OR(H49="",K49=""),"",ROUND(H49*VLOOKUP(K49,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M49" s="7">
+      <c r="M49" s="7" t="str">
         <f>IF(L49="","",IF(L49&gt;=17,"Critical",IF(L49&gt;=10,"High",IF(L49&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N49" s="7">
+      <c r="N49" s="7" t="str">
         <f>IF(M49="","",IF(OR(M49="Low",M49="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5074,7 +5074,7 @@
           <t>AI service availability vs SLA</t>
         </is>
       </c>
-      <c r="V49">
+      <c r="V49" t="str">
         <f>IF(L49="","",L49+ROW()/100000)</f>
         <v/>
       </c>
@@ -5103,11 +5103,11 @@
       </c>
       <c r="F50" s="15" t="n"/>
       <c r="G50" s="15" t="n"/>
-      <c r="H50" s="7">
+      <c r="H50" s="7" t="str">
         <f>IF(OR($A50&lt;&gt;"Yes",F50="",G50=""),"",MATCH(F50,Lists!$B$1:$B$5,0)*MATCH(G50,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I50" s="7">
+      <c r="I50" s="7" t="str">
         <f>IF(H50="","",IF(H50&gt;=17,"Critical",IF(H50&gt;=10,"High",IF(H50&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -5117,15 +5117,15 @@
         </is>
       </c>
       <c r="K50" s="15" t="n"/>
-      <c r="L50" s="7">
+      <c r="L50" s="7" t="str">
         <f>IF(OR(H50="",K50=""),"",ROUND(H50*VLOOKUP(K50,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M50" s="7">
+      <c r="M50" s="7" t="str">
         <f>IF(L50="","",IF(L50&gt;=17,"Critical",IF(L50&gt;=10,"High",IF(L50&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N50" s="7">
+      <c r="N50" s="7" t="str">
         <f>IF(M50="","",IF(OR(M50="Low",M50="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5139,7 +5139,7 @@
           <t>AI spend vs budget</t>
         </is>
       </c>
-      <c r="V50">
+      <c r="V50" t="str">
         <f>IF(L50="","",L50+ROW()/100000)</f>
         <v/>
       </c>
@@ -5168,11 +5168,11 @@
       </c>
       <c r="F51" s="15" t="n"/>
       <c r="G51" s="15" t="n"/>
-      <c r="H51" s="7">
+      <c r="H51" s="7" t="str">
         <f>IF(OR($A51&lt;&gt;"Yes",F51="",G51=""),"",MATCH(F51,Lists!$B$1:$B$5,0)*MATCH(G51,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I51" s="7">
+      <c r="I51" s="7" t="str">
         <f>IF(H51="","",IF(H51&gt;=17,"Critical",IF(H51&gt;=10,"High",IF(H51&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -5182,15 +5182,15 @@
         </is>
       </c>
       <c r="K51" s="15" t="n"/>
-      <c r="L51" s="7">
+      <c r="L51" s="7" t="str">
         <f>IF(OR(H51="",K51=""),"",ROUND(H51*VLOOKUP(K51,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M51" s="7">
+      <c r="M51" s="7" t="str">
         <f>IF(L51="","",IF(L51&gt;=17,"Critical",IF(L51&gt;=10,"High",IF(L51&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N51" s="7">
+      <c r="N51" s="7" t="str">
         <f>IF(M51="","",IF(OR(M51="Low",M51="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5204,7 +5204,7 @@
           <t>Kill-switch test age (days)</t>
         </is>
       </c>
-      <c r="V51">
+      <c r="V51" t="str">
         <f>IF(L51="","",L51+ROW()/100000)</f>
         <v/>
       </c>
@@ -5233,11 +5233,11 @@
       </c>
       <c r="F52" s="15" t="n"/>
       <c r="G52" s="15" t="n"/>
-      <c r="H52" s="7">
+      <c r="H52" s="7" t="str">
         <f>IF(OR($A52&lt;&gt;"Yes",F52="",G52=""),"",MATCH(F52,Lists!$B$1:$B$5,0)*MATCH(G52,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I52" s="7">
+      <c r="I52" s="7" t="str">
         <f>IF(H52="","",IF(H52&gt;=17,"Critical",IF(H52&gt;=10,"High",IF(H52&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -5247,15 +5247,15 @@
         </is>
       </c>
       <c r="K52" s="15" t="n"/>
-      <c r="L52" s="7">
+      <c r="L52" s="7" t="str">
         <f>IF(OR(H52="",K52=""),"",ROUND(H52*VLOOKUP(K52,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M52" s="7">
+      <c r="M52" s="7" t="str">
         <f>IF(L52="","",IF(L52&gt;=17,"Critical",IF(L52&gt;=10,"High",IF(L52&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N52" s="7">
+      <c r="N52" s="7" t="str">
         <f>IF(M52="","",IF(OR(M52="Low",M52="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5269,7 +5269,7 @@
           <t>kgCO2e per 1,000 inferences</t>
         </is>
       </c>
-      <c r="V52">
+      <c r="V52" t="str">
         <f>IF(L52="","",L52+ROW()/100000)</f>
         <v/>
       </c>
@@ -5298,11 +5298,11 @@
       </c>
       <c r="F53" s="15" t="n"/>
       <c r="G53" s="15" t="n"/>
-      <c r="H53" s="7">
+      <c r="H53" s="7" t="str">
         <f>IF(OR($A53&lt;&gt;"Yes",F53="",G53=""),"",MATCH(F53,Lists!$B$1:$B$5,0)*MATCH(G53,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I53" s="7">
+      <c r="I53" s="7" t="str">
         <f>IF(H53="","",IF(H53&gt;=17,"Critical",IF(H53&gt;=10,"High",IF(H53&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -5312,15 +5312,15 @@
         </is>
       </c>
       <c r="K53" s="15" t="n"/>
-      <c r="L53" s="7">
+      <c r="L53" s="7" t="str">
         <f>IF(OR(H53="",K53=""),"",ROUND(H53*VLOOKUP(K53,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M53" s="7">
+      <c r="M53" s="7" t="str">
         <f>IF(L53="","",IF(L53&gt;=17,"Critical",IF(L53&gt;=10,"High",IF(L53&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N53" s="7">
+      <c r="N53" s="7" t="str">
         <f>IF(M53="","",IF(OR(M53="Low",M53="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5334,7 +5334,7 @@
           <t>Content-policy violations per 1,000 outputs</t>
         </is>
       </c>
-      <c r="V53">
+      <c r="V53" t="str">
         <f>IF(L53="","",L53+ROW()/100000)</f>
         <v/>
       </c>
@@ -5363,11 +5363,11 @@
       </c>
       <c r="F54" s="15" t="n"/>
       <c r="G54" s="15" t="n"/>
-      <c r="H54" s="7">
+      <c r="H54" s="7" t="str">
         <f>IF(OR($A54&lt;&gt;"Yes",F54="",G54=""),"",MATCH(F54,Lists!$B$1:$B$5,0)*MATCH(G54,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I54" s="7">
+      <c r="I54" s="7" t="str">
         <f>IF(H54="","",IF(H54&gt;=17,"Critical",IF(H54&gt;=10,"High",IF(H54&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -5377,15 +5377,15 @@
         </is>
       </c>
       <c r="K54" s="15" t="n"/>
-      <c r="L54" s="7">
+      <c r="L54" s="7" t="str">
         <f>IF(OR(H54="",K54=""),"",ROUND(H54*VLOOKUP(K54,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M54" s="7">
+      <c r="M54" s="7" t="str">
         <f>IF(L54="","",IF(L54&gt;=17,"Critical",IF(L54&gt;=10,"High",IF(L54&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N54" s="7">
+      <c r="N54" s="7" t="str">
         <f>IF(M54="","",IF(OR(M54="Low",M54="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5399,7 +5399,7 @@
           <t>Client complaints linked to AI</t>
         </is>
       </c>
-      <c r="V54">
+      <c r="V54" t="str">
         <f>IF(L54="","",L54+ROW()/100000)</f>
         <v/>
       </c>
@@ -5428,11 +5428,11 @@
       </c>
       <c r="F55" s="15" t="n"/>
       <c r="G55" s="15" t="n"/>
-      <c r="H55" s="7">
+      <c r="H55" s="7" t="str">
         <f>IF(OR($A55&lt;&gt;"Yes",F55="",G55=""),"",MATCH(F55,Lists!$B$1:$B$5,0)*MATCH(G55,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I55" s="7">
+      <c r="I55" s="7" t="str">
         <f>IF(H55="","",IF(H55&gt;=17,"Critical",IF(H55&gt;=10,"High",IF(H55&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -5442,15 +5442,15 @@
         </is>
       </c>
       <c r="K55" s="15" t="n"/>
-      <c r="L55" s="7">
+      <c r="L55" s="7" t="str">
         <f>IF(OR(H55="",K55=""),"",ROUND(H55*VLOOKUP(K55,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M55" s="7">
+      <c r="M55" s="7" t="str">
         <f>IF(L55="","",IF(L55&gt;=17,"Critical",IF(L55&gt;=10,"High",IF(L55&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N55" s="7">
+      <c r="N55" s="7" t="str">
         <f>IF(M55="","",IF(OR(M55="Low",M55="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5464,7 +5464,7 @@
           <t>Deepfake / BEC attempts detected</t>
         </is>
       </c>
-      <c r="V55">
+      <c r="V55" t="str">
         <f>IF(L55="","",L55+ROW()/100000)</f>
         <v/>
       </c>
@@ -5493,11 +5493,11 @@
       </c>
       <c r="F56" s="15" t="n"/>
       <c r="G56" s="15" t="n"/>
-      <c r="H56" s="7">
+      <c r="H56" s="7" t="str">
         <f>IF(OR($A56&lt;&gt;"Yes",F56="",G56=""),"",MATCH(F56,Lists!$B$1:$B$5,0)*MATCH(G56,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I56" s="7">
+      <c r="I56" s="7" t="str">
         <f>IF(H56="","",IF(H56&gt;=17,"Critical",IF(H56&gt;=10,"High",IF(H56&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
@@ -5507,15 +5507,15 @@
         </is>
       </c>
       <c r="K56" s="15" t="n"/>
-      <c r="L56" s="7">
+      <c r="L56" s="7" t="str">
         <f>IF(OR(H56="",K56=""),"",ROUND(H56*VLOOKUP(K56,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M56" s="7">
+      <c r="M56" s="7" t="str">
         <f>IF(L56="","",IF(L56&gt;=17,"Critical",IF(L56&gt;=10,"High",IF(L56&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N56" s="7">
+      <c r="N56" s="7" t="str">
         <f>IF(M56="","",IF(OR(M56="Low",M56="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5529,7 +5529,7 @@
           <t>Mean time to remediate critical vulnerabilities</t>
         </is>
       </c>
-      <c r="V56">
+      <c r="V56" t="str">
         <f>IF(L56="","",L56+ROW()/100000)</f>
         <v/>
       </c>
@@ -5546,25 +5546,25 @@
       <c r="E57" s="5" t="n"/>
       <c r="F57" s="15" t="n"/>
       <c r="G57" s="15" t="n"/>
-      <c r="H57" s="7">
+      <c r="H57" s="7" t="str">
         <f>IF(OR($A57&lt;&gt;"Yes",F57="",G57=""),"",MATCH(F57,Lists!$B$1:$B$5,0)*MATCH(G57,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I57" s="7">
+      <c r="I57" s="7" t="str">
         <f>IF(H57="","",IF(H57&gt;=17,"Critical",IF(H57&gt;=10,"High",IF(H57&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
       <c r="J57" s="5" t="n"/>
       <c r="K57" s="15" t="n"/>
-      <c r="L57" s="7">
+      <c r="L57" s="7" t="str">
         <f>IF(OR(H57="",K57=""),"",ROUND(H57*VLOOKUP(K57,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M57" s="7">
+      <c r="M57" s="7" t="str">
         <f>IF(L57="","",IF(L57&gt;=17,"Critical",IF(L57&gt;=10,"High",IF(L57&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N57" s="7">
+      <c r="N57" s="7" t="str">
         <f>IF(M57="","",IF(OR(M57="Low",M57="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5574,7 +5574,7 @@
       <c r="R57" s="15" t="n"/>
       <c r="S57" s="15" t="n"/>
       <c r="T57" s="5" t="n"/>
-      <c r="V57">
+      <c r="V57" t="str">
         <f>IF(L57="","",L57+ROW()/100000)</f>
         <v/>
       </c>
@@ -5591,25 +5591,25 @@
       <c r="E58" s="5" t="n"/>
       <c r="F58" s="15" t="n"/>
       <c r="G58" s="15" t="n"/>
-      <c r="H58" s="7">
+      <c r="H58" s="7" t="str">
         <f>IF(OR($A58&lt;&gt;"Yes",F58="",G58=""),"",MATCH(F58,Lists!$B$1:$B$5,0)*MATCH(G58,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I58" s="7">
+      <c r="I58" s="7" t="str">
         <f>IF(H58="","",IF(H58&gt;=17,"Critical",IF(H58&gt;=10,"High",IF(H58&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
       <c r="J58" s="5" t="n"/>
       <c r="K58" s="15" t="n"/>
-      <c r="L58" s="7">
+      <c r="L58" s="7" t="str">
         <f>IF(OR(H58="",K58=""),"",ROUND(H58*VLOOKUP(K58,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M58" s="7">
+      <c r="M58" s="7" t="str">
         <f>IF(L58="","",IF(L58&gt;=17,"Critical",IF(L58&gt;=10,"High",IF(L58&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N58" s="7">
+      <c r="N58" s="7" t="str">
         <f>IF(M58="","",IF(OR(M58="Low",M58="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5619,7 +5619,7 @@
       <c r="R58" s="15" t="n"/>
       <c r="S58" s="15" t="n"/>
       <c r="T58" s="5" t="n"/>
-      <c r="V58">
+      <c r="V58" t="str">
         <f>IF(L58="","",L58+ROW()/100000)</f>
         <v/>
       </c>
@@ -5636,25 +5636,25 @@
       <c r="E59" s="5" t="n"/>
       <c r="F59" s="15" t="n"/>
       <c r="G59" s="15" t="n"/>
-      <c r="H59" s="7">
+      <c r="H59" s="7" t="str">
         <f>IF(OR($A59&lt;&gt;"Yes",F59="",G59=""),"",MATCH(F59,Lists!$B$1:$B$5,0)*MATCH(G59,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I59" s="7">
+      <c r="I59" s="7" t="str">
         <f>IF(H59="","",IF(H59&gt;=17,"Critical",IF(H59&gt;=10,"High",IF(H59&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
       <c r="J59" s="5" t="n"/>
       <c r="K59" s="15" t="n"/>
-      <c r="L59" s="7">
+      <c r="L59" s="7" t="str">
         <f>IF(OR(H59="",K59=""),"",ROUND(H59*VLOOKUP(K59,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M59" s="7">
+      <c r="M59" s="7" t="str">
         <f>IF(L59="","",IF(L59&gt;=17,"Critical",IF(L59&gt;=10,"High",IF(L59&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N59" s="7">
+      <c r="N59" s="7" t="str">
         <f>IF(M59="","",IF(OR(M59="Low",M59="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5664,7 +5664,7 @@
       <c r="R59" s="15" t="n"/>
       <c r="S59" s="15" t="n"/>
       <c r="T59" s="5" t="n"/>
-      <c r="V59">
+      <c r="V59" t="str">
         <f>IF(L59="","",L59+ROW()/100000)</f>
         <v/>
       </c>
@@ -5681,25 +5681,25 @@
       <c r="E60" s="5" t="n"/>
       <c r="F60" s="15" t="n"/>
       <c r="G60" s="15" t="n"/>
-      <c r="H60" s="7">
+      <c r="H60" s="7" t="str">
         <f>IF(OR($A60&lt;&gt;"Yes",F60="",G60=""),"",MATCH(F60,Lists!$B$1:$B$5,0)*MATCH(G60,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I60" s="7">
+      <c r="I60" s="7" t="str">
         <f>IF(H60="","",IF(H60&gt;=17,"Critical",IF(H60&gt;=10,"High",IF(H60&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
       <c r="J60" s="5" t="n"/>
       <c r="K60" s="15" t="n"/>
-      <c r="L60" s="7">
+      <c r="L60" s="7" t="str">
         <f>IF(OR(H60="",K60=""),"",ROUND(H60*VLOOKUP(K60,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M60" s="7">
+      <c r="M60" s="7" t="str">
         <f>IF(L60="","",IF(L60&gt;=17,"Critical",IF(L60&gt;=10,"High",IF(L60&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N60" s="7">
+      <c r="N60" s="7" t="str">
         <f>IF(M60="","",IF(OR(M60="Low",M60="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5709,7 +5709,7 @@
       <c r="R60" s="15" t="n"/>
       <c r="S60" s="15" t="n"/>
       <c r="T60" s="5" t="n"/>
-      <c r="V60">
+      <c r="V60" t="str">
         <f>IF(L60="","",L60+ROW()/100000)</f>
         <v/>
       </c>
@@ -5726,25 +5726,25 @@
       <c r="E61" s="5" t="n"/>
       <c r="F61" s="15" t="n"/>
       <c r="G61" s="15" t="n"/>
-      <c r="H61" s="7">
+      <c r="H61" s="7" t="str">
         <f>IF(OR($A61&lt;&gt;"Yes",F61="",G61=""),"",MATCH(F61,Lists!$B$1:$B$5,0)*MATCH(G61,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I61" s="7">
+      <c r="I61" s="7" t="str">
         <f>IF(H61="","",IF(H61&gt;=17,"Critical",IF(H61&gt;=10,"High",IF(H61&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
       <c r="J61" s="5" t="n"/>
       <c r="K61" s="15" t="n"/>
-      <c r="L61" s="7">
+      <c r="L61" s="7" t="str">
         <f>IF(OR(H61="",K61=""),"",ROUND(H61*VLOOKUP(K61,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M61" s="7">
+      <c r="M61" s="7" t="str">
         <f>IF(L61="","",IF(L61&gt;=17,"Critical",IF(L61&gt;=10,"High",IF(L61&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N61" s="7">
+      <c r="N61" s="7" t="str">
         <f>IF(M61="","",IF(OR(M61="Low",M61="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5754,7 +5754,7 @@
       <c r="R61" s="15" t="n"/>
       <c r="S61" s="15" t="n"/>
       <c r="T61" s="5" t="n"/>
-      <c r="V61">
+      <c r="V61" t="str">
         <f>IF(L61="","",L61+ROW()/100000)</f>
         <v/>
       </c>
@@ -5771,25 +5771,25 @@
       <c r="E62" s="5" t="n"/>
       <c r="F62" s="15" t="n"/>
       <c r="G62" s="15" t="n"/>
-      <c r="H62" s="7">
+      <c r="H62" s="7" t="str">
         <f>IF(OR($A62&lt;&gt;"Yes",F62="",G62=""),"",MATCH(F62,Lists!$B$1:$B$5,0)*MATCH(G62,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I62" s="7">
+      <c r="I62" s="7" t="str">
         <f>IF(H62="","",IF(H62&gt;=17,"Critical",IF(H62&gt;=10,"High",IF(H62&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
       <c r="J62" s="5" t="n"/>
       <c r="K62" s="15" t="n"/>
-      <c r="L62" s="7">
+      <c r="L62" s="7" t="str">
         <f>IF(OR(H62="",K62=""),"",ROUND(H62*VLOOKUP(K62,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M62" s="7">
+      <c r="M62" s="7" t="str">
         <f>IF(L62="","",IF(L62&gt;=17,"Critical",IF(L62&gt;=10,"High",IF(L62&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N62" s="7">
+      <c r="N62" s="7" t="str">
         <f>IF(M62="","",IF(OR(M62="Low",M62="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5799,7 +5799,7 @@
       <c r="R62" s="15" t="n"/>
       <c r="S62" s="15" t="n"/>
       <c r="T62" s="5" t="n"/>
-      <c r="V62">
+      <c r="V62" t="str">
         <f>IF(L62="","",L62+ROW()/100000)</f>
         <v/>
       </c>
@@ -5816,25 +5816,25 @@
       <c r="E63" s="5" t="n"/>
       <c r="F63" s="15" t="n"/>
       <c r="G63" s="15" t="n"/>
-      <c r="H63" s="7">
+      <c r="H63" s="7" t="str">
         <f>IF(OR($A63&lt;&gt;"Yes",F63="",G63=""),"",MATCH(F63,Lists!$B$1:$B$5,0)*MATCH(G63,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I63" s="7">
+      <c r="I63" s="7" t="str">
         <f>IF(H63="","",IF(H63&gt;=17,"Critical",IF(H63&gt;=10,"High",IF(H63&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
       <c r="J63" s="5" t="n"/>
       <c r="K63" s="15" t="n"/>
-      <c r="L63" s="7">
+      <c r="L63" s="7" t="str">
         <f>IF(OR(H63="",K63=""),"",ROUND(H63*VLOOKUP(K63,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M63" s="7">
+      <c r="M63" s="7" t="str">
         <f>IF(L63="","",IF(L63&gt;=17,"Critical",IF(L63&gt;=10,"High",IF(L63&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N63" s="7">
+      <c r="N63" s="7" t="str">
         <f>IF(M63="","",IF(OR(M63="Low",M63="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5844,7 +5844,7 @@
       <c r="R63" s="15" t="n"/>
       <c r="S63" s="15" t="n"/>
       <c r="T63" s="5" t="n"/>
-      <c r="V63">
+      <c r="V63" t="str">
         <f>IF(L63="","",L63+ROW()/100000)</f>
         <v/>
       </c>
@@ -5861,25 +5861,25 @@
       <c r="E64" s="5" t="n"/>
       <c r="F64" s="15" t="n"/>
       <c r="G64" s="15" t="n"/>
-      <c r="H64" s="7">
+      <c r="H64" s="7" t="str">
         <f>IF(OR($A64&lt;&gt;"Yes",F64="",G64=""),"",MATCH(F64,Lists!$B$1:$B$5,0)*MATCH(G64,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I64" s="7">
+      <c r="I64" s="7" t="str">
         <f>IF(H64="","",IF(H64&gt;=17,"Critical",IF(H64&gt;=10,"High",IF(H64&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
       <c r="J64" s="5" t="n"/>
       <c r="K64" s="15" t="n"/>
-      <c r="L64" s="7">
+      <c r="L64" s="7" t="str">
         <f>IF(OR(H64="",K64=""),"",ROUND(H64*VLOOKUP(K64,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M64" s="7">
+      <c r="M64" s="7" t="str">
         <f>IF(L64="","",IF(L64&gt;=17,"Critical",IF(L64&gt;=10,"High",IF(L64&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N64" s="7">
+      <c r="N64" s="7" t="str">
         <f>IF(M64="","",IF(OR(M64="Low",M64="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5889,7 +5889,7 @@
       <c r="R64" s="15" t="n"/>
       <c r="S64" s="15" t="n"/>
       <c r="T64" s="5" t="n"/>
-      <c r="V64">
+      <c r="V64" t="str">
         <f>IF(L64="","",L64+ROW()/100000)</f>
         <v/>
       </c>
@@ -5906,25 +5906,25 @@
       <c r="E65" s="5" t="n"/>
       <c r="F65" s="15" t="n"/>
       <c r="G65" s="15" t="n"/>
-      <c r="H65" s="7">
+      <c r="H65" s="7" t="str">
         <f>IF(OR($A65&lt;&gt;"Yes",F65="",G65=""),"",MATCH(F65,Lists!$B$1:$B$5,0)*MATCH(G65,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I65" s="7">
+      <c r="I65" s="7" t="str">
         <f>IF(H65="","",IF(H65&gt;=17,"Critical",IF(H65&gt;=10,"High",IF(H65&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
       <c r="J65" s="5" t="n"/>
       <c r="K65" s="15" t="n"/>
-      <c r="L65" s="7">
+      <c r="L65" s="7" t="str">
         <f>IF(OR(H65="",K65=""),"",ROUND(H65*VLOOKUP(K65,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M65" s="7">
+      <c r="M65" s="7" t="str">
         <f>IF(L65="","",IF(L65&gt;=17,"Critical",IF(L65&gt;=10,"High",IF(L65&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N65" s="7">
+      <c r="N65" s="7" t="str">
         <f>IF(M65="","",IF(OR(M65="Low",M65="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5934,7 +5934,7 @@
       <c r="R65" s="15" t="n"/>
       <c r="S65" s="15" t="n"/>
       <c r="T65" s="5" t="n"/>
-      <c r="V65">
+      <c r="V65" t="str">
         <f>IF(L65="","",L65+ROW()/100000)</f>
         <v/>
       </c>
@@ -5951,25 +5951,25 @@
       <c r="E66" s="5" t="n"/>
       <c r="F66" s="15" t="n"/>
       <c r="G66" s="15" t="n"/>
-      <c r="H66" s="7">
+      <c r="H66" s="7" t="str">
         <f>IF(OR($A66&lt;&gt;"Yes",F66="",G66=""),"",MATCH(F66,Lists!$B$1:$B$5,0)*MATCH(G66,Lists!$C$1:$C$5,0))</f>
         <v/>
       </c>
-      <c r="I66" s="7">
+      <c r="I66" s="7" t="str">
         <f>IF(H66="","",IF(H66&gt;=17,"Critical",IF(H66&gt;=10,"High",IF(H66&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
       <c r="J66" s="5" t="n"/>
       <c r="K66" s="15" t="n"/>
-      <c r="L66" s="7">
+      <c r="L66" s="7" t="str">
         <f>IF(OR(H66="",K66=""),"",ROUND(H66*VLOOKUP(K66,Scales!$A$22:$B$25,2,FALSE),1))</f>
         <v/>
       </c>
-      <c r="M66" s="7">
+      <c r="M66" s="7" t="str">
         <f>IF(L66="","",IF(L66&gt;=17,"Critical",IF(L66&gt;=10,"High",IF(L66&gt;=5,"Medium","Low"))))</f>
         <v/>
       </c>
-      <c r="N66" s="7">
+      <c r="N66" s="7" t="str">
         <f>IF(M66="","",IF(OR(M66="Low",M66="Medium"),"Yes","No"))</f>
         <v/>
       </c>
@@ -5979,7 +5979,7 @@
       <c r="R66" s="15" t="n"/>
       <c r="S66" s="15" t="n"/>
       <c r="T66" s="5" t="n"/>
-      <c r="V66">
+      <c r="V66" t="str">
         <f>IF(L66="","",L66+ROW()/100000)</f>
         <v/>
       </c>
@@ -6094,9 +6094,9 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16">
+      <c r="A2" s="16" t="str">
         <f>"Use case: "&amp;IF('1. Use Case Profile'!$C$5="","(not specified)",'1. Use Case Profile'!$C$5)&amp;"   |   Inherent tier: "&amp;'3. Risk Tiering'!$C$21&amp;"   |   Tiering score: "&amp;'3. Risk Tiering'!$C$17</f>
-        <v/>
+        <v>Use case: (not specified)   |   Inherent tier: Incomplete   |   Tiering score: </v>
       </c>
     </row>
     <row r="4">
@@ -6161,23 +6161,23 @@
       </c>
       <c r="B6" s="18">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Almost certain",'4. Risk Register'!$G$5:$G$66,"Insignificant")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C6" s="19">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Almost certain",'4. Risk Register'!$G$5:$G$66,"Minor")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D6" s="19">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Almost certain",'4. Risk Register'!$G$5:$G$66,"Moderate")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E6" s="20">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Almost certain",'4. Risk Register'!$G$5:$G$66,"Major")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F6" s="20">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Almost certain",'4. Risk Register'!$G$5:$G$66,"Severe")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H6" s="21" t="inlineStr">
         <is>
@@ -6186,11 +6186,11 @@
       </c>
       <c r="I6" s="7">
         <f>COUNTIF('4. Risk Register'!$I$5:$I$66,"Critical")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J6" s="7">
         <f>COUNTIF('4. Risk Register'!$M$5:$M$66,"Critical")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
@@ -6201,23 +6201,23 @@
       </c>
       <c r="B7" s="22">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Likely",'4. Risk Register'!$G$5:$G$66,"Insignificant")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C7" s="18">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Likely",'4. Risk Register'!$G$5:$G$66,"Minor")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D7" s="19">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Likely",'4. Risk Register'!$G$5:$G$66,"Moderate")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E7" s="19">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Likely",'4. Risk Register'!$G$5:$G$66,"Major")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F7" s="20">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Likely",'4. Risk Register'!$G$5:$G$66,"Severe")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H7" s="23" t="inlineStr">
         <is>
@@ -6226,11 +6226,11 @@
       </c>
       <c r="I7" s="7">
         <f>COUNTIF('4. Risk Register'!$I$5:$I$66,"High")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J7" s="7">
         <f>COUNTIF('4. Risk Register'!$M$5:$M$66,"High")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
@@ -6241,23 +6241,23 @@
       </c>
       <c r="B8" s="22">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Possible",'4. Risk Register'!$G$5:$G$66,"Insignificant")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C8" s="18">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Possible",'4. Risk Register'!$G$5:$G$66,"Minor")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D8" s="18">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Possible",'4. Risk Register'!$G$5:$G$66,"Moderate")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E8" s="19">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Possible",'4. Risk Register'!$G$5:$G$66,"Major")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F8" s="19">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Possible",'4. Risk Register'!$G$5:$G$66,"Severe")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H8" s="24" t="inlineStr">
         <is>
@@ -6266,11 +6266,11 @@
       </c>
       <c r="I8" s="7">
         <f>COUNTIF('4. Risk Register'!$I$5:$I$66,"Medium")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J8" s="7">
         <f>COUNTIF('4. Risk Register'!$M$5:$M$66,"Medium")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
@@ -6281,23 +6281,23 @@
       </c>
       <c r="B9" s="22">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Unlikely",'4. Risk Register'!$G$5:$G$66,"Insignificant")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C9" s="22">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Unlikely",'4. Risk Register'!$G$5:$G$66,"Minor")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D9" s="18">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Unlikely",'4. Risk Register'!$G$5:$G$66,"Moderate")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E9" s="18">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Unlikely",'4. Risk Register'!$G$5:$G$66,"Major")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F9" s="19">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Unlikely",'4. Risk Register'!$G$5:$G$66,"Severe")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H9" s="25" t="inlineStr">
         <is>
@@ -6306,11 +6306,11 @@
       </c>
       <c r="I9" s="7">
         <f>COUNTIF('4. Risk Register'!$I$5:$I$66,"Low")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J9" s="7">
         <f>COUNTIF('4. Risk Register'!$M$5:$M$66,"Low")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
@@ -6321,23 +6321,23 @@
       </c>
       <c r="B10" s="22">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Rare",'4. Risk Register'!$G$5:$G$66,"Insignificant")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C10" s="22">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Rare",'4. Risk Register'!$G$5:$G$66,"Minor")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D10" s="22">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Rare",'4. Risk Register'!$G$5:$G$66,"Moderate")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E10" s="22">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Rare",'4. Risk Register'!$G$5:$G$66,"Major")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F10" s="18">
         <f>COUNTIFS('4. Risk Register'!$A$5:$A$66,"Yes",'4. Risk Register'!$F$5:$F$66,"Rare",'4. Risk Register'!$G$5:$G$66,"Severe")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
@@ -6346,11 +6346,11 @@
       </c>
       <c r="I10" s="9">
         <f>SUM(I6:I9)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J10" s="9">
         <f>SUM(J6:J9)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -6367,7 +6367,7 @@
       <c r="I11" s="10" t="n"/>
       <c r="J11" s="9">
         <f>J6+J7</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -6424,27 +6424,27 @@
       </c>
       <c r="D16" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Governance &amp; Accountability",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E16" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Governance &amp; Accountability",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F16" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Governance &amp; Accountability",'4. Risk Register'!$M$5:$M$66,"High")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G16" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Governance &amp; Accountability",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H16" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Governance &amp; Accountability",'4. Risk Register'!$M$5:$M$66,"Low")</f>
-        <v/>
-      </c>
-      <c r="I16" s="7">
+        <v>0</v>
+      </c>
+      <c r="I16" s="7" t="str">
         <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Governance &amp; Accountability",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
-        <v/>
+        <v>-</v>
       </c>
     </row>
     <row r="17">
@@ -6455,27 +6455,27 @@
       </c>
       <c r="D17" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Legal, Regulatory &amp; Compliance",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E17" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Legal, Regulatory &amp; Compliance",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F17" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Legal, Regulatory &amp; Compliance",'4. Risk Register'!$M$5:$M$66,"High")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G17" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Legal, Regulatory &amp; Compliance",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H17" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Legal, Regulatory &amp; Compliance",'4. Risk Register'!$M$5:$M$66,"Low")</f>
-        <v/>
-      </c>
-      <c r="I17" s="7">
+        <v>0</v>
+      </c>
+      <c r="I17" s="7" t="str">
         <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Legal, Regulatory &amp; Compliance",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
-        <v/>
+        <v>-</v>
       </c>
     </row>
     <row r="18">
@@ -6486,27 +6486,27 @@
       </c>
       <c r="D18" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Fairness, Bias &amp; Human Rights",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E18" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Fairness, Bias &amp; Human Rights",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F18" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Fairness, Bias &amp; Human Rights",'4. Risk Register'!$M$5:$M$66,"High")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G18" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Fairness, Bias &amp; Human Rights",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H18" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Fairness, Bias &amp; Human Rights",'4. Risk Register'!$M$5:$M$66,"Low")</f>
-        <v/>
-      </c>
-      <c r="I18" s="7">
+        <v>0</v>
+      </c>
+      <c r="I18" s="7" t="str">
         <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Fairness, Bias &amp; Human Rights",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
-        <v/>
+        <v>-</v>
       </c>
     </row>
     <row r="19">
@@ -6517,27 +6517,27 @@
       </c>
       <c r="D19" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Privacy &amp; Data Protection",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E19" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Privacy &amp; Data Protection",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F19" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Privacy &amp; Data Protection",'4. Risk Register'!$M$5:$M$66,"High")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G19" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Privacy &amp; Data Protection",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H19" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Privacy &amp; Data Protection",'4. Risk Register'!$M$5:$M$66,"Low")</f>
-        <v/>
-      </c>
-      <c r="I19" s="7">
+        <v>0</v>
+      </c>
+      <c r="I19" s="7" t="str">
         <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Privacy &amp; Data Protection",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
-        <v/>
+        <v>-</v>
       </c>
     </row>
     <row r="20">
@@ -6548,27 +6548,27 @@
       </c>
       <c r="D20" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Data Quality &amp; Integrity",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E20" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Data Quality &amp; Integrity",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F20" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Data Quality &amp; Integrity",'4. Risk Register'!$M$5:$M$66,"High")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G20" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Data Quality &amp; Integrity",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H20" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Data Quality &amp; Integrity",'4. Risk Register'!$M$5:$M$66,"Low")</f>
-        <v/>
-      </c>
-      <c r="I20" s="7">
+        <v>0</v>
+      </c>
+      <c r="I20" s="7" t="str">
         <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Data Quality &amp; Integrity",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
-        <v/>
+        <v>-</v>
       </c>
     </row>
     <row r="21">
@@ -6579,27 +6579,27 @@
       </c>
       <c r="D21" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Model Performance, Reliability &amp; Robustness",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E21" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Model Performance, Reliability &amp; Robustness",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F21" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Model Performance, Reliability &amp; Robustness",'4. Risk Register'!$M$5:$M$66,"High")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G21" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Model Performance, Reliability &amp; Robustness",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H21" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Model Performance, Reliability &amp; Robustness",'4. Risk Register'!$M$5:$M$66,"Low")</f>
-        <v/>
-      </c>
-      <c r="I21" s="7">
+        <v>0</v>
+      </c>
+      <c r="I21" s="7" t="str">
         <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Model Performance, Reliability &amp; Robustness",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
-        <v/>
+        <v>-</v>
       </c>
     </row>
     <row r="22">
@@ -6610,27 +6610,27 @@
       </c>
       <c r="D22" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Transparency, Explainability &amp; Contestability",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E22" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Transparency, Explainability &amp; Contestability",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F22" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Transparency, Explainability &amp; Contestability",'4. Risk Register'!$M$5:$M$66,"High")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G22" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Transparency, Explainability &amp; Contestability",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H22" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Transparency, Explainability &amp; Contestability",'4. Risk Register'!$M$5:$M$66,"Low")</f>
-        <v/>
-      </c>
-      <c r="I22" s="7">
+        <v>0</v>
+      </c>
+      <c r="I22" s="7" t="str">
         <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Transparency, Explainability &amp; Contestability",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
-        <v/>
+        <v>-</v>
       </c>
     </row>
     <row r="23">
@@ -6641,27 +6641,27 @@
       </c>
       <c r="D23" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Security of AI Systems",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E23" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Security of AI Systems",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F23" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Security of AI Systems",'4. Risk Register'!$M$5:$M$66,"High")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G23" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Security of AI Systems",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H23" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Security of AI Systems",'4. Risk Register'!$M$5:$M$66,"Low")</f>
-        <v/>
-      </c>
-      <c r="I23" s="7">
+        <v>0</v>
+      </c>
+      <c r="I23" s="7" t="str">
         <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Security of AI Systems",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
-        <v/>
+        <v>-</v>
       </c>
     </row>
     <row r="24">
@@ -6672,27 +6672,27 @@
       </c>
       <c r="D24" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Human Oversight &amp; Autonomy",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E24" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Human Oversight &amp; Autonomy",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F24" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Human Oversight &amp; Autonomy",'4. Risk Register'!$M$5:$M$66,"High")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G24" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Human Oversight &amp; Autonomy",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H24" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Human Oversight &amp; Autonomy",'4. Risk Register'!$M$5:$M$66,"Low")</f>
-        <v/>
-      </c>
-      <c r="I24" s="7">
+        <v>0</v>
+      </c>
+      <c r="I24" s="7" t="str">
         <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Human Oversight &amp; Autonomy",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
-        <v/>
+        <v>-</v>
       </c>
     </row>
     <row r="25">
@@ -6703,27 +6703,27 @@
       </c>
       <c r="D25" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Third-Party &amp; Supply Chain",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E25" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Third-Party &amp; Supply Chain",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F25" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Third-Party &amp; Supply Chain",'4. Risk Register'!$M$5:$M$66,"High")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G25" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Third-Party &amp; Supply Chain",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H25" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Third-Party &amp; Supply Chain",'4. Risk Register'!$M$5:$M$66,"Low")</f>
-        <v/>
-      </c>
-      <c r="I25" s="7">
+        <v>0</v>
+      </c>
+      <c r="I25" s="7" t="str">
         <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Third-Party &amp; Supply Chain",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
-        <v/>
+        <v>-</v>
       </c>
     </row>
     <row r="26">
@@ -6734,27 +6734,27 @@
       </c>
       <c r="D26" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Operational, Financial &amp; Sustainability",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E26" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Operational, Financial &amp; Sustainability",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F26" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Operational, Financial &amp; Sustainability",'4. Risk Register'!$M$5:$M$66,"High")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G26" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Operational, Financial &amp; Sustainability",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H26" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Operational, Financial &amp; Sustainability",'4. Risk Register'!$M$5:$M$66,"Low")</f>
-        <v/>
-      </c>
-      <c r="I26" s="7">
+        <v>0</v>
+      </c>
+      <c r="I26" s="7" t="str">
         <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Operational, Financial &amp; Sustainability",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
-        <v/>
+        <v>-</v>
       </c>
     </row>
     <row r="27">
@@ -6765,27 +6765,27 @@
       </c>
       <c r="D27" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Societal, Reputational &amp; AI-Enabled Threats",'4. Risk Register'!$A$5:$A$66,"Yes")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E27" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Societal, Reputational &amp; AI-Enabled Threats",'4. Risk Register'!$M$5:$M$66,"Critical")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F27" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Societal, Reputational &amp; AI-Enabled Threats",'4. Risk Register'!$M$5:$M$66,"High")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G27" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Societal, Reputational &amp; AI-Enabled Threats",'4. Risk Register'!$M$5:$M$66,"Medium")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H27" s="7">
         <f>COUNTIFS('4. Risk Register'!$C$5:$C$66,"Societal, Reputational &amp; AI-Enabled Threats",'4. Risk Register'!$M$5:$M$66,"Low")</f>
-        <v/>
-      </c>
-      <c r="I27" s="7">
+        <v>0</v>
+      </c>
+      <c r="I27" s="7" t="str">
         <f>IFERROR(ROUND(AVERAGEIFS('4. Risk Register'!$L$5:$L$66,'4. Risk Register'!$C$5:$C$66,"Societal, Reputational &amp; AI-Enabled Threats",'4. Risk Register'!$A$5:$A$66,"Yes"),1),"-")</f>
-        <v/>
+        <v>-</v>
       </c>
     </row>
     <row r="30">
@@ -6844,34 +6844,34 @@
       <c r="A32" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B32" s="7">
+      <c r="B32" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,1),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="C32" s="12">
+      <c r="C32" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,1),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D32" s="12" t="n"/>
       <c r="E32" s="12" t="n"/>
       <c r="F32" s="12" t="n"/>
-      <c r="G32" s="7">
+      <c r="G32" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,1),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="H32" s="7">
+      <c r="H32" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,1),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="I32" s="7">
+      <c r="I32" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,1),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="J32" s="12">
+      <c r="J32" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,1),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="K32" s="7">
+      <c r="K32" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,1),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
@@ -6880,34 +6880,34 @@
       <c r="A33" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B33" s="7">
+      <c r="B33" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,2),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="C33" s="12">
+      <c r="C33" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,2),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D33" s="12" t="n"/>
       <c r="E33" s="12" t="n"/>
       <c r="F33" s="12" t="n"/>
-      <c r="G33" s="7">
+      <c r="G33" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,2),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="H33" s="7">
+      <c r="H33" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,2),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="I33" s="7">
+      <c r="I33" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,2),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="J33" s="12">
+      <c r="J33" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,2),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="K33" s="7">
+      <c r="K33" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,2),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
@@ -6916,34 +6916,34 @@
       <c r="A34" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B34" s="7">
+      <c r="B34" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,3),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="C34" s="12">
+      <c r="C34" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,3),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D34" s="12" t="n"/>
       <c r="E34" s="12" t="n"/>
       <c r="F34" s="12" t="n"/>
-      <c r="G34" s="7">
+      <c r="G34" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,3),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="H34" s="7">
+      <c r="H34" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,3),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="I34" s="7">
+      <c r="I34" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,3),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="J34" s="12">
+      <c r="J34" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,3),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="K34" s="7">
+      <c r="K34" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,3),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
@@ -6952,34 +6952,34 @@
       <c r="A35" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B35" s="7">
+      <c r="B35" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,4),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="C35" s="12">
+      <c r="C35" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,4),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D35" s="12" t="n"/>
       <c r="E35" s="12" t="n"/>
       <c r="F35" s="12" t="n"/>
-      <c r="G35" s="7">
+      <c r="G35" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,4),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="H35" s="7">
+      <c r="H35" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,4),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="I35" s="7">
+      <c r="I35" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,4),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="J35" s="12">
+      <c r="J35" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,4),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="K35" s="7">
+      <c r="K35" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,4),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
@@ -6988,34 +6988,34 @@
       <c r="A36" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B36" s="7">
+      <c r="B36" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,5),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="C36" s="12">
+      <c r="C36" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,5),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D36" s="12" t="n"/>
       <c r="E36" s="12" t="n"/>
       <c r="F36" s="12" t="n"/>
-      <c r="G36" s="7">
+      <c r="G36" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,5),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="H36" s="7">
+      <c r="H36" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,5),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="I36" s="7">
+      <c r="I36" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,5),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="J36" s="12">
+      <c r="J36" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,5),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="K36" s="7">
+      <c r="K36" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,5),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
@@ -7024,34 +7024,34 @@
       <c r="A37" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B37" s="7">
+      <c r="B37" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,6),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="C37" s="12">
+      <c r="C37" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,6),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D37" s="12" t="n"/>
       <c r="E37" s="12" t="n"/>
       <c r="F37" s="12" t="n"/>
-      <c r="G37" s="7">
+      <c r="G37" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,6),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="H37" s="7">
+      <c r="H37" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,6),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="I37" s="7">
+      <c r="I37" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,6),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="J37" s="12">
+      <c r="J37" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,6),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="K37" s="7">
+      <c r="K37" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,6),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
@@ -7060,34 +7060,34 @@
       <c r="A38" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B38" s="7">
+      <c r="B38" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,7),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="C38" s="12">
+      <c r="C38" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,7),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D38" s="12" t="n"/>
       <c r="E38" s="12" t="n"/>
       <c r="F38" s="12" t="n"/>
-      <c r="G38" s="7">
+      <c r="G38" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,7),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="H38" s="7">
+      <c r="H38" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,7),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="I38" s="7">
+      <c r="I38" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,7),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="J38" s="12">
+      <c r="J38" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,7),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="K38" s="7">
+      <c r="K38" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,7),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
@@ -7096,34 +7096,34 @@
       <c r="A39" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B39" s="7">
+      <c r="B39" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,8),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="C39" s="12">
+      <c r="C39" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,8),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D39" s="12" t="n"/>
       <c r="E39" s="12" t="n"/>
       <c r="F39" s="12" t="n"/>
-      <c r="G39" s="7">
+      <c r="G39" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,8),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="H39" s="7">
+      <c r="H39" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,8),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="I39" s="7">
+      <c r="I39" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,8),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="J39" s="12">
+      <c r="J39" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,8),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="K39" s="7">
+      <c r="K39" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,8),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
@@ -7132,34 +7132,34 @@
       <c r="A40" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B40" s="7">
+      <c r="B40" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,9),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="C40" s="12">
+      <c r="C40" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,9),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D40" s="12" t="n"/>
       <c r="E40" s="12" t="n"/>
       <c r="F40" s="12" t="n"/>
-      <c r="G40" s="7">
+      <c r="G40" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,9),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="H40" s="7">
+      <c r="H40" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,9),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="I40" s="7">
+      <c r="I40" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,9),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="J40" s="12">
+      <c r="J40" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,9),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="K40" s="7">
+      <c r="K40" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,9),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
@@ -7168,34 +7168,34 @@
       <c r="A41" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B41" s="7">
+      <c r="B41" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$B$5:$B$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,10),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="C41" s="12">
+      <c r="C41" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$D$5:$D$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,10),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
       <c r="D41" s="12" t="n"/>
       <c r="E41" s="12" t="n"/>
       <c r="F41" s="12" t="n"/>
-      <c r="G41" s="7">
+      <c r="G41" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$L$5:$L$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,10),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="H41" s="7">
+      <c r="H41" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$M$5:$M$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,10),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="I41" s="7">
+      <c r="I41" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$O$5:$O$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,10),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="J41" s="12">
+      <c r="J41" s="12" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$Q$5:$Q$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,10),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
-      <c r="K41" s="7">
+      <c r="K41" s="7" t="str">
         <f>IFERROR(INDEX('4. Risk Register'!$S$5:$S$66,MATCH(LARGE('4. Risk Register'!$V$5:$V$66,10),'4. Risk Register'!$V$5:$V$66,0)),"")</f>
         <v/>
       </c>
@@ -7213,7 +7213,7 @@
           <t>Required approval authority:</t>
         </is>
       </c>
-      <c r="D44">
+      <c r="D44" t="str">
         <f>'3. Risk Tiering'!C23</f>
         <v/>
       </c>

</xml_diff>